<commit_message>
chore(web): complete Sprint 0 foundation
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R246fac9b78de4818"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R32e8fad96ebc4b84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R6f65648b768b4706"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R5e27f06704cc4f6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R0ef9b7cc7d944865"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Raa397d2820064bc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R553db6d2f7f84447"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R61645b69700f48f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R0d7d4c55642b4ddd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="Rd7df099411ab4894"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R8a8ccd5513ed4f97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R40d7406f196e4301"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,6 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+  </x:numFmts>
   <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
@@ -110,7 +113,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="68">
+  <x:cellXfs count="69">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -256,6 +259,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -424,9 +430,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="48672768"/>
-        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="48672768"/>
@@ -491,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0d8f403d18524e55"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R19b1f16a7e51479b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -800,7 +804,7 @@
       </x:c>
       <x:c r="B6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_PROGRESO")</x:f>
@@ -816,7 +820,7 @@
       </x:c>
       <x:c r="F6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>0</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -849,7 +853,7 @@
       </x:c>
       <x:c r="C10" s="12" t="n">
         <x:f>COUNTIFS('01_Backlog'!E2:E142,A10,'01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E10" t="str">
         <x:v>WEB</x:v>
@@ -860,7 +864,7 @@
       </x:c>
       <x:c r="G10" t="n">
         <x:f>COUNTIFS('01_Backlog'!C2:C142,E10,'01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>0</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
@@ -1043,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a04b1be9a594908"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46b3765cdd114514"/>
 </x:worksheet>
 </file>
 
@@ -1188,7 +1192,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J2" s="14" t="str">
-        <x:v>READY</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K2" s="14" t="str"/>
       <x:c r="L2" s="14" t="str">
@@ -1222,9 +1226,13 @@
       <x:c r="V2" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W2" s="14" t="str"/>
+      <x:c r="W2" s="14" t="str">
+        <x:v>Next/npm, lockfile y build PASS; sin features.</x:v>
+      </x:c>
       <x:c r="X2" s="14" t="str"/>
-      <x:c r="Y2" s="14" t="str"/>
+      <x:c r="Y2" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z2" s="14" t="str"/>
     </x:row>
     <x:row r="3" ht="84" customHeight="1">
@@ -1256,7 +1264,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J3" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K3" s="14" t="str">
         <x:v>IMP-WEB-0001</x:v>
@@ -1292,9 +1300,13 @@
       <x:c r="V3" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W3" s="14" t="str"/>
+      <x:c r="W3" s="14" t="str">
+        <x:v>Strict, alias @/* y carpetas base; typecheck PASS.</x:v>
+      </x:c>
       <x:c r="X3" s="14" t="str"/>
-      <x:c r="Y3" s="14" t="str"/>
+      <x:c r="Y3" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z3" s="14" t="str"/>
     </x:row>
     <x:row r="4" ht="84" customHeight="1">
@@ -1326,7 +1338,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J4" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K4" s="14" t="str">
         <x:v>IMP-WEB-0002</x:v>
@@ -1362,9 +1374,13 @@
       <x:c r="V4" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W4" s="14" t="str"/>
+      <x:c r="W4" s="14" t="str">
+        <x:v>Route Groups; / y /dashboard smoke PASS.</x:v>
+      </x:c>
       <x:c r="X4" s="14" t="str"/>
-      <x:c r="Y4" s="14" t="str"/>
+      <x:c r="Y4" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z4" s="14" t="str"/>
     </x:row>
     <x:row r="5" ht="84" customHeight="1">
@@ -1396,7 +1412,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J5" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K5" s="14" t="str">
         <x:v>IMP-WEB-0001</x:v>
@@ -1432,9 +1448,13 @@
       <x:c r="V5" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W5" s="14" t="str"/>
+      <x:c r="W5" s="14" t="str">
+        <x:v>tokens.css 1:1 contra documento 31; build PASS.</x:v>
+      </x:c>
       <x:c r="X5" s="14" t="str"/>
-      <x:c r="Y5" s="14" t="str"/>
+      <x:c r="Y5" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z5" s="14" t="str"/>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -1466,7 +1486,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J6" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K6" s="14" t="str">
         <x:v>IMP-WEB-0003, IMP-WEB-0004</x:v>
@@ -1502,9 +1522,13 @@
       <x:c r="V6" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W6" s="14" t="str"/>
+      <x:c r="W6" s="14" t="str">
+        <x:v>globals + Inter/Lora; smoke visual PASS.</x:v>
+      </x:c>
       <x:c r="X6" s="14" t="str"/>
-      <x:c r="Y6" s="14" t="str"/>
+      <x:c r="Y6" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z6" s="14" t="str"/>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -1536,7 +1560,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J7" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K7" s="14" t="str">
         <x:v>IMP-WEB-0002</x:v>
@@ -1572,9 +1596,13 @@
       <x:c r="V7" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W7" s="14" t="str"/>
+      <x:c r="W7" s="14" t="str">
+        <x:v>fetch/env/errores tipados; pruebas del cliente PASS.</x:v>
+      </x:c>
       <x:c r="X7" s="14" t="str"/>
-      <x:c r="Y7" s="14" t="str"/>
+      <x:c r="Y7" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z7" s="14" t="str"/>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -1606,7 +1634,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J8" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K8" s="14" t="str">
         <x:v>IMP-WEB-0002</x:v>
@@ -1642,9 +1670,13 @@
       <x:c r="V8" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W8" s="14" t="str"/>
+      <x:c r="W8" s="14" t="str">
+        <x:v>DomainMappingError seguro; prueba PASS.</x:v>
+      </x:c>
       <x:c r="X8" s="14" t="str"/>
-      <x:c r="Y8" s="14" t="str"/>
+      <x:c r="Y8" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z8" s="14" t="str"/>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -1676,7 +1708,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J9" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K9" s="14" t="str">
         <x:v>IMP-WEB-0002</x:v>
@@ -1712,9 +1744,13 @@
       <x:c r="V9" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W9" s="14" t="str"/>
+      <x:c r="W9" s="14" t="str">
+        <x:v>QueryClientProvider técnico; RTL/build PASS.</x:v>
+      </x:c>
       <x:c r="X9" s="14" t="str"/>
-      <x:c r="Y9" s="14" t="str"/>
+      <x:c r="Y9" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z9" s="14" t="str"/>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -1746,7 +1782,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J10" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K10" s="14" t="str">
         <x:v>IMP-WEB-0006</x:v>
@@ -1782,9 +1818,13 @@
       <x:c r="V10" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W10" s="14" t="str"/>
+      <x:c r="W10" s="14" t="str">
+        <x:v>MSW técnico con flag; Vitest PASS.</x:v>
+      </x:c>
       <x:c r="X10" s="14" t="str"/>
-      <x:c r="Y10" s="14" t="str"/>
+      <x:c r="Y10" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z10" s="14" t="str"/>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -1816,7 +1856,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J11" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K11" s="14" t="str">
         <x:v>IMP-WEB-0001</x:v>
@@ -1852,9 +1892,13 @@
       <x:c r="V11" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W11" s="14" t="str"/>
+      <x:c r="W11" s="14" t="str">
+        <x:v>Vitest + RTL/jsdom; 4 pruebas PASS; sin Playwright.</x:v>
+      </x:c>
       <x:c r="X11" s="14" t="str"/>
-      <x:c r="Y11" s="14" t="str"/>
+      <x:c r="Y11" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z11" s="14" t="str"/>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -1886,7 +1930,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J12" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K12" s="14" t="str">
         <x:v>IMP-WEB-0002</x:v>
@@ -1922,9 +1966,13 @@
       <x:c r="V12" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W12" s="14" t="str"/>
+      <x:c r="W12" s="14" t="str">
+        <x:v>Flat config/boundaries; violación temporal detectada; lint PASS.</x:v>
+      </x:c>
       <x:c r="X12" s="14" t="str"/>
-      <x:c r="Y12" s="14" t="str"/>
+      <x:c r="Y12" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z12" s="14" t="str"/>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -1956,7 +2004,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J13" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K13" s="14" t="str">
         <x:v>IMP-WEB-0003, IMP-WEB-0005</x:v>
@@ -1994,9 +2042,13 @@
       <x:c r="V13" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W13" s="14" t="str"/>
+      <x:c r="W13" s="14" t="str">
+        <x:v>PublicLayout técnico; / responde 200.</x:v>
+      </x:c>
       <x:c r="X13" s="14" t="str"/>
-      <x:c r="Y13" s="14" t="str"/>
+      <x:c r="Y13" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z13" s="14" t="str"/>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -2028,7 +2080,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J14" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K14" s="14" t="str">
         <x:v>IMP-WEB-0003, IMP-WEB-0005</x:v>
@@ -2064,9 +2116,13 @@
       <x:c r="V14" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W14" s="14" t="str"/>
+      <x:c r="W14" s="14" t="str">
+        <x:v>PrivateLayout técnico; /dashboard responde 200.</x:v>
+      </x:c>
       <x:c r="X14" s="14" t="str"/>
-      <x:c r="Y14" s="14" t="str"/>
+      <x:c r="Y14" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z14" s="14" t="str"/>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -2098,7 +2154,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J15" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K15" s="14" t="str">
         <x:v>IMP-WEB-0010, IMP-WEB-0011</x:v>
@@ -2134,9 +2190,13 @@
       <x:c r="V15" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W15" s="14" t="str"/>
+      <x:c r="W15" s="14" t="str">
+        <x:v>web-ci.yml raíz; secuencia local equivalente PASS.</x:v>
+      </x:c>
       <x:c r="X15" s="14" t="str"/>
-      <x:c r="Y15" s="14" t="str"/>
+      <x:c r="Y15" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z15" s="14" t="str"/>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -2168,7 +2228,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J16" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K16" s="14" t="str">
         <x:v>IMP-WEB-0010, IMP-WEB-0011</x:v>
@@ -2204,9 +2264,13 @@
       <x:c r="V16" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W16" s="14" t="str"/>
+      <x:c r="W16" s="14" t="str">
+        <x:v>Scripts estándar y check PASS; sin e2e.</x:v>
+      </x:c>
       <x:c r="X16" s="14" t="str"/>
-      <x:c r="Y16" s="14" t="str"/>
+      <x:c r="Y16" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z16" s="14" t="str"/>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -2238,7 +2302,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J17" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K17" s="14" t="str">
         <x:v>IMP-WEB-0001, IMP-WEB-0002, IMP-WEB-0003, IMP-WEB-0004, IMP-WEB-0005, IMP-WEB-0006, IMP-WEB-0007, IMP-WEB-0008, IMP-WEB-0009, IMP-WEB-0010, IMP-WEB-0011, IMP-WEB-0012, IMP-WEB-0013, IMP-WEB-0014, IMP-WEB-0015</x:v>
@@ -2274,9 +2338,13 @@
       <x:c r="V17" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W17" s="14" t="str"/>
+      <x:c r="W17" s="14" t="str">
+        <x:v>README, ADR y docs Web sincronizados.</x:v>
+      </x:c>
       <x:c r="X17" s="14" t="str"/>
-      <x:c r="Y17" s="14" t="str"/>
+      <x:c r="Y17" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z17" s="14" t="str"/>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -2308,7 +2376,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J18" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K18" s="14" t="str">
         <x:v>IMP-WEB-0001, IMP-WEB-0002, IMP-WEB-0003, IMP-WEB-0004, IMP-WEB-0005, IMP-WEB-0006, IMP-WEB-0007, IMP-WEB-0008, IMP-WEB-0009, IMP-WEB-0010, IMP-WEB-0011, IMP-WEB-0012, IMP-WEB-0013, IMP-WEB-0014, IMP-WEB-0015, IMP-WEB-0016</x:v>
@@ -2344,9 +2412,13 @@
       <x:c r="V18" s="14" t="str">
         <x:v>chore/web-sprint-0</x:v>
       </x:c>
-      <x:c r="W18" s="14" t="str"/>
+      <x:c r="W18" s="14" t="str">
+        <x:v>check PASS; build, rutas, tokens, Query, MSW y boundaries validados.</x:v>
+      </x:c>
       <x:c r="X18" s="14" t="str"/>
-      <x:c r="Y18" s="14" t="str"/>
+      <x:c r="Y18" s="68" t="n">
+        <x:v>46274</x:v>
+      </x:c>
       <x:c r="Z18" s="14" t="str"/>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -11134,7 +11206,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4618bc73524441b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a943fe68caf4c75"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(android): approve sprint zero stack
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R553db6d2f7f84447"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R61645b69700f48f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R0d7d4c55642b4ddd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="Rd7df099411ab4894"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R8a8ccd5513ed4f97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R40d7406f196e4301"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="Rfe73230685e54f89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="Rcc1cdaad58d74a17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Ra24a09736d37480d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R1d33809fee1d4c8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R91522239842b4246"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R2bdc77512db045d6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R19b1f16a7e51479b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6c850d49a9884d20"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -804,7 +804,7 @@
       </x:c>
       <x:c r="B6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_PROGRESO")</x:f>
@@ -820,7 +820,7 @@
       </x:c>
       <x:c r="F6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -888,7 +888,7 @@
       </x:c>
       <x:c r="G11" t="n">
         <x:f>COUNTIFS('01_Backlog'!C2:C142,E11,'01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -927,7 +927,7 @@
       </x:c>
       <x:c r="C14" s="12" t="n">
         <x:f>COUNTIFS('01_Backlog'!E2:E142,A14,'01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46b3765cdd114514"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7c3a07910814aef"/>
 </x:worksheet>
 </file>
 
@@ -9250,7 +9250,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J116" s="14" t="str">
-        <x:v>READY</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K116" s="14" t="str"/>
       <x:c r="L116" s="14" t="str">
@@ -9286,10 +9286,16 @@
       <x:c r="V116" s="14" t="str">
         <x:v>chore/android-sprint-0</x:v>
       </x:c>
-      <x:c r="W116" s="14" t="str"/>
+      <x:c r="W116" s="14" t="str">
+        <x:v>DEC-A-001/002 y docs Android actualizados; review documental PASS.</x:v>
+      </x:c>
       <x:c r="X116" s="14" t="str"/>
-      <x:c r="Y116" s="14" t="str"/>
-      <x:c r="Z116" s="14" t="str"/>
+      <x:c r="Y116" s="14" t="str">
+        <x:v>2026-09-09</x:v>
+      </x:c>
+      <x:c r="Z116" s="14" t="str">
+        <x:v>Stack oficial aprobado por el equipo; Figma canónico 238:132 registrado.</x:v>
+      </x:c>
     </x:row>
     <x:row r="117" ht="84" customHeight="1">
       <x:c r="A117" s="14" t="str">
@@ -11206,7 +11212,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a943fe68caf4c75"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e75d91040da4275"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
chore(android): complete Sprint 0 foundation
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="Rfe73230685e54f89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="Rcc1cdaad58d74a17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Ra24a09736d37480d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R1d33809fee1d4c8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R91522239842b4246"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R2bdc77512db045d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="Rcf6db0241c664943"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="Rfdf00f631d2c405d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Raff21bc3ef814ec2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R64fd4fd14d7b4394"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Ra56c032c8b0b4658"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Re9429219fbcf454b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6c850d49a9884d20"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdcd18f1515184f6c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -820,7 +820,7 @@
       </x:c>
       <x:c r="F6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>18</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -888,7 +888,7 @@
       </x:c>
       <x:c r="G11" t="n">
         <x:f>COUNTIFS('01_Backlog'!C2:C142,E11,'01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>1</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7c3a07910814aef"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd88c3d51a4544fd8"/>
 </x:worksheet>
 </file>
 
@@ -9326,13 +9326,13 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J117" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K117" s="14" t="str">
         <x:v>IMP-AND-0001</x:v>
       </x:c>
       <x:c r="L117" s="14" t="str">
-        <x:v>Android architecture docs</x:v>
+        <x:v>DEC-A-003 / Android architecture docs</x:v>
       </x:c>
       <x:c r="M117" s="14" t="str">
         <x:v>238:132</x:v>
@@ -9344,30 +9344,36 @@
         <x:v>Inicializar proyecto Android</x:v>
       </x:c>
       <x:c r="P117" s="14" t="str">
-        <x:v>Crear dentro frontend/pms-hotel-android; no git init; conservar docs; build mínimo.</x:v>
+        <x:v>Crear proyecto Expo CNG dentro de frontend/pms-hotel-android; no git init; conservar docs; ignorar android/ e ios/; app técnica mínima.</x:v>
       </x:c>
       <x:c r="Q117" s="14" t="str">
-        <x:v>Proyecto compila; un solo .git; no feature screens.</x:v>
+        <x:v>Proyecto Expo CNG compila/exporta; un solo .git; android/ e ios/ no versionados; 0 pantallas funcionales.</x:v>
       </x:c>
       <x:c r="R117" s="14" t="str">
-        <x:v>0001 COMPLETADA.</x:v>
+        <x:v>IMP-AND-0001 COMPLETADA; Node/npm compatibles con la versión Expo elegida.</x:v>
       </x:c>
       <x:c r="S117" s="14" t="str">
-        <x:v>Build PASS.</x:v>
+        <x:v>npm ci + expo-doctor + tsc --noEmit + expo export + smoke navegación/app técnica PASS.</x:v>
       </x:c>
       <x:c r="T117" s="14" t="str">
-        <x:v>Gradle build/assemble</x:v>
+        <x:v>npm ci; npx expo-doctor; npx tsc --noEmit; npx expo export; smoke navegación/app técnica</x:v>
       </x:c>
       <x:c r="U117" s="14" t="str">
-        <x:v>project files</x:v>
+        <x:v>Expo project files + .gitignore para android/ e ios/</x:v>
       </x:c>
       <x:c r="V117" s="14" t="str">
         <x:v>chore/android-sprint-0</x:v>
       </x:c>
-      <x:c r="W117" s="14" t="str"/>
+      <x:c r="W117" s="14" t="str">
+        <x:v>CNG + package-lock; npm ci, doctor, typecheck, export y smoke PASS.</x:v>
+      </x:c>
       <x:c r="X117" s="14" t="str"/>
-      <x:c r="Y117" s="14" t="str"/>
-      <x:c r="Z117" s="14" t="str"/>
+      <x:c r="Y117" s="14" t="str">
+        <x:v>2026-09-09</x:v>
+      </x:c>
+      <x:c r="Z117" s="14" t="str">
+        <x:v>CNG aprobado. Gradle build/assemble sustituido por validación Expo Foundation.</x:v>
+      </x:c>
     </x:row>
     <x:row r="118" ht="84" customHeight="1">
       <x:c r="A118" s="14" t="str">
@@ -9398,7 +9404,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J118" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K118" s="14" t="str">
         <x:v>IMP-AND-0002</x:v>
@@ -9436,9 +9442,13 @@
       <x:c r="V118" s="14" t="str">
         <x:v>chore/android-sprint-0</x:v>
       </x:c>
-      <x:c r="W118" s="14" t="str"/>
+      <x:c r="W118" s="14" t="str">
+        <x:v>Tokens Figma 238:132, docs/15 y StyleSheet; smoke técnico/export PASS.</x:v>
+      </x:c>
       <x:c r="X118" s="14" t="str"/>
-      <x:c r="Y118" s="14" t="str"/>
+      <x:c r="Y118" s="14" t="str">
+        <x:v>2026-09-09</x:v>
+      </x:c>
       <x:c r="Z118" s="14" t="str"/>
     </x:row>
     <x:row r="119" ht="84" customHeight="1">
@@ -9470,7 +9480,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J119" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K119" s="14" t="str">
         <x:v>IMP-AND-0002</x:v>
@@ -9506,9 +9516,13 @@
       <x:c r="V119" s="14" t="str">
         <x:v>chore/android-sprint-0</x:v>
       </x:c>
-      <x:c r="W119" s="14" t="str"/>
+      <x:c r="W119" s="14" t="str">
+        <x:v>Capas base, DomainMappingError y guard puro; arquitectura/typecheck PASS.</x:v>
+      </x:c>
       <x:c r="X119" s="14" t="str"/>
-      <x:c r="Y119" s="14" t="str"/>
+      <x:c r="Y119" s="14" t="str">
+        <x:v>2026-09-09</x:v>
+      </x:c>
       <x:c r="Z119" s="14" t="str"/>
     </x:row>
     <x:row r="120" ht="84" customHeight="1">
@@ -9540,7 +9554,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J120" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K120" s="14" t="str">
         <x:v>IMP-AND-0004</x:v>
@@ -9576,9 +9590,13 @@
       <x:c r="V120" s="14" t="str">
         <x:v>chore/android-sprint-0</x:v>
       </x:c>
-      <x:c r="W120" s="14" t="str"/>
+      <x:c r="W120" s="14" t="str">
+        <x:v>FetchTransport, environment y errores tipados; sin endpoints; transport tests PASS.</x:v>
+      </x:c>
       <x:c r="X120" s="14" t="str"/>
-      <x:c r="Y120" s="14" t="str"/>
+      <x:c r="Y120" s="14" t="str">
+        <x:v>2026-09-09</x:v>
+      </x:c>
       <x:c r="Z120" s="14" t="str"/>
     </x:row>
     <x:row r="121" ht="84" customHeight="1">
@@ -9610,7 +9628,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J121" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K121" s="14" t="str">
         <x:v>IMP-AND-0002</x:v>
@@ -9646,9 +9664,13 @@
       <x:c r="V121" s="14" t="str">
         <x:v>chore/android-sprint-0</x:v>
       </x:c>
-      <x:c r="W121" s="14" t="str"/>
+      <x:c r="W121" s="14" t="str">
+        <x:v>Jest + RNTL: 4 suites / 8 tests PASS.</x:v>
+      </x:c>
       <x:c r="X121" s="14" t="str"/>
-      <x:c r="Y121" s="14" t="str"/>
+      <x:c r="Y121" s="14" t="str">
+        <x:v>2026-09-09</x:v>
+      </x:c>
       <x:c r="Z121" s="14" t="str"/>
     </x:row>
     <x:row r="122" ht="84" customHeight="1">
@@ -9680,7 +9702,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J122" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K122" s="14" t="str">
         <x:v>IMP-AND-0002, IMP-AND-0003</x:v>
@@ -9695,13 +9717,13 @@
         <x:v>N/A</x:v>
       </x:c>
       <x:c r="O122" s="14" t="str">
-        <x:v>Configurar navegación técnica</x:v>
+        <x:v>Configurar navegación técnica Foundation</x:v>
       </x:c>
       <x:c r="P122" s="14" t="str">
-        <x:v>Destinations Stay/Account/Loyalty/States sin screens finales; back stack policy.</x:v>
+        <x:v>Usar únicamente app/_layout.tsx, app/index.tsx, app/(guest)/_layout.tsx y app/(guest)/index.tsx; probar navegación/back stack con renderRouter in-memory; no crear rutas funcionales.</x:v>
       </x:c>
       <x:c r="Q122" s="14" t="str">
-        <x:v>Navigation compila; 0 business logic placeholder.</x:v>
+        <x:v>Navegación y back stack compilan y pasan; una sola pantalla técnica Foundation; 0 lógica de negocio o reproducción Figma.</x:v>
       </x:c>
       <x:c r="R122" s="14" t="str">
         <x:v>Stack/navigation approved.</x:v>
@@ -9710,18 +9732,24 @@
         <x:v>Navigation smoke.</x:v>
       </x:c>
       <x:c r="T122" s="14" t="str">
-        <x:v>ui smoke</x:v>
+        <x:v>smoke de navegación con expo-router/testing-library</x:v>
       </x:c>
       <x:c r="U122" s="14" t="str">
-        <x:v>navigation foundation</x:v>
+        <x:v>app/_layout.tsx, app/index.tsx, app/(guest)/_layout.tsx, app/(guest)/index.tsx y test navegación</x:v>
       </x:c>
       <x:c r="V122" s="14" t="str">
         <x:v>chore/android-sprint-0</x:v>
       </x:c>
-      <x:c r="W122" s="14" t="str"/>
+      <x:c r="W122" s="14" t="str">
+        <x:v>Expo Router Guest Foundation y renderRouter/back stack PASS; sin rutas funcionales.</x:v>
+      </x:c>
       <x:c r="X122" s="14" t="str"/>
-      <x:c r="Y122" s="14" t="str"/>
-      <x:c r="Z122" s="14" t="str"/>
+      <x:c r="Y122" s="14" t="str">
+        <x:v>2026-09-09</x:v>
+      </x:c>
+      <x:c r="Z122" s="14" t="str">
+        <x:v>Alcance de rutas ajustado por decisión aprobada: solo Foundation Guest en Sprint 0.</x:v>
+      </x:c>
     </x:row>
     <x:row r="123" ht="84" customHeight="1">
       <x:c r="A123" s="14" t="str">
@@ -9752,7 +9780,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J123" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K123" s="14" t="str">
         <x:v>IMP-AND-0004, IMP-AND-0005</x:v>
@@ -9788,9 +9816,13 @@
       <x:c r="V123" s="14" t="str">
         <x:v>chore/android-sprint-0</x:v>
       </x:c>
-      <x:c r="W123" s="14" t="str"/>
+      <x:c r="W123" s="14" t="str">
+        <x:v>MockTransport y RemoteState derivado; escenarios técnicos PASS.</x:v>
+      </x:c>
       <x:c r="X123" s="14" t="str"/>
-      <x:c r="Y123" s="14" t="str"/>
+      <x:c r="Y123" s="14" t="str">
+        <x:v>2026-09-09</x:v>
+      </x:c>
       <x:c r="Z123" s="14" t="str"/>
     </x:row>
     <x:row r="124" ht="84" customHeight="1">
@@ -9822,7 +9854,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J124" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K124" s="14" t="str">
         <x:v>IMP-AND-0002, IMP-AND-0003, IMP-AND-0004, IMP-AND-0005, IMP-AND-0006, IMP-AND-0007, IMP-AND-0008</x:v>
@@ -9860,9 +9892,13 @@
       <x:c r="V124" s="14" t="str">
         <x:v>chore/android-sprint-0</x:v>
       </x:c>
-      <x:c r="W124" s="14" t="str"/>
+      <x:c r="W124" s="14" t="str">
+        <x:v>npm ci PASS; expo-doctor 21/21 PASS; lint PASS; typecheck PASS; test PASS: 4 suites / 8 tests; expo export PASS; npm run check PASS; revisión final: 0 features.</x:v>
+      </x:c>
       <x:c r="X124" s="14" t="str"/>
-      <x:c r="Y124" s="14" t="str"/>
+      <x:c r="Y124" s="14" t="str">
+        <x:v>2026-09-09</x:v>
+      </x:c>
       <x:c r="Z124" s="14" t="str"/>
     </x:row>
     <x:row r="125" ht="84" customHeight="1">
@@ -11212,7 +11248,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e75d91040da4275"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1056817bd8e84520"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(android): add ReservationStay contract
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="Rcf6db0241c664943"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="Rfdf00f631d2c405d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Raff21bc3ef814ec2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R64fd4fd14d7b4394"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Ra56c032c8b0b4658"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Re9429219fbcf454b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R797ddfe8a5824fbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R2fd8b05e27b144c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Rd0093aa30a4b4f5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="Rd12dca6e5517456d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Rb693af0e52824a04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Ree0320944eb6463a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdcd18f1515184f6c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2a520e53b73a4d41"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -820,7 +820,7 @@
       </x:c>
       <x:c r="F6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -888,7 +888,7 @@
       </x:c>
       <x:c r="G11" t="n">
         <x:f>COUNTIFS('01_Backlog'!C2:C142,E11,'01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd88c3d51a4544fd8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4f32fc88d1b43e8"/>
 </x:worksheet>
 </file>
 
@@ -9930,7 +9930,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J125" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K125" s="14" t="str">
         <x:v>IMP-AND-0009</x:v>
@@ -9968,10 +9968,18 @@
       <x:c r="V125" s="14" t="str">
         <x:v>feature/android-stay-contract</x:v>
       </x:c>
-      <x:c r="W125" s="14" t="str"/>
-      <x:c r="X125" s="14" t="str"/>
-      <x:c r="Y125" s="14" t="str"/>
-      <x:c r="Z125" s="14" t="str"/>
+      <x:c r="W125" s="14" t="str">
+        <x:v>Mapper/MockStayService PASS; npm run check PASS (lint, doctor 21/21, typecheck, 5 suites/11 tests y export).</x:v>
+      </x:c>
+      <x:c r="X125" s="14" t="str">
+        <x:v>2026-09-10</x:v>
+      </x:c>
+      <x:c r="Y125" s="14" t="str">
+        <x:v>2026-09-10</x:v>
+      </x:c>
+      <x:c r="Z125" s="14" t="str">
+        <x:v>Contrato local de mock; no representa endpoint ni contrato API confirmado. Sin endpoint, UI ni enum de StayStatus inventado.</x:v>
+      </x:c>
     </x:row>
     <x:row r="126" ht="84" customHeight="1">
       <x:c r="A126" s="14" t="str">
@@ -11248,7 +11256,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1056817bd8e84520"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red6b7856158f4549"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(android): implement stay home (IMP-AND-0102)
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R797ddfe8a5824fbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R2fd8b05e27b144c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Rd0093aa30a4b4f5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="Rd12dca6e5517456d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Rb693af0e52824a04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Ree0320944eb6463a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R6e8acb802c2642b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="Rf9135b304f0b4463"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R52b872c90a3e4b53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R960caaa4cabe4fe8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R847815e4204b4f39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R66bb3d45d8a046e6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2a520e53b73a4d41"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb78840587fda48fe"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -820,7 +820,7 @@
       </x:c>
       <x:c r="F6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -888,7 +888,7 @@
       </x:c>
       <x:c r="G11" t="n">
         <x:f>COUNTIFS('01_Backlog'!C2:C142,E11,'01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4f32fc88d1b43e8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd90fa1df703d4d89"/>
 </x:worksheet>
 </file>
 
@@ -10010,16 +10010,16 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J126" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K126" s="14" t="str">
         <x:v>IMP-AND-0101</x:v>
       </x:c>
       <x:c r="L126" s="14" t="str">
-        <x:v>Android 01 Estancia y servicios</x:v>
+        <x:v>Reference — Android Early Journey (excepción IMP-AND-0102)</x:v>
       </x:c>
       <x:c r="M126" s="14" t="str">
-        <x:v>238:132</x:v>
+        <x:v>31:154</x:v>
       </x:c>
       <x:c r="N126" s="14" t="str">
         <x:v>Stay Home</x:v>
@@ -10034,7 +10034,7 @@
         <x:v>No DTO UI; navigation a services; offline explicit.</x:v>
       </x:c>
       <x:c r="R126" s="14" t="str">
-        <x:v>0101 COMPLETADA.</x:v>
+        <x:v>0101 COMPLETADA. Excepción Figma 31:154 aprobada.</x:v>
       </x:c>
       <x:c r="S126" s="14" t="str">
         <x:v>UI + visual.</x:v>
@@ -10048,10 +10048,18 @@
       <x:c r="V126" s="14" t="str">
         <x:v>feature/android-stay-home</x:v>
       </x:c>
-      <x:c r="W126" s="14" t="str"/>
-      <x:c r="X126" s="14" t="str"/>
-      <x:c r="Y126" s="14" t="str"/>
-      <x:c r="Z126" s="14" t="str"/>
+      <x:c r="W126" s="14" t="str">
+        <x:v>PASS: validación visual Android contra 31:154. StayStatus opaco visible; room nullable, loading/error/offline y back stack PASS. Offline se deriva antes de empty. npm run check PASS: lint, doctor 21/21, typecheck, Jest 6 suites/15, export.</x:v>
+      </x:c>
+      <x:c r="X126" s="14" t="str">
+        <x:v>2026-09-10</x:v>
+      </x:c>
+      <x:c r="Y126" s="14" t="str">
+        <x:v>2026-09-10</x:v>
+      </x:c>
+      <x:c r="Z126" s="14" t="str">
+        <x:v>Excepción exclusiva: 31:154 MOB-02. No sustituir por 238:133, 240:193 ni otra pantalla V2/V3.</x:v>
+      </x:c>
     </x:row>
     <x:row r="127" ht="84" customHeight="1">
       <x:c r="A127" s="14" t="str">
@@ -11256,7 +11264,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red6b7856158f4549"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70f013f1ebae4690"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(android): propose services contract for IMP-AND-0103
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R6e8acb802c2642b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="Rf9135b304f0b4463"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R52b872c90a3e4b53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R960caaa4cabe4fe8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R847815e4204b4f39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R66bb3d45d8a046e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R7debb747189f45f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="Raa7d00039f6448e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Rd883eac1d4e34503"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R056df23bde604d75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Rdf79408cd22e4b4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R4635319086744c4e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb78840587fda48fe"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R151fa26068e9432f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd90fa1df703d4d89"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97955a77f35a48a3"/>
 </x:worksheet>
 </file>
 
@@ -10128,7 +10128,9 @@
       <x:c r="V127" s="14" t="str">
         <x:v>feature/android-services</x:v>
       </x:c>
-      <x:c r="W127" s="14" t="str"/>
+      <x:c r="W127" s="14" t="str">
+        <x:v>Propuesta pendiente de revisión: frontend/pms-hotel-android/docs/16_SERVICES_CONTRACT_PROPOSAL.md. No es contrato aprobado; DoR Service contract ready continúa pendiente.</x:v>
+      </x:c>
       <x:c r="X127" s="14" t="str"/>
       <x:c r="Y127" s="14" t="str"/>
       <x:c r="Z127" s="14" t="str"/>
@@ -11264,7 +11266,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70f013f1ebae4690"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8c962ad8c6a4b30"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(android): propose frontend-first services contract
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R7debb747189f45f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="Raa7d00039f6448e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Rd883eac1d4e34503"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R056df23bde604d75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Rdf79408cd22e4b4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R4635319086744c4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R9fb7675efe314cc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="Raec40e4f9a9047cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Rd6e1bdc865034a9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="Ra3f6a5b2a89e42f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R7257daea11f74d5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Rc8e93f85d04240d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R151fa26068e9432f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra74c60d67c2b410c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97955a77f35a48a3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6df0ab6698a04cad"/>
 </x:worksheet>
 </file>
 
@@ -10129,7 +10129,7 @@
         <x:v>feature/android-services</x:v>
       </x:c>
       <x:c r="W127" s="14" t="str">
-        <x:v>Propuesta pendiente de revisión: frontend/pms-hotel-android/docs/16_SERVICES_CONTRACT_PROPOSAL.md. No es contrato aprobado; DoR Service contract ready continúa pendiente.</x:v>
+        <x:v>Propuesta frontend-first pendiente de revisión: frontend/pms-hotel-android/docs/16_SERVICES_CONTRACT_PROPOSAL.md. Reemplazo candidato de DoR documentado; Service contract ready sigue vigente y no cumplido. IMP-AND-0103 permanece PENDIENTE.</x:v>
       </x:c>
       <x:c r="X127" s="14" t="str"/>
       <x:c r="Y127" s="14" t="str"/>
@@ -11266,7 +11266,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8c962ad8c6a4b30"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cf6c74838f64b35"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(android): approve V3 navigation and frontend-first contract
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R9fb7675efe314cc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="Raec40e4f9a9047cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Rd6e1bdc865034a9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="Ra3f6a5b2a89e42f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R7257daea11f74d5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Rc8e93f85d04240d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R64f8d28645274f9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R5df768171ff14a6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R3a5f013e26274fd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="Rb1d35938644d495f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R58a53252fb974a4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Raf6741aa85bd4906"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra74c60d67c2b410c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5b934b47dba94480"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6df0ab6698a04cad"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf26dc0040c9843b4"/>
 </x:worksheet>
 </file>
 
@@ -9903,7 +9903,7 @@
     </x:row>
     <x:row r="125" ht="84" customHeight="1">
       <x:c r="A125" s="14" t="str">
-        <x:v>IMP-AND-0101</x:v>
+        <x:v>IMP-AND-0100</x:v>
       </x:c>
       <x:c r="B125" s="14" t="str">
         <x:v>S1 Android Stay &amp; Services</x:v>
@@ -9912,25 +9912,25 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D125" s="14" t="str">
-        <x:v>Estancia</x:v>
+        <x:v>Navigation</x:v>
       </x:c>
       <x:c r="E125" s="14" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F125" s="14" t="str">
-        <x:v>WEB-3</x:v>
+        <x:v>PENDIENTE DE DESIGNACIÓN</x:v>
       </x:c>
       <x:c r="G125" s="14" t="str">
-        <x:v>stay</x:v>
+        <x:v>navigation</x:v>
       </x:c>
       <x:c r="H125" s="14" t="str">
-        <x:v>FEATURE</x:v>
+        <x:v>INFRA</x:v>
       </x:c>
       <x:c r="I125" s="14" t="str">
-        <x:v>CRÍTICA</x:v>
+        <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J125" s="14" t="str">
-        <x:v>COMPLETADA</x:v>
+        <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K125" s="14" t="str">
         <x:v>IMP-AND-0009</x:v>
@@ -9942,48 +9942,44 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N125" s="14" t="str">
-        <x:v>Stay Home</x:v>
+        <x:v>Guest shell</x:v>
       </x:c>
       <x:c r="O125" s="14" t="str">
-        <x:v>Crear Stay contracts</x:v>
+        <x:v>Implementar Android Guest Navigation Shell V3</x:v>
       </x:c>
       <x:c r="P125" s="14" t="str">
-        <x:v>ReservationStay/room/dates/status DTO-&gt;Domain; mock remote.</x:v>
+        <x:v>Shell Guest compartido; Servicios/Chat/Valet/Cuenta; selected state; Expo Router; back stack; tabs accesibles; destinos no implementados; decisión explícita sobre Home V2.</x:v>
       </x:c>
       <x:c r="Q125" s="14" t="str">
-        <x:v>Reservation != Stay; mapper tests; UI-ready Domain.</x:v>
+        <x:v>Features V3 consumen un shell único; no footbars privadas; item seleccionado y destinos no implementados son accesibles y semánticamente honestos; IMP-AND-0102 no se modifica; back stack PASS.</x:v>
       </x:c>
       <x:c r="R125" s="14" t="str">
-        <x:v>S0 Android complete.</x:v>
+        <x:v>IMP-AND-0009 COMPLETADA; owner y reviewer designados; 238:132 y pantallas V3 verificadas; política de destinos no implementados, selección y accesibilidad aprobada; Home V2 no migra en esta tarea; rutas Guest y back stack definidos.</x:v>
       </x:c>
       <x:c r="S125" s="14" t="str">
-        <x:v>Unit mapper/service.</x:v>
+        <x:v>Shell Guest V3 compartido Servicios/Chat/Valet/Cuenta; punto único sin footbars privadas; tab activo; destinos accesibles y honestos; Expo Router/back stack/a11y/tab tests PASS; Figma 238:132 PASS; IMP-AND-0102 intacta; lint, typecheck, test y check PASS.</x:v>
       </x:c>
       <x:c r="T125" s="14" t="str">
-        <x:v>unit</x:v>
+        <x:v>unit/ui navigation con expo-router/testing-library</x:v>
       </x:c>
       <x:c r="U125" s="14" t="str">
-        <x:v>stay layers</x:v>
+        <x:v>shared navigation shell y tests de navegación</x:v>
       </x:c>
       <x:c r="V125" s="14" t="str">
-        <x:v>feature/android-stay-contract</x:v>
+        <x:v>feature/android-guest-navigation-shell</x:v>
       </x:c>
       <x:c r="W125" s="14" t="str">
-        <x:v>Mapper/MockStayService PASS; npm run check PASS (lint, doctor 21/21, typecheck, 5 suites/11 tests y export).</x:v>
-      </x:c>
-      <x:c r="X125" s="14" t="str">
-        <x:v>2026-09-10</x:v>
-      </x:c>
-      <x:c r="Y125" s="14" t="str">
-        <x:v>2026-09-10</x:v>
-      </x:c>
+        <x:v>Change Control aprobado. IMP-AND-0100 permanece PENDIENTE, no READY: reviewer por designar y DoR operativo pendiente.</x:v>
+      </x:c>
+      <x:c r="X125" s="14"/>
+      <x:c r="Y125" s="14"/>
       <x:c r="Z125" s="14" t="str">
-        <x:v>Contrato local de mock; no representa endpoint ni contrato API confirmado. Sin endpoint, UI ni enum de StayStatus inventado.</x:v>
+        <x:v>No crea un módulo nuevo; usa el módulo navigation existente.</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="84" customHeight="1">
       <x:c r="A126" s="14" t="str">
-        <x:v>IMP-AND-0102</x:v>
+        <x:v>IMP-AND-0101</x:v>
       </x:c>
       <x:c r="B126" s="14" t="str">
         <x:v>S1 Android Stay &amp; Services</x:v>
@@ -10013,43 +10009,43 @@
         <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K126" s="14" t="str">
-        <x:v>IMP-AND-0101</x:v>
+        <x:v>IMP-AND-0009</x:v>
       </x:c>
       <x:c r="L126" s="14" t="str">
-        <x:v>Reference — Android Early Journey (excepción IMP-AND-0102)</x:v>
+        <x:v>Android 01 Estancia y servicios</x:v>
       </x:c>
       <x:c r="M126" s="14" t="str">
-        <x:v>31:154</x:v>
+        <x:v>238:132</x:v>
       </x:c>
       <x:c r="N126" s="14" t="str">
         <x:v>Stay Home</x:v>
       </x:c>
       <x:c r="O126" s="14" t="str">
-        <x:v>Implementar pantalla Estancia</x:v>
+        <x:v>Crear Stay contracts</x:v>
       </x:c>
       <x:c r="P126" s="14" t="str">
-        <x:v>Room/type/dates/status/actions; loading/error/offline; Figma.</x:v>
+        <x:v>ReservationStay/room/dates/status DTO-&gt;Domain; mock remote.</x:v>
       </x:c>
       <x:c r="Q126" s="14" t="str">
-        <x:v>No DTO UI; navigation a services; offline explicit.</x:v>
+        <x:v>Reservation != Stay; mapper tests; UI-ready Domain.</x:v>
       </x:c>
       <x:c r="R126" s="14" t="str">
-        <x:v>0101 COMPLETADA. Excepción Figma 31:154 aprobada.</x:v>
+        <x:v>S0 Android complete.</x:v>
       </x:c>
       <x:c r="S126" s="14" t="str">
-        <x:v>UI + visual.</x:v>
+        <x:v>Unit mapper/service.</x:v>
       </x:c>
       <x:c r="T126" s="14" t="str">
-        <x:v>unit/ui</x:v>
+        <x:v>unit</x:v>
       </x:c>
       <x:c r="U126" s="14" t="str">
-        <x:v>stay screen</x:v>
+        <x:v>stay layers</x:v>
       </x:c>
       <x:c r="V126" s="14" t="str">
-        <x:v>feature/android-stay-home</x:v>
+        <x:v>feature/android-stay-contract</x:v>
       </x:c>
       <x:c r="W126" s="14" t="str">
-        <x:v>PASS: validación visual Android contra 31:154. StayStatus opaco visible; room nullable, loading/error/offline y back stack PASS. Offline se deriva antes de empty. npm run check PASS: lint, doctor 21/21, typecheck, Jest 6 suites/15, export.</x:v>
+        <x:v>Mapper/MockStayService PASS; npm run check PASS (lint, doctor 21/21, typecheck, 5 suites/11 tests y export).</x:v>
       </x:c>
       <x:c r="X126" s="14" t="str">
         <x:v>2026-09-10</x:v>
@@ -10058,12 +10054,12 @@
         <x:v>2026-09-10</x:v>
       </x:c>
       <x:c r="Z126" s="14" t="str">
-        <x:v>Excepción exclusiva: 31:154 MOB-02. No sustituir por 238:133, 240:193 ni otra pantalla V2/V3.</x:v>
+        <x:v>Contrato local de mock; no representa endpoint ni contrato API confirmado. Sin endpoint, UI ni enum de StayStatus inventado.</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="84" customHeight="1">
       <x:c r="A127" s="14" t="str">
-        <x:v>IMP-AND-0103</x:v>
+        <x:v>IMP-AND-0102</x:v>
       </x:c>
       <x:c r="B127" s="14" t="str">
         <x:v>S1 Android Stay &amp; Services</x:v>
@@ -10072,7 +10068,7 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D127" s="14" t="str">
-        <x:v>Servicios</x:v>
+        <x:v>Estancia</x:v>
       </x:c>
       <x:c r="E127" s="14" t="str">
         <x:v>ANDROID-1</x:v>
@@ -10081,63 +10077,69 @@
         <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G127" s="14" t="str">
-        <x:v>services</x:v>
+        <x:v>stay</x:v>
       </x:c>
       <x:c r="H127" s="14" t="str">
         <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I127" s="14" t="str">
-        <x:v>ALTA</x:v>
+        <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J127" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K127" s="14" t="str">
-        <x:v>IMP-AND-0102</x:v>
+        <x:v>IMP-AND-0101</x:v>
       </x:c>
       <x:c r="L127" s="14" t="str">
-        <x:v>Android 01 Estancia y servicios</x:v>
+        <x:v>Reference — Android Early Journey (excepción IMP-AND-0102)</x:v>
       </x:c>
       <x:c r="M127" s="14" t="str">
-        <x:v>238:132</x:v>
+        <x:v>31:154</x:v>
       </x:c>
       <x:c r="N127" s="14" t="str">
-        <x:v>Services</x:v>
+        <x:v>Stay Home</x:v>
       </x:c>
       <x:c r="O127" s="14" t="str">
-        <x:v>Implementar servicios y solicitud</x:v>
+        <x:v>Implementar pantalla Estancia</x:v>
       </x:c>
       <x:c r="P127" s="14" t="str">
-        <x:v>Catalog DTO-&gt;Domain; detail/request; submitting/success/error/offline.</x:v>
+        <x:v>Room/type/dates/status/actions; loading/error/offline; Figma.</x:v>
       </x:c>
       <x:c r="Q127" s="14" t="str">
-        <x:v>Only services current stay/property; no false success/double submit.</x:v>
+        <x:v>No DTO UI; navigation a services; offline explicit.</x:v>
       </x:c>
       <x:c r="R127" s="14" t="str">
-        <x:v>Service contract ready.</x:v>
+        <x:v>0101 COMPLETADA. Excepción Figma 31:154 aprobada.</x:v>
       </x:c>
       <x:c r="S127" s="14" t="str">
-        <x:v>Mapper + UI.</x:v>
+        <x:v>UI + visual.</x:v>
       </x:c>
       <x:c r="T127" s="14" t="str">
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U127" s="14" t="str">
-        <x:v>services module</x:v>
+        <x:v>stay screen</x:v>
       </x:c>
       <x:c r="V127" s="14" t="str">
-        <x:v>feature/android-services</x:v>
+        <x:v>feature/android-stay-home</x:v>
       </x:c>
       <x:c r="W127" s="14" t="str">
-        <x:v>Propuesta frontend-first pendiente de revisión: frontend/pms-hotel-android/docs/16_SERVICES_CONTRACT_PROPOSAL.md. Reemplazo candidato de DoR documentado; Service contract ready sigue vigente y no cumplido. IMP-AND-0103 permanece PENDIENTE.</x:v>
-      </x:c>
-      <x:c r="X127" s="14" t="str"/>
-      <x:c r="Y127" s="14" t="str"/>
-      <x:c r="Z127" s="14" t="str"/>
+        <x:v>PASS: validación visual Android contra 31:154. StayStatus opaco visible; room nullable, loading/error/offline y back stack PASS. Offline se deriva antes de empty. npm run check PASS: lint, doctor 21/21, typecheck, Jest 6 suites/15, export.</x:v>
+      </x:c>
+      <x:c r="X127" s="14" t="str">
+        <x:v>2026-09-10</x:v>
+      </x:c>
+      <x:c r="Y127" s="14" t="str">
+        <x:v>2026-09-10</x:v>
+      </x:c>
+      <x:c r="Z127" s="14" t="str">
+        <x:v>Excepción exclusiva: 31:154 MOB-02. No sustituir por 238:133, 240:193 ni otra pantalla V2/V3.</x:v>
+      </x:c>
     </x:row>
     <x:row r="128" ht="84" customHeight="1">
       <x:c r="A128" s="14" t="str">
-        <x:v>IMP-AND-0104</x:v>
+        <x:v>IMP-AND-0103</x:v>
       </x:c>
       <x:c r="B128" s="14" t="str">
         <x:v>S1 Android Stay &amp; Services</x:v>
@@ -10146,7 +10148,7 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D128" s="14" t="str">
-        <x:v>Chat</x:v>
+        <x:v>Servicios</x:v>
       </x:c>
       <x:c r="E128" s="14" t="str">
         <x:v>ANDROID-1</x:v>
@@ -10155,7 +10157,7 @@
         <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G128" s="14" t="str">
-        <x:v>messaging</x:v>
+        <x:v>services</x:v>
       </x:c>
       <x:c r="H128" s="14" t="str">
         <x:v>FEATURE</x:v>
@@ -10167,7 +10169,7 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K128" s="14" t="str">
-        <x:v>IMP-AND-0102</x:v>
+        <x:v>IMP-AND-0100, IMP-AND-0102</x:v>
       </x:c>
       <x:c r="L128" s="14" t="str">
         <x:v>Android 01 Estancia y servicios</x:v>
@@ -10176,40 +10178,42 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N128" s="14" t="str">
-        <x:v>Chat</x:v>
+        <x:v>Services</x:v>
       </x:c>
       <x:c r="O128" s="14" t="str">
-        <x:v>Implementar chat con Recepción</x:v>
+        <x:v>Implementar servicios y solicitud</x:v>
       </x:c>
       <x:c r="P128" s="14" t="str">
-        <x:v>Thread/messages; send to Reception only; offline/error.</x:v>
+        <x:v>Catalog DTO-&gt;Domain; detail/request; submitting/success/error/offline.</x:v>
       </x:c>
       <x:c r="Q128" s="14" t="str">
-        <x:v>No direct HK/Maintenance recipient; no PII logs.</x:v>
+        <x:v>Only services current stay/property; no false success/double submit.</x:v>
       </x:c>
       <x:c r="R128" s="14" t="str">
-        <x:v>Messaging contract reviewed.</x:v>
+        <x:v>Frontend service data/mock contract approved: fuente Figma y ruta confirmadas; formas de mock para catálogo, selección y solicitud simulada; asociación con estadía/property actual sin alterar semántica de dominio; escenarios loading, submitting, success, error y offline; boundaries Mapper/UI y pruebas unitarias/UI definidos. No constituye contrato API Backend ni define endpoints, HTTP, auth, permisos, persistencia, entidades o estados de negocio Backend.</x:v>
       </x:c>
       <x:c r="S128" s="14" t="str">
-        <x:v>Mapper + UI send/offline.</x:v>
+        <x:v>Mapper + UI.</x:v>
       </x:c>
       <x:c r="T128" s="14" t="str">
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U128" s="14" t="str">
-        <x:v>messaging</x:v>
+        <x:v>services module</x:v>
       </x:c>
       <x:c r="V128" s="14" t="str">
-        <x:v>feature/android-chat</x:v>
-      </x:c>
-      <x:c r="W128" s="14" t="str"/>
-      <x:c r="X128" s="14" t="str"/>
-      <x:c r="Y128" s="14" t="str"/>
-      <x:c r="Z128" s="14" t="str"/>
+        <x:v>feature/android-services</x:v>
+      </x:c>
+      <x:c r="W128" s="14" t="str">
+        <x:v>Change Control aprobó DEC-G-013 y el DoR frontend-first. Contrato mock sigue propuesta: Figma 239:132 confirmado; faltan aprobar contrato mock y diseños Services loading/submitting/success/error/offline, y completar IMP-AND-0100. IMP-AND-0103 permanece PENDIENTE.</x:v>
+      </x:c>
+      <x:c r="X128" s="14"/>
+      <x:c r="Y128" s="14"/>
+      <x:c r="Z128" s="14"/>
     </x:row>
     <x:row r="129" ht="84" customHeight="1">
       <x:c r="A129" s="14" t="str">
-        <x:v>IMP-AND-0105</x:v>
+        <x:v>IMP-AND-0104</x:v>
       </x:c>
       <x:c r="B129" s="14" t="str">
         <x:v>S1 Android Stay &amp; Services</x:v>
@@ -10218,7 +10222,7 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D129" s="14" t="str">
-        <x:v>Valet</x:v>
+        <x:v>Chat</x:v>
       </x:c>
       <x:c r="E129" s="14" t="str">
         <x:v>ANDROID-1</x:v>
@@ -10227,13 +10231,13 @@
         <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G129" s="14" t="str">
-        <x:v>valet</x:v>
+        <x:v>messaging</x:v>
       </x:c>
       <x:c r="H129" s="14" t="str">
         <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I129" s="14" t="str">
-        <x:v>MEDIA</x:v>
+        <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J129" s="14" t="str">
         <x:v>PENDIENTE</x:v>
@@ -10248,40 +10252,40 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N129" s="14" t="str">
-        <x:v>Valet</x:v>
+        <x:v>Chat</x:v>
       </x:c>
       <x:c r="O129" s="14" t="str">
-        <x:v>Implementar Valet/Parking</x:v>
+        <x:v>Implementar chat con Recepción</x:v>
       </x:c>
       <x:c r="P129" s="14" t="str">
-        <x:v>Status/request/pickup según Figma; remote mock; offline/error.</x:v>
+        <x:v>Thread/messages; send to Reception only; offline/error.</x:v>
       </x:c>
       <x:c r="Q129" s="14" t="str">
-        <x:v>No financial assumptions fuera Figma; linked to stay/property.</x:v>
+        <x:v>No direct HK/Maintenance recipient; no PII logs.</x:v>
       </x:c>
       <x:c r="R129" s="14" t="str">
-        <x:v>Valet contract confirmed.</x:v>
+        <x:v>Messaging contract reviewed.</x:v>
       </x:c>
       <x:c r="S129" s="14" t="str">
-        <x:v>UI tests.</x:v>
+        <x:v>Mapper + UI send/offline.</x:v>
       </x:c>
       <x:c r="T129" s="14" t="str">
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U129" s="14" t="str">
-        <x:v>valet</x:v>
+        <x:v>messaging</x:v>
       </x:c>
       <x:c r="V129" s="14" t="str">
-        <x:v>feature/android-valet</x:v>
-      </x:c>
-      <x:c r="W129" s="14" t="str"/>
-      <x:c r="X129" s="14" t="str"/>
-      <x:c r="Y129" s="14" t="str"/>
-      <x:c r="Z129" s="14" t="str"/>
+        <x:v>feature/android-chat</x:v>
+      </x:c>
+      <x:c r="W129" s="14"/>
+      <x:c r="X129" s="14"/>
+      <x:c r="Y129" s="14"/>
+      <x:c r="Z129" s="14"/>
     </x:row>
     <x:row r="130" ht="84" customHeight="1">
       <x:c r="A130" s="14" t="str">
-        <x:v>IMP-AND-0106</x:v>
+        <x:v>IMP-AND-0105</x:v>
       </x:c>
       <x:c r="B130" s="14" t="str">
         <x:v>S1 Android Stay &amp; Services</x:v>
@@ -10290,7 +10294,7 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D130" s="14" t="str">
-        <x:v>QA</x:v>
+        <x:v>Valet</x:v>
       </x:c>
       <x:c r="E130" s="14" t="str">
         <x:v>ANDROID-1</x:v>
@@ -10299,19 +10303,19 @@
         <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G130" s="14" t="str">
-        <x:v>stay-services</x:v>
+        <x:v>valet</x:v>
       </x:c>
       <x:c r="H130" s="14" t="str">
-        <x:v>QA</x:v>
+        <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I130" s="14" t="str">
-        <x:v>CRÍTICA</x:v>
+        <x:v>MEDIA</x:v>
       </x:c>
       <x:c r="J130" s="14" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K130" s="14" t="str">
-        <x:v>IMP-AND-0102, IMP-AND-0103, IMP-AND-0104, IMP-AND-0105</x:v>
+        <x:v>IMP-AND-0102</x:v>
       </x:c>
       <x:c r="L130" s="14" t="str">
         <x:v>Android 01 Estancia y servicios</x:v>
@@ -10320,61 +10324,61 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N130" s="14" t="str">
-        <x:v>Stay/Services</x:v>
+        <x:v>Valet</x:v>
       </x:c>
       <x:c r="O130" s="14" t="str">
-        <x:v>QA Estancia/Servicios</x:v>
+        <x:v>Implementar Valet/Parking</x:v>
       </x:c>
       <x:c r="P130" s="14" t="str">
-        <x:v>Stay/services/chat/valet/loading/error/offline/navigation.</x:v>
+        <x:v>Status/request/pickup según Figma; remote mock; offline/error.</x:v>
       </x:c>
       <x:c r="Q130" s="14" t="str">
-        <x:v>All flows PASS; Reception boundary; Figma parity.</x:v>
+        <x:v>No financial assumptions fuera Figma; linked to stay/property.</x:v>
       </x:c>
       <x:c r="R130" s="14" t="str">
-        <x:v>S1 tasks done.</x:v>
+        <x:v>Valet contract confirmed.</x:v>
       </x:c>
       <x:c r="S130" s="14" t="str">
-        <x:v>Android Global DoD.</x:v>
+        <x:v>UI tests.</x:v>
       </x:c>
       <x:c r="T130" s="14" t="str">
-        <x:v>build/tests/manual</x:v>
+        <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U130" s="14" t="str">
-        <x:v>Android S1</x:v>
+        <x:v>valet</x:v>
       </x:c>
       <x:c r="V130" s="14" t="str">
-        <x:v>test/android-stay-services</x:v>
-      </x:c>
-      <x:c r="W130" s="14" t="str"/>
-      <x:c r="X130" s="14" t="str"/>
-      <x:c r="Y130" s="14" t="str"/>
-      <x:c r="Z130" s="14" t="str"/>
+        <x:v>feature/android-valet</x:v>
+      </x:c>
+      <x:c r="W130" s="14"/>
+      <x:c r="X130" s="14"/>
+      <x:c r="Y130" s="14"/>
+      <x:c r="Z130" s="14"/>
     </x:row>
     <x:row r="131" ht="84" customHeight="1">
       <x:c r="A131" s="14" t="str">
-        <x:v>IMP-AND-0201</x:v>
+        <x:v>IMP-AND-0106</x:v>
       </x:c>
       <x:c r="B131" s="14" t="str">
-        <x:v>S2 Android Account</x:v>
+        <x:v>S1 Android Stay &amp; Services</x:v>
       </x:c>
       <x:c r="C131" s="14" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D131" s="14" t="str">
-        <x:v>Cuenta</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="E131" s="14" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F131" s="14" t="str">
-        <x:v>WEB-2</x:v>
+        <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G131" s="14" t="str">
-        <x:v>account</x:v>
+        <x:v>stay-services</x:v>
       </x:c>
       <x:c r="H131" s="14" t="str">
-        <x:v>FEATURE</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="I131" s="14" t="str">
         <x:v>CRÍTICA</x:v>
@@ -10383,49 +10387,49 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K131" s="14" t="str">
-        <x:v>IMP-AND-0009</x:v>
+        <x:v>IMP-AND-0102, IMP-AND-0103, IMP-AND-0104, IMP-AND-0105</x:v>
       </x:c>
       <x:c r="L131" s="14" t="str">
-        <x:v>Android 02 Cuenta, checkout y factura</x:v>
+        <x:v>Android 01 Estancia y servicios</x:v>
       </x:c>
       <x:c r="M131" s="14" t="str">
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N131" s="14" t="str">
-        <x:v>Account</x:v>
+        <x:v>Stay/Services</x:v>
       </x:c>
       <x:c r="O131" s="14" t="str">
-        <x:v>Crear Account/Profile contracts</x:v>
+        <x:v>QA Estancia/Servicios</x:v>
       </x:c>
       <x:c r="P131" s="14" t="str">
-        <x:v>GuestAccount/Profile separados; remote-&gt;DTO-&gt;Mapper-&gt;Domain.</x:v>
+        <x:v>Stay/services/chat/valet/loading/error/offline/navigation.</x:v>
       </x:c>
       <x:c r="Q131" s="14" t="str">
-        <x:v>No Staff auth; no provider JSON UI; mapper tests.</x:v>
+        <x:v>All flows PASS; Reception boundary; Figma parity.</x:v>
       </x:c>
       <x:c r="R131" s="14" t="str">
-        <x:v>S0 complete.</x:v>
+        <x:v>S1 tasks done.</x:v>
       </x:c>
       <x:c r="S131" s="14" t="str">
-        <x:v>Unit.</x:v>
+        <x:v>Android Global DoD.</x:v>
       </x:c>
       <x:c r="T131" s="14" t="str">
-        <x:v>unit</x:v>
+        <x:v>build/tests/manual</x:v>
       </x:c>
       <x:c r="U131" s="14" t="str">
-        <x:v>account layers</x:v>
+        <x:v>Android S1</x:v>
       </x:c>
       <x:c r="V131" s="14" t="str">
-        <x:v>feature/android-account-contract</x:v>
-      </x:c>
-      <x:c r="W131" s="14" t="str"/>
-      <x:c r="X131" s="14" t="str"/>
-      <x:c r="Y131" s="14" t="str"/>
-      <x:c r="Z131" s="14" t="str"/>
+        <x:v>test/android-stay-services</x:v>
+      </x:c>
+      <x:c r="W131" s="14"/>
+      <x:c r="X131" s="14"/>
+      <x:c r="Y131" s="14"/>
+      <x:c r="Z131" s="14"/>
     </x:row>
     <x:row r="132" ht="84" customHeight="1">
       <x:c r="A132" s="14" t="str">
-        <x:v>IMP-AND-0202</x:v>
+        <x:v>IMP-AND-0201</x:v>
       </x:c>
       <x:c r="B132" s="14" t="str">
         <x:v>S2 Android Account</x:v>
@@ -10449,13 +10453,13 @@
         <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I132" s="14" t="str">
-        <x:v>ALTA</x:v>
+        <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J132" s="14" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K132" s="14" t="str">
-        <x:v>IMP-AND-0201</x:v>
+        <x:v>IMP-AND-0009</x:v>
       </x:c>
       <x:c r="L132" s="14" t="str">
         <x:v>Android 02 Cuenta, checkout y factura</x:v>
@@ -10464,40 +10468,40 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N132" s="14" t="str">
-        <x:v>Account/Profile</x:v>
+        <x:v>Account</x:v>
       </x:c>
       <x:c r="O132" s="14" t="str">
-        <x:v>Implementar cuenta/perfil</x:v>
+        <x:v>Crear Account/Profile contracts</x:v>
       </x:c>
       <x:c r="P132" s="14" t="str">
-        <x:v>Display/edit Profile; loading/error/offline; submit.</x:v>
+        <x:v>GuestAccount/Profile separados; remote-&gt;DTO-&gt;Mapper-&gt;Domain.</x:v>
       </x:c>
       <x:c r="Q132" s="14" t="str">
-        <x:v>Account/Profile separation; no secrets; save states correct.</x:v>
+        <x:v>No Staff auth; no provider JSON UI; mapper tests.</x:v>
       </x:c>
       <x:c r="R132" s="14" t="str">
-        <x:v>0201 complete.</x:v>
+        <x:v>S0 complete.</x:v>
       </x:c>
       <x:c r="S132" s="14" t="str">
-        <x:v>UI tests.</x:v>
+        <x:v>Unit.</x:v>
       </x:c>
       <x:c r="T132" s="14" t="str">
-        <x:v>unit/ui</x:v>
+        <x:v>unit</x:v>
       </x:c>
       <x:c r="U132" s="14" t="str">
-        <x:v>account/profile screens</x:v>
+        <x:v>account layers</x:v>
       </x:c>
       <x:c r="V132" s="14" t="str">
-        <x:v>feature/android-account-profile</x:v>
-      </x:c>
-      <x:c r="W132" s="14" t="str"/>
-      <x:c r="X132" s="14" t="str"/>
-      <x:c r="Y132" s="14" t="str"/>
-      <x:c r="Z132" s="14" t="str"/>
+        <x:v>feature/android-account-contract</x:v>
+      </x:c>
+      <x:c r="W132" s="14"/>
+      <x:c r="X132" s="14"/>
+      <x:c r="Y132" s="14"/>
+      <x:c r="Z132" s="14"/>
     </x:row>
     <x:row r="133" ht="84" customHeight="1">
       <x:c r="A133" s="14" t="str">
-        <x:v>IMP-AND-0203</x:v>
+        <x:v>IMP-AND-0202</x:v>
       </x:c>
       <x:c r="B133" s="14" t="str">
         <x:v>S2 Android Account</x:v>
@@ -10506,28 +10510,28 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D133" s="14" t="str">
-        <x:v>Checkout/Factura</x:v>
+        <x:v>Cuenta</x:v>
       </x:c>
       <x:c r="E133" s="14" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F133" s="14" t="str">
-        <x:v>WEB-4</x:v>
+        <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G133" s="14" t="str">
-        <x:v>checkout</x:v>
+        <x:v>account</x:v>
       </x:c>
       <x:c r="H133" s="14" t="str">
         <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I133" s="14" t="str">
-        <x:v>CRÍTICA</x:v>
+        <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J133" s="14" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K133" s="14" t="str">
-        <x:v>IMP-AND-0102</x:v>
+        <x:v>IMP-AND-0201</x:v>
       </x:c>
       <x:c r="L133" s="14" t="str">
         <x:v>Android 02 Cuenta, checkout y factura</x:v>
@@ -10536,40 +10540,40 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N133" s="14" t="str">
-        <x:v>Checkout/Invoice</x:v>
+        <x:v>Account/Profile</x:v>
       </x:c>
       <x:c r="O133" s="14" t="str">
-        <x:v>Implementar checkout e invoice</x:v>
+        <x:v>Implementar cuenta/perfil</x:v>
       </x:c>
       <x:c r="P133" s="14" t="str">
-        <x:v>Charges/balance/status Folio read model; invoice ref/status/date/total; offline/error.</x:v>
+        <x:v>Display/edit Profile; loading/error/offline; submit.</x:v>
       </x:c>
       <x:c r="Q133" s="14" t="str">
-        <x:v>Finance no recalculated in UI; no sensitive file persisted; no provider raw data.</x:v>
+        <x:v>Account/Profile separation; no secrets; save states correct.</x:v>
       </x:c>
       <x:c r="R133" s="14" t="str">
-        <x:v>Folio/Fiscal mobile contract reviewed.</x:v>
+        <x:v>0201 complete.</x:v>
       </x:c>
       <x:c r="S133" s="14" t="str">
-        <x:v>Mapper + UI/security.</x:v>
+        <x:v>UI tests.</x:v>
       </x:c>
       <x:c r="T133" s="14" t="str">
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U133" s="14" t="str">
-        <x:v>checkout/invoice</x:v>
+        <x:v>account/profile screens</x:v>
       </x:c>
       <x:c r="V133" s="14" t="str">
-        <x:v>feature/android-checkout-invoice</x:v>
-      </x:c>
-      <x:c r="W133" s="14" t="str"/>
-      <x:c r="X133" s="14" t="str"/>
-      <x:c r="Y133" s="14" t="str"/>
-      <x:c r="Z133" s="14" t="str"/>
+        <x:v>feature/android-account-profile</x:v>
+      </x:c>
+      <x:c r="W133" s="14"/>
+      <x:c r="X133" s="14"/>
+      <x:c r="Y133" s="14"/>
+      <x:c r="Z133" s="14"/>
     </x:row>
     <x:row r="134" ht="84" customHeight="1">
       <x:c r="A134" s="14" t="str">
-        <x:v>IMP-AND-0204</x:v>
+        <x:v>IMP-AND-0203</x:v>
       </x:c>
       <x:c r="B134" s="14" t="str">
         <x:v>S2 Android Account</x:v>
@@ -10578,19 +10582,19 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D134" s="14" t="str">
-        <x:v>QA</x:v>
+        <x:v>Checkout/Factura</x:v>
       </x:c>
       <x:c r="E134" s="14" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F134" s="14" t="str">
-        <x:v>WEB-2</x:v>
+        <x:v>WEB-4</x:v>
       </x:c>
       <x:c r="G134" s="14" t="str">
-        <x:v>account-checkout</x:v>
+        <x:v>checkout</x:v>
       </x:c>
       <x:c r="H134" s="14" t="str">
-        <x:v>QA</x:v>
+        <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I134" s="14" t="str">
         <x:v>CRÍTICA</x:v>
@@ -10599,7 +10603,7 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K134" s="14" t="str">
-        <x:v>IMP-AND-0202, IMP-AND-0203</x:v>
+        <x:v>IMP-AND-0102</x:v>
       </x:c>
       <x:c r="L134" s="14" t="str">
         <x:v>Android 02 Cuenta, checkout y factura</x:v>
@@ -10608,49 +10612,49 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N134" s="14" t="str">
-        <x:v>Account/Checkout</x:v>
+        <x:v>Checkout/Invoice</x:v>
       </x:c>
       <x:c r="O134" s="14" t="str">
-        <x:v>QA Cuenta/Checkout/Factura</x:v>
+        <x:v>Implementar checkout e invoice</x:v>
       </x:c>
       <x:c r="P134" s="14" t="str">
-        <x:v>Profile/checkout/invoice/states/navigation/contracts.</x:v>
+        <x:v>Charges/balance/status Folio read model; invoice ref/status/date/total; offline/error.</x:v>
       </x:c>
       <x:c r="Q134" s="14" t="str">
-        <x:v>Guest/Staff separation; finance coherent; Figma parity.</x:v>
+        <x:v>Finance no recalculated in UI; no sensitive file persisted; no provider raw data.</x:v>
       </x:c>
       <x:c r="R134" s="14" t="str">
-        <x:v>S2 done.</x:v>
+        <x:v>Folio/Fiscal mobile contract reviewed.</x:v>
       </x:c>
       <x:c r="S134" s="14" t="str">
-        <x:v>Android Global DoD.</x:v>
+        <x:v>Mapper + UI/security.</x:v>
       </x:c>
       <x:c r="T134" s="14" t="str">
-        <x:v>build/tests/manual</x:v>
+        <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U134" s="14" t="str">
-        <x:v>Android S2</x:v>
+        <x:v>checkout/invoice</x:v>
       </x:c>
       <x:c r="V134" s="14" t="str">
-        <x:v>test/android-account-checkout</x:v>
-      </x:c>
-      <x:c r="W134" s="14" t="str"/>
-      <x:c r="X134" s="14" t="str"/>
-      <x:c r="Y134" s="14" t="str"/>
-      <x:c r="Z134" s="14" t="str"/>
+        <x:v>feature/android-checkout-invoice</x:v>
+      </x:c>
+      <x:c r="W134" s="14"/>
+      <x:c r="X134" s="14"/>
+      <x:c r="Y134" s="14"/>
+      <x:c r="Z134" s="14"/>
     </x:row>
     <x:row r="135" ht="84" customHeight="1">
       <x:c r="A135" s="14" t="str">
-        <x:v>IMP-AND-0301</x:v>
+        <x:v>IMP-AND-0204</x:v>
       </x:c>
       <x:c r="B135" s="14" t="str">
-        <x:v>S3 Android Loyalty</x:v>
+        <x:v>S2 Android Account</x:v>
       </x:c>
       <x:c r="C135" s="14" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D135" s="14" t="str">
-        <x:v>Loyalty</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="E135" s="14" t="str">
         <x:v>ANDROID-1</x:v>
@@ -10659,61 +10663,61 @@
         <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G135" s="14" t="str">
-        <x:v>rewards</x:v>
+        <x:v>account-checkout</x:v>
       </x:c>
       <x:c r="H135" s="14" t="str">
-        <x:v>FEATURE</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="I135" s="14" t="str">
-        <x:v>ALTA</x:v>
+        <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J135" s="14" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K135" s="14" t="str">
-        <x:v>IMP-AND-0009</x:v>
+        <x:v>IMP-AND-0202, IMP-AND-0203</x:v>
       </x:c>
       <x:c r="L135" s="14" t="str">
-        <x:v>Android 03 Loyalty, promociones y perfil</x:v>
+        <x:v>Android 02 Cuenta, checkout y factura</x:v>
       </x:c>
       <x:c r="M135" s="14" t="str">
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N135" s="14" t="str">
-        <x:v>Rewards</x:v>
+        <x:v>Account/Checkout</x:v>
       </x:c>
       <x:c r="O135" s="14" t="str">
-        <x:v>Implementar Rewards</x:v>
+        <x:v>QA Cuenta/Checkout/Factura</x:v>
       </x:c>
       <x:c r="P135" s="14" t="str">
-        <x:v>Ledger/balance Domain cross-app; offline/error/empty.</x:v>
+        <x:v>Profile/checkout/invoice/states/navigation/contracts.</x:v>
       </x:c>
       <x:c r="Q135" s="14" t="str">
-        <x:v>CANCELLED/NO_SHOW no elegibles; ledger read-only.</x:v>
+        <x:v>Guest/Staff separation; finance coherent; Figma parity.</x:v>
       </x:c>
       <x:c r="R135" s="14" t="str">
-        <x:v>Reward contract reviewed.</x:v>
+        <x:v>S2 done.</x:v>
       </x:c>
       <x:c r="S135" s="14" t="str">
-        <x:v>Mapper + UI.</x:v>
+        <x:v>Android Global DoD.</x:v>
       </x:c>
       <x:c r="T135" s="14" t="str">
-        <x:v>unit/ui</x:v>
+        <x:v>build/tests/manual</x:v>
       </x:c>
       <x:c r="U135" s="14" t="str">
-        <x:v>rewards</x:v>
+        <x:v>Android S2</x:v>
       </x:c>
       <x:c r="V135" s="14" t="str">
-        <x:v>feature/android-rewards</x:v>
-      </x:c>
-      <x:c r="W135" s="14" t="str"/>
-      <x:c r="X135" s="14" t="str"/>
-      <x:c r="Y135" s="14" t="str"/>
-      <x:c r="Z135" s="14" t="str"/>
+        <x:v>test/android-account-checkout</x:v>
+      </x:c>
+      <x:c r="W135" s="14"/>
+      <x:c r="X135" s="14"/>
+      <x:c r="Y135" s="14"/>
+      <x:c r="Z135" s="14"/>
     </x:row>
     <x:row r="136" ht="84" customHeight="1">
       <x:c r="A136" s="14" t="str">
-        <x:v>IMP-AND-0302</x:v>
+        <x:v>IMP-AND-0301</x:v>
       </x:c>
       <x:c r="B136" s="14" t="str">
         <x:v>S3 Android Loyalty</x:v>
@@ -10722,7 +10726,7 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D136" s="14" t="str">
-        <x:v>Promociones</x:v>
+        <x:v>Loyalty</x:v>
       </x:c>
       <x:c r="E136" s="14" t="str">
         <x:v>ANDROID-1</x:v>
@@ -10731,7 +10735,7 @@
         <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G136" s="14" t="str">
-        <x:v>promotions</x:v>
+        <x:v>rewards</x:v>
       </x:c>
       <x:c r="H136" s="14" t="str">
         <x:v>FEATURE</x:v>
@@ -10752,19 +10756,19 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N136" s="14" t="str">
-        <x:v>Promotions</x:v>
+        <x:v>Rewards</x:v>
       </x:c>
       <x:c r="O136" s="14" t="str">
-        <x:v>Implementar Promotions</x:v>
+        <x:v>Implementar Rewards</x:v>
       </x:c>
       <x:c r="P136" s="14" t="str">
-        <x:v>Eligibility/vigencia/stacking reason; states.</x:v>
+        <x:v>Ledger/balance Domain cross-app; offline/error/empty.</x:v>
       </x:c>
       <x:c r="Q136" s="14" t="str">
-        <x:v>Incompatible no combinable; reasons correct.</x:v>
+        <x:v>CANCELLED/NO_SHOW no elegibles; ledger read-only.</x:v>
       </x:c>
       <x:c r="R136" s="14" t="str">
-        <x:v>Promotion contract reviewed.</x:v>
+        <x:v>Reward contract reviewed.</x:v>
       </x:c>
       <x:c r="S136" s="14" t="str">
         <x:v>Mapper + UI.</x:v>
@@ -10773,19 +10777,19 @@
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U136" s="14" t="str">
-        <x:v>promotions</x:v>
+        <x:v>rewards</x:v>
       </x:c>
       <x:c r="V136" s="14" t="str">
-        <x:v>feature/android-promotions</x:v>
-      </x:c>
-      <x:c r="W136" s="14" t="str"/>
-      <x:c r="X136" s="14" t="str"/>
-      <x:c r="Y136" s="14" t="str"/>
-      <x:c r="Z136" s="14" t="str"/>
+        <x:v>feature/android-rewards</x:v>
+      </x:c>
+      <x:c r="W136" s="14"/>
+      <x:c r="X136" s="14"/>
+      <x:c r="Y136" s="14"/>
+      <x:c r="Z136" s="14"/>
     </x:row>
     <x:row r="137" ht="84" customHeight="1">
       <x:c r="A137" s="14" t="str">
-        <x:v>IMP-AND-0303</x:v>
+        <x:v>IMP-AND-0302</x:v>
       </x:c>
       <x:c r="B137" s="14" t="str">
         <x:v>S3 Android Loyalty</x:v>
@@ -10794,7 +10798,7 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D137" s="14" t="str">
-        <x:v>Perfil</x:v>
+        <x:v>Promociones</x:v>
       </x:c>
       <x:c r="E137" s="14" t="str">
         <x:v>ANDROID-1</x:v>
@@ -10803,7 +10807,7 @@
         <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G137" s="14" t="str">
-        <x:v>profile</x:v>
+        <x:v>promotions</x:v>
       </x:c>
       <x:c r="H137" s="14" t="str">
         <x:v>FEATURE</x:v>
@@ -10815,7 +10819,7 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K137" s="14" t="str">
-        <x:v>IMP-AND-0201</x:v>
+        <x:v>IMP-AND-0009</x:v>
       </x:c>
       <x:c r="L137" s="14" t="str">
         <x:v>Android 03 Loyalty, promociones y perfil</x:v>
@@ -10824,40 +10828,40 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N137" s="14" t="str">
-        <x:v>Profile</x:v>
+        <x:v>Promotions</x:v>
       </x:c>
       <x:c r="O137" s="14" t="str">
-        <x:v>Implementar perfil final</x:v>
+        <x:v>Implementar Promotions</x:v>
       </x:c>
       <x:c r="P137" s="14" t="str">
-        <x:v>Figma layout/edit/states; reuse Account/Profile Domain.</x:v>
+        <x:v>Eligibility/vigencia/stacking reason; states.</x:v>
       </x:c>
       <x:c r="Q137" s="14" t="str">
-        <x:v>No duplicated model; PII safe; save states correct.</x:v>
+        <x:v>Incompatible no combinable; reasons correct.</x:v>
       </x:c>
       <x:c r="R137" s="14" t="str">
-        <x:v>Profile contract ready.</x:v>
+        <x:v>Promotion contract reviewed.</x:v>
       </x:c>
       <x:c r="S137" s="14" t="str">
-        <x:v>UI tests.</x:v>
+        <x:v>Mapper + UI.</x:v>
       </x:c>
       <x:c r="T137" s="14" t="str">
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U137" s="14" t="str">
-        <x:v>profile</x:v>
+        <x:v>promotions</x:v>
       </x:c>
       <x:c r="V137" s="14" t="str">
-        <x:v>feature/android-profile</x:v>
-      </x:c>
-      <x:c r="W137" s="14" t="str"/>
-      <x:c r="X137" s="14" t="str"/>
-      <x:c r="Y137" s="14" t="str"/>
-      <x:c r="Z137" s="14" t="str"/>
+        <x:v>feature/android-promotions</x:v>
+      </x:c>
+      <x:c r="W137" s="14"/>
+      <x:c r="X137" s="14"/>
+      <x:c r="Y137" s="14"/>
+      <x:c r="Z137" s="14"/>
     </x:row>
     <x:row r="138" ht="84" customHeight="1">
       <x:c r="A138" s="14" t="str">
-        <x:v>IMP-AND-0304</x:v>
+        <x:v>IMP-AND-0303</x:v>
       </x:c>
       <x:c r="B138" s="14" t="str">
         <x:v>S3 Android Loyalty</x:v>
@@ -10866,7 +10870,7 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D138" s="14" t="str">
-        <x:v>QA</x:v>
+        <x:v>Perfil</x:v>
       </x:c>
       <x:c r="E138" s="14" t="str">
         <x:v>ANDROID-1</x:v>
@@ -10875,19 +10879,19 @@
         <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G138" s="14" t="str">
-        <x:v>loyalty-profile</x:v>
+        <x:v>profile</x:v>
       </x:c>
       <x:c r="H138" s="14" t="str">
-        <x:v>QA</x:v>
+        <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I138" s="14" t="str">
-        <x:v>CRÍTICA</x:v>
+        <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J138" s="14" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K138" s="14" t="str">
-        <x:v>IMP-AND-0301, IMP-AND-0302, IMP-AND-0303</x:v>
+        <x:v>IMP-AND-0201</x:v>
       </x:c>
       <x:c r="L138" s="14" t="str">
         <x:v>Android 03 Loyalty, promociones y perfil</x:v>
@@ -10896,49 +10900,49 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N138" s="14" t="str">
-        <x:v>Rewards/Promos/Profile</x:v>
+        <x:v>Profile</x:v>
       </x:c>
       <x:c r="O138" s="14" t="str">
-        <x:v>QA Loyalty/Profile</x:v>
+        <x:v>Implementar perfil final</x:v>
       </x:c>
       <x:c r="P138" s="14" t="str">
-        <x:v>Rewards/promotions/profile/offline/error/empty/navigation.</x:v>
+        <x:v>Figma layout/edit/states; reuse Account/Profile Domain.</x:v>
       </x:c>
       <x:c r="Q138" s="14" t="str">
-        <x:v>Cross-app semantics PASS; Figma parity; no DTO UI.</x:v>
+        <x:v>No duplicated model; PII safe; save states correct.</x:v>
       </x:c>
       <x:c r="R138" s="14" t="str">
-        <x:v>S3 done.</x:v>
+        <x:v>Profile contract ready.</x:v>
       </x:c>
       <x:c r="S138" s="14" t="str">
-        <x:v>Android Global DoD.</x:v>
+        <x:v>UI tests.</x:v>
       </x:c>
       <x:c r="T138" s="14" t="str">
-        <x:v>build/tests/manual</x:v>
+        <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U138" s="14" t="str">
-        <x:v>Android S3</x:v>
+        <x:v>profile</x:v>
       </x:c>
       <x:c r="V138" s="14" t="str">
-        <x:v>test/android-loyalty</x:v>
-      </x:c>
-      <x:c r="W138" s="14" t="str"/>
-      <x:c r="X138" s="14" t="str"/>
-      <x:c r="Y138" s="14" t="str"/>
-      <x:c r="Z138" s="14" t="str"/>
+        <x:v>feature/android-profile</x:v>
+      </x:c>
+      <x:c r="W138" s="14"/>
+      <x:c r="X138" s="14"/>
+      <x:c r="Y138" s="14"/>
+      <x:c r="Z138" s="14"/>
     </x:row>
     <x:row r="139" ht="84" customHeight="1">
       <x:c r="A139" s="14" t="str">
-        <x:v>IMP-AND-0401</x:v>
+        <x:v>IMP-AND-0304</x:v>
       </x:c>
       <x:c r="B139" s="14" t="str">
-        <x:v>S4 Android Release</x:v>
+        <x:v>S3 Android Loyalty</x:v>
       </x:c>
       <x:c r="C139" s="14" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D139" s="14" t="str">
-        <x:v>Estados</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="E139" s="14" t="str">
         <x:v>ANDROID-1</x:v>
@@ -10947,10 +10951,10 @@
         <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G139" s="14" t="str">
-        <x:v>ui-states</x:v>
+        <x:v>loyalty-profile</x:v>
       </x:c>
       <x:c r="H139" s="14" t="str">
-        <x:v>SHARED</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="I139" s="14" t="str">
         <x:v>CRÍTICA</x:v>
@@ -10959,49 +10963,49 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K139" s="14" t="str">
-        <x:v>IMP-AND-0009</x:v>
+        <x:v>IMP-AND-0301, IMP-AND-0302, IMP-AND-0303</x:v>
       </x:c>
       <x:c r="L139" s="14" t="str">
-        <x:v>Android 04 Loading, error y offline</x:v>
+        <x:v>Android 03 Loyalty, promociones y perfil</x:v>
       </x:c>
       <x:c r="M139" s="14" t="str">
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N139" s="14" t="str">
-        <x:v>Universal States</x:v>
+        <x:v>Rewards/Promos/Profile</x:v>
       </x:c>
       <x:c r="O139" s="14" t="str">
-        <x:v>Implementar Loading/Error/Empty/Offline shared</x:v>
+        <x:v>QA Loyalty/Profile</x:v>
       </x:c>
       <x:c r="P139" s="14" t="str">
-        <x:v>Reusable state UI; retry callback; accessible; no business logic.</x:v>
+        <x:v>Rewards/promotions/profile/offline/error/empty/navigation.</x:v>
       </x:c>
       <x:c r="Q139" s="14" t="str">
-        <x:v>Features reutilizan states; offline explicit; retry actionable.</x:v>
+        <x:v>Cross-app semantics PASS; Figma parity; no DTO UI.</x:v>
       </x:c>
       <x:c r="R139" s="14" t="str">
-        <x:v>Figma states reviewed.</x:v>
+        <x:v>S3 done.</x:v>
       </x:c>
       <x:c r="S139" s="14" t="str">
-        <x:v>UI tests.</x:v>
+        <x:v>Android Global DoD.</x:v>
       </x:c>
       <x:c r="T139" s="14" t="str">
-        <x:v>ui</x:v>
+        <x:v>build/tests/manual</x:v>
       </x:c>
       <x:c r="U139" s="14" t="str">
-        <x:v>shared state UI</x:v>
+        <x:v>Android S3</x:v>
       </x:c>
       <x:c r="V139" s="14" t="str">
-        <x:v>feature/android-universal-states</x:v>
-      </x:c>
-      <x:c r="W139" s="14" t="str"/>
-      <x:c r="X139" s="14" t="str"/>
-      <x:c r="Y139" s="14" t="str"/>
-      <x:c r="Z139" s="14" t="str"/>
+        <x:v>test/android-loyalty</x:v>
+      </x:c>
+      <x:c r="W139" s="14"/>
+      <x:c r="X139" s="14"/>
+      <x:c r="Y139" s="14"/>
+      <x:c r="Z139" s="14"/>
     </x:row>
     <x:row r="140" ht="84" customHeight="1">
       <x:c r="A140" s="14" t="str">
-        <x:v>IMP-AND-0402</x:v>
+        <x:v>IMP-AND-0401</x:v>
       </x:c>
       <x:c r="B140" s="14" t="str">
         <x:v>S4 Android Release</x:v>
@@ -11016,13 +11020,13 @@
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F140" s="14" t="str">
-        <x:v>WEB-3</x:v>
+        <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G140" s="14" t="str">
-        <x:v>offline</x:v>
+        <x:v>ui-states</x:v>
       </x:c>
       <x:c r="H140" s="14" t="str">
-        <x:v>FEATURE</x:v>
+        <x:v>SHARED</x:v>
       </x:c>
       <x:c r="I140" s="14" t="str">
         <x:v>CRÍTICA</x:v>
@@ -11031,7 +11035,7 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K140" s="14" t="str">
-        <x:v>IMP-AND-0401, IMP-AND-0106, IMP-AND-0204, IMP-AND-0304</x:v>
+        <x:v>IMP-AND-0009</x:v>
       </x:c>
       <x:c r="L140" s="14" t="str">
         <x:v>Android 04 Loading, error y offline</x:v>
@@ -11040,40 +11044,40 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N140" s="14" t="str">
-        <x:v>All</x:v>
+        <x:v>Universal States</x:v>
       </x:c>
       <x:c r="O140" s="14" t="str">
-        <x:v>Integrar states universales</x:v>
+        <x:v>Implementar Loading/Error/Empty/Offline shared</x:v>
       </x:c>
       <x:c r="P140" s="14" t="str">
-        <x:v>Reemplazar estados ad-hoc; retry; stale indication donde aplica.</x:v>
+        <x:v>Reusable state UI; retry callback; accessible; no business logic.</x:v>
       </x:c>
       <x:c r="Q140" s="14" t="str">
-        <x:v>0 remote screen sin Loading/Error; Offline según Figma; no false success.</x:v>
+        <x:v>Features reutilizan states; offline explicit; retry actionable.</x:v>
       </x:c>
       <x:c r="R140" s="14" t="str">
-        <x:v>Feature screens done.</x:v>
+        <x:v>Figma states reviewed.</x:v>
       </x:c>
       <x:c r="S140" s="14" t="str">
-        <x:v>Regression states.</x:v>
+        <x:v>UI tests.</x:v>
       </x:c>
       <x:c r="T140" s="14" t="str">
-        <x:v>ui/manual</x:v>
+        <x:v>ui</x:v>
       </x:c>
       <x:c r="U140" s="14" t="str">
-        <x:v>all Android</x:v>
+        <x:v>shared state UI</x:v>
       </x:c>
       <x:c r="V140" s="14" t="str">
-        <x:v>feature/android-state-integration</x:v>
-      </x:c>
-      <x:c r="W140" s="14" t="str"/>
-      <x:c r="X140" s="14" t="str"/>
-      <x:c r="Y140" s="14" t="str"/>
-      <x:c r="Z140" s="14" t="str"/>
+        <x:v>feature/android-universal-states</x:v>
+      </x:c>
+      <x:c r="W140" s="14"/>
+      <x:c r="X140" s="14"/>
+      <x:c r="Y140" s="14"/>
+      <x:c r="Z140" s="14"/>
     </x:row>
     <x:row r="141" ht="84" customHeight="1">
       <x:c r="A141" s="14" t="str">
-        <x:v>IMP-AND-0403</x:v>
+        <x:v>IMP-AND-0402</x:v>
       </x:c>
       <x:c r="B141" s="14" t="str">
         <x:v>S4 Android Release</x:v>
@@ -11082,19 +11086,19 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D141" s="14" t="str">
-        <x:v>QA</x:v>
+        <x:v>Estados</x:v>
       </x:c>
       <x:c r="E141" s="14" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F141" s="14" t="str">
-        <x:v>WEB-2</x:v>
+        <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G141" s="14" t="str">
-        <x:v>accessibility</x:v>
+        <x:v>offline</x:v>
       </x:c>
       <x:c r="H141" s="14" t="str">
-        <x:v>QA</x:v>
+        <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I141" s="14" t="str">
         <x:v>CRÍTICA</x:v>
@@ -11103,10 +11107,10 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K141" s="14" t="str">
-        <x:v>IMP-AND-0402</x:v>
+        <x:v>IMP-AND-0401, IMP-AND-0106, IMP-AND-0204, IMP-AND-0304</x:v>
       </x:c>
       <x:c r="L141" s="14" t="str">
-        <x:v>Android final regression</x:v>
+        <x:v>Android 04 Loading, error y offline</x:v>
       </x:c>
       <x:c r="M141" s="14" t="str">
         <x:v>238:132</x:v>
@@ -11115,37 +11119,37 @@
         <x:v>All</x:v>
       </x:c>
       <x:c r="O141" s="14" t="str">
-        <x:v>Auditoría accesibilidad Android</x:v>
+        <x:v>Integrar states universales</x:v>
       </x:c>
       <x:c r="P141" s="14" t="str">
-        <x:v>TalkBack/labels/targets/contrast/focus/auth/errors.</x:v>
+        <x:v>Reemplazar estados ad-hoc; retry; stale indication donde aplica.</x:v>
       </x:c>
       <x:c r="Q141" s="14" t="str">
-        <x:v>0 critical/high accessibility defects; primary journeys operable.</x:v>
+        <x:v>0 remote screen sin Loading/Error; Offline según Figma; no false success.</x:v>
       </x:c>
       <x:c r="R141" s="14" t="str">
-        <x:v>Features done.</x:v>
+        <x:v>Feature screens done.</x:v>
       </x:c>
       <x:c r="S141" s="14" t="str">
-        <x:v>A11y PASS.</x:v>
+        <x:v>Regression states.</x:v>
       </x:c>
       <x:c r="T141" s="14" t="str">
-        <x:v>manual/tooling</x:v>
+        <x:v>ui/manual</x:v>
       </x:c>
       <x:c r="U141" s="14" t="str">
-        <x:v>whole Android</x:v>
+        <x:v>all Android</x:v>
       </x:c>
       <x:c r="V141" s="14" t="str">
-        <x:v>test/android-a11y</x:v>
-      </x:c>
-      <x:c r="W141" s="14" t="str"/>
-      <x:c r="X141" s="14" t="str"/>
-      <x:c r="Y141" s="14" t="str"/>
-      <x:c r="Z141" s="14" t="str"/>
+        <x:v>feature/android-state-integration</x:v>
+      </x:c>
+      <x:c r="W141" s="14"/>
+      <x:c r="X141" s="14"/>
+      <x:c r="Y141" s="14"/>
+      <x:c r="Z141" s="14"/>
     </x:row>
     <x:row r="142" ht="84" customHeight="1">
       <x:c r="A142" s="14" t="str">
-        <x:v>IMP-AND-0404</x:v>
+        <x:v>IMP-AND-0403</x:v>
       </x:c>
       <x:c r="B142" s="14" t="str">
         <x:v>S4 Android Release</x:v>
@@ -11160,10 +11164,10 @@
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F142" s="14" t="str">
-        <x:v>WEB-3</x:v>
+        <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G142" s="14" t="str">
-        <x:v>release</x:v>
+        <x:v>accessibility</x:v>
       </x:c>
       <x:c r="H142" s="14" t="str">
         <x:v>QA</x:v>
@@ -11175,7 +11179,7 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K142" s="14" t="str">
-        <x:v>IMP-AND-0403</x:v>
+        <x:v>IMP-AND-0402</x:v>
       </x:c>
       <x:c r="L142" s="14" t="str">
         <x:v>Android final regression</x:v>
@@ -11187,33 +11191,105 @@
         <x:v>All</x:v>
       </x:c>
       <x:c r="O142" s="14" t="str">
-        <x:v>Regresión final Android</x:v>
+        <x:v>Auditoría accesibilidad Android</x:v>
       </x:c>
       <x:c r="P142" s="14" t="str">
-        <x:v>Build/tests/navigation/states/contracts/no DTO UI/no secrets.</x:v>
+        <x:v>TalkBack/labels/targets/contrast/focus/auth/errors.</x:v>
       </x:c>
       <x:c r="Q142" s="14" t="str">
-        <x:v>0 critical/high; all checks PASS; release candidate.</x:v>
+        <x:v>0 critical/high accessibility defects; primary journeys operable.</x:v>
       </x:c>
       <x:c r="R142" s="14" t="str">
-        <x:v>All Android tasks done.</x:v>
+        <x:v>Features done.</x:v>
       </x:c>
       <x:c r="S142" s="14" t="str">
-        <x:v>Release DoD PASS.</x:v>
+        <x:v>A11y PASS.</x:v>
       </x:c>
       <x:c r="T142" s="14" t="str">
-        <x:v>build/tests/manual</x:v>
+        <x:v>manual/tooling</x:v>
       </x:c>
       <x:c r="U142" s="14" t="str">
         <x:v>whole Android</x:v>
       </x:c>
       <x:c r="V142" s="14" t="str">
+        <x:v>test/android-a11y</x:v>
+      </x:c>
+      <x:c r="W142" s="14"/>
+      <x:c r="X142" s="14"/>
+      <x:c r="Y142" s="14"/>
+      <x:c r="Z142" s="14"/>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" t="str">
+        <x:v>IMP-AND-0404</x:v>
+      </x:c>
+      <x:c r="B143" t="str">
+        <x:v>S4 Android Release</x:v>
+      </x:c>
+      <x:c r="C143" t="str">
+        <x:v>ANDROID</x:v>
+      </x:c>
+      <x:c r="D143" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="E143" t="str">
+        <x:v>ANDROID-1</x:v>
+      </x:c>
+      <x:c r="F143" t="str">
+        <x:v>WEB-3</x:v>
+      </x:c>
+      <x:c r="G143" t="str">
+        <x:v>release</x:v>
+      </x:c>
+      <x:c r="H143" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="I143" t="str">
+        <x:v>CRÍTICA</x:v>
+      </x:c>
+      <x:c r="J143" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="K143" t="str">
+        <x:v>IMP-AND-0403</x:v>
+      </x:c>
+      <x:c r="L143" t="str">
+        <x:v>Android final regression</x:v>
+      </x:c>
+      <x:c r="M143" t="str">
+        <x:v>238:132</x:v>
+      </x:c>
+      <x:c r="N143" t="str">
+        <x:v>All</x:v>
+      </x:c>
+      <x:c r="O143" t="str">
+        <x:v>Regresión final Android</x:v>
+      </x:c>
+      <x:c r="P143" t="str">
+        <x:v>Build/tests/navigation/states/contracts/no DTO UI/no secrets.</x:v>
+      </x:c>
+      <x:c r="Q143" t="str">
+        <x:v>0 critical/high; all checks PASS; release candidate.</x:v>
+      </x:c>
+      <x:c r="R143" t="str">
+        <x:v>All Android tasks done.</x:v>
+      </x:c>
+      <x:c r="S143" t="str">
+        <x:v>Release DoD PASS.</x:v>
+      </x:c>
+      <x:c r="T143" t="str">
+        <x:v>build/tests/manual</x:v>
+      </x:c>
+      <x:c r="U143" t="str">
+        <x:v>whole Android</x:v>
+      </x:c>
+      <x:c r="V143" t="str">
         <x:v>release/android-rc</x:v>
       </x:c>
-      <x:c r="W142" s="14" t="str"/>
-      <x:c r="X142" s="14" t="str"/>
-      <x:c r="Y142" s="14" t="str"/>
-      <x:c r="Z142" s="14" t="str"/>
+      <x:c r="W143"/>
+      <x:c r="X143"/>
+      <x:c r="Y143"/>
+      <x:c r="Z143"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="J2:J142">
@@ -11266,7 +11342,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cf6c74838f64b35"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc106a70828af4c62"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(android): ready guest navigation shell V3
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R64f8d28645274f9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R5df768171ff14a6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R3a5f013e26274fd5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="Rb1d35938644d495f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R58a53252fb974a4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Raf6741aa85bd4906"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="Re99e16acd6334b73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R598a48e7a9aa4d8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R343cd6e001014e45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="Ra185a3f58dfd44a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Rad20d11f86504b61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Rf7dee78c0ce64235"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5b934b47dba94480"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8326edf4131e4e04"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -804,7 +804,7 @@
       </x:c>
       <x:c r="B6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_PROGRESO")</x:f>
@@ -927,7 +927,7 @@
       </x:c>
       <x:c r="C14" s="12" t="n">
         <x:f>COUNTIFS('01_Backlog'!E2:E142,A14,'01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf26dc0040c9843b4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40d7d4f105064649"/>
 </x:worksheet>
 </file>
 
@@ -9901,7 +9901,7 @@
       </x:c>
       <x:c r="Z124" s="14" t="str"/>
     </x:row>
-    <x:row r="125" ht="84" customHeight="1">
+    <x:row r="125" ht="90" customHeight="1">
       <x:c r="A125" s="14" t="str">
         <x:v>IMP-AND-0100</x:v>
       </x:c>
@@ -9918,7 +9918,7 @@
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F125" s="14" t="str">
-        <x:v>PENDIENTE DE DESIGNACIÓN</x:v>
+        <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G125" s="14" t="str">
         <x:v>navigation</x:v>
@@ -9930,7 +9930,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J125" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>READY</x:v>
       </x:c>
       <x:c r="K125" s="14" t="str">
         <x:v>IMP-AND-0009</x:v>
@@ -9954,7 +9954,7 @@
         <x:v>Features V3 consumen un shell único; no footbars privadas; item seleccionado y destinos no implementados son accesibles y semánticamente honestos; IMP-AND-0102 no se modifica; back stack PASS.</x:v>
       </x:c>
       <x:c r="R125" s="14" t="str">
-        <x:v>IMP-AND-0009 COMPLETADA; owner y reviewer designados; 238:132 y pantallas V3 verificadas; política de destinos no implementados, selección y accesibilidad aprobada; Home V2 no migra en esta tarea; rutas Guest y back stack definidos.</x:v>
+        <x:v>IMP-AND-0009 COMPLETADA; owner ANDROID-1 y reviewer WEB-3 asignados; 238:132 y Chat 238:192, Servicios 239:132, Valet 239:197 y Cuenta 240:132 verificados; rutas objetivo /services, /chat, /valet y /account definidas; políticas de destinos disabled, selección usePathname(), accesibilidad y back stack aprobadas; Home V2 no migra; creación de src/modules/navigation y estrategia de montaje aislado autorizadas mediante DEC-A-004.</x:v>
       </x:c>
       <x:c r="S125" s="14" t="str">
         <x:v>Shell Guest V3 compartido Servicios/Chat/Valet/Cuenta; punto único sin footbars privadas; tab activo; destinos accesibles y honestos; Expo Router/back stack/a11y/tab tests PASS; Figma 238:132 PASS; IMP-AND-0102 intacta; lint, typecheck, test y check PASS.</x:v>
@@ -9969,7 +9969,7 @@
         <x:v>feature/android-guest-navigation-shell</x:v>
       </x:c>
       <x:c r="W125" s="14" t="str">
-        <x:v>Change Control aprobado. IMP-AND-0100 permanece PENDIENTE, no READY: reviewer por designar y DoR operativo pendiente.</x:v>
+        <x:v>DoR PASS mediante Change Control 2026-09-10: IMP-AND-0009 COMPLETADA; owner ANDROID-1; reviewer WEB-3; Figma V3 y cuatro frames; rutas objetivo; destinos disabled; usePathname(); accesibilidad; back stack; Home V2 intacta; src/modules/navigation y montaje aislado autorizados. IMP-AND-0100 pasa a READY. DoD no evaluado ni cumplido.</x:v>
       </x:c>
       <x:c r="X125" s="14"/>
       <x:c r="Y125" s="14"/>
@@ -11342,7 +11342,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc106a70828af4c62"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf01ff4e133442f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(android): implement guest navigation shell V3 (IMP-AND-0100)
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="Re99e16acd6334b73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R598a48e7a9aa4d8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R343cd6e001014e45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="Ra185a3f58dfd44a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Rad20d11f86504b61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Rf7dee78c0ce64235"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R8008f4a3ab6041fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R14214a68228d4758"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Rab1efb3d00fd487c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R93539ee067884c3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Rbc8a997d18774836"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R2e8ee89978e34433"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8326edf4131e4e04"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Recab93d9e3244c4d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -804,7 +804,7 @@
       </x:c>
       <x:c r="B6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_PROGRESO")</x:f>
@@ -812,7 +812,7 @@
       </x:c>
       <x:c r="D6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_QA")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"BLOQUEADA")</x:f>
@@ -927,7 +927,7 @@
       </x:c>
       <x:c r="C14" s="12" t="n">
         <x:f>COUNTIFS('01_Backlog'!E2:E142,A14,'01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40d7d4f105064649"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f078465705b41b4"/>
 </x:worksheet>
 </file>
 
@@ -9901,7 +9901,7 @@
       </x:c>
       <x:c r="Z124" s="14" t="str"/>
     </x:row>
-    <x:row r="125" ht="90" customHeight="1">
+    <x:row r="125" ht="180" customHeight="1">
       <x:c r="A125" s="14" t="str">
         <x:v>IMP-AND-0100</x:v>
       </x:c>
@@ -9930,7 +9930,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J125" s="14" t="str">
-        <x:v>READY</x:v>
+        <x:v>EN_QA</x:v>
       </x:c>
       <x:c r="K125" s="14" t="str">
         <x:v>IMP-AND-0009</x:v>
@@ -9969,7 +9969,7 @@
         <x:v>feature/android-guest-navigation-shell</x:v>
       </x:c>
       <x:c r="W125" s="14" t="str">
-        <x:v>DoR PASS mediante Change Control 2026-09-10: IMP-AND-0009 COMPLETADA; owner ANDROID-1; reviewer WEB-3; Figma V3 y cuatro frames; rutas objetivo; destinos disabled; usePathname(); accesibilidad; back stack; Home V2 intacta; src/modules/navigation y montaje aislado autorizados. IMP-AND-0100 pasa a READY. DoD no evaluado ni cumplido.</x:v>
+        <x:v>Implementación técnica PASS 2026-09-10: módulo navigation con configuración declarativa, shell reutilizable, resolver usePathname(), disabled sin handler, accesibilidad tab/tablist y replace preparado; 7 suites/21 tests PASS; lint, typecheck y npm run check PASS; Expo Doctor 21/21; export Android PASS. IMP-AND-0102 y su Home V2 no cambiaron; IMP-AND-0103 no inició. Pendiente QA visual/revisión WEB-3 contra 238:132 para declarar DoD PASS y COMPLETADA.</x:v>
       </x:c>
       <x:c r="X125" s="14"/>
       <x:c r="Y125" s="14"/>
@@ -11342,7 +11342,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf01ff4e133442f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1675d017d1244307"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(android): close IMP-AND-0100 after QA
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R8008f4a3ab6041fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R14214a68228d4758"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Rab1efb3d00fd487c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R93539ee067884c3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Rbc8a997d18774836"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R2e8ee89978e34433"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R187bbe9775bf408b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R5c079b7d92ea4d8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R21a35027e5ab4591"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="Rb8f7c850e73b4b33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R3677167bb5a344e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Ra466ba0cca934702"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Recab93d9e3244c4d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R21c3dce3c0f94ddc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -812,7 +812,7 @@
       </x:c>
       <x:c r="D6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_QA")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"BLOQUEADA")</x:f>
@@ -820,7 +820,7 @@
       </x:c>
       <x:c r="F6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -888,7 +888,7 @@
       </x:c>
       <x:c r="G11" t="n">
         <x:f>COUNTIFS('01_Backlog'!C2:C142,E11,'01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f078465705b41b4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65ce83d56fcd4ab3"/>
 </x:worksheet>
 </file>
 
@@ -9930,7 +9930,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J125" s="14" t="str">
-        <x:v>EN_QA</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K125" s="14" t="str">
         <x:v>IMP-AND-0009</x:v>
@@ -9969,7 +9969,7 @@
         <x:v>feature/android-guest-navigation-shell</x:v>
       </x:c>
       <x:c r="W125" s="14" t="str">
-        <x:v>Implementación técnica PASS 2026-09-10: módulo navigation con configuración declarativa, shell reutilizable, resolver usePathname(), disabled sin handler, accesibilidad tab/tablist y replace preparado; 7 suites/21 tests PASS; lint, typecheck y npm run check PASS; Expo Doctor 21/21; export Android PASS. IMP-AND-0102 y su Home V2 no cambiaron; IMP-AND-0103 no inició. Pendiente QA visual/revisión WEB-3 contra 238:132 para declarar DoD PASS y COMPLETADA.</x:v>
+        <x:v>Cierre 2026-09-10: revisión independiente WEB-3 PASS; revisión visual directa contra Figma V3 PASS (238:132; Chat 238:192, Servicios 239:132, Valet 239:197, Cuenta 240:132). Desviación conocida y aceptada: algunos frames V3 de Chat/Valet muestran incorrectamente Servicios como activo. Android conserva la regla aprobada con usePathname(): /services -&gt; Servicios; /chat -&gt; Chat; /valet -&gt; Valet; /account -&gt; Cuenta. lint PASS; typecheck PASS; test PASS — 7 suites / 21 tests; npm run check PASS — Expo Doctor 21/21 + export Android; git diff --check PASS. IMP-AND-0102 intacta; IMP-AND-0103 no iniciada.</x:v>
       </x:c>
       <x:c r="X125" s="14"/>
       <x:c r="Y125" s="14"/>
@@ -11342,7 +11342,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1675d017d1244307"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5720a2748204159"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(android): approve services mock contract (IMP-AND-0103)
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R8008f4a3ab6041fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R14214a68228d4758"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Rab1efb3d00fd487c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R93539ee067884c3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Rbc8a997d18774836"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R2e8ee89978e34433"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R24b1de2e257d4440"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R6bfd1324111d494f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Rdb64a3d1b7f54970"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R641152c97eb14f46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Rd2fc1e3be9cc40c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Rd7821257e98145a5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Recab93d9e3244c4d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6ff6a59949ab400e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -804,7 +804,7 @@
       </x:c>
       <x:c r="B6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_PROGRESO")</x:f>
@@ -927,7 +927,7 @@
       </x:c>
       <x:c r="C14" s="12" t="n">
         <x:f>COUNTIFS('01_Backlog'!E2:E142,A14,'01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f078465705b41b4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9f5b1486ddb49f9"/>
 </x:worksheet>
 </file>
 
@@ -10166,7 +10166,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J128" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>READY</x:v>
       </x:c>
       <x:c r="K128" s="14" t="str">
         <x:v>IMP-AND-0100, IMP-AND-0102</x:v>
@@ -10205,7 +10205,7 @@
         <x:v>feature/android-services</x:v>
       </x:c>
       <x:c r="W128" s="14" t="str">
-        <x:v>Change Control aprobó DEC-G-013 y el DoR frontend-first. Contrato mock sigue propuesta: Figma 239:132 confirmado; faltan aprobar contrato mock y diseños Services loading/submitting/success/error/offline, y completar IMP-AND-0100. IMP-AND-0103 permanece PENDIENTE.</x:v>
+        <x:v>DoR PASS 2026-09-10: DEC-G-013 APPROVED; contrato frontend data/mock APPROVED en Android doc 16; Figma base 239:132 y sección de estados 1818:410 (Base 1821:410; Selected 1818:411; Loading 1819:410; Submitting 1820:410; Success 1820:13372; Error 1820:13290; Offline 1820:13331). Fixture catálogo/contexto/mutation exactos; priceText solo presentación; Mapper/Domain/UI, TanStack Query/RemoteState y NetworkError definidos. Matriz DoR 15/15 PASS; sin gate adicional pendiente. DoD no iniciado: sin código, tests, feature branch ni cambios a IMP-AND-0100/0102.</x:v>
       </x:c>
       <x:c r="X128" s="14"/>
       <x:c r="Y128" s="14"/>
@@ -11342,7 +11342,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1675d017d1244307"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1db797273d14a10"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(android): implement services flow (IMP-AND-0103)
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R24b1de2e257d4440"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R6bfd1324111d494f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Rdb64a3d1b7f54970"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R641152c97eb14f46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Rd2fc1e3be9cc40c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Rd7821257e98145a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="Rb18b1d3e474b409a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="Rc27383600f8d482d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R205fb67c07e54c9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R174f0bcd7d834c1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Re7607aac63db443b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Re7252a74c7a54854"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6ff6a59949ab400e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4f26b5e607404998"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -804,7 +804,7 @@
       </x:c>
       <x:c r="B6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_PROGRESO")</x:f>
@@ -820,7 +820,7 @@
       </x:c>
       <x:c r="F6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -888,7 +888,7 @@
       </x:c>
       <x:c r="G11" t="n">
         <x:f>COUNTIFS('01_Backlog'!C2:C142,E11,'01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -927,7 +927,7 @@
       </x:c>
       <x:c r="C14" s="12" t="n">
         <x:f>COUNTIFS('01_Backlog'!E2:E142,A14,'01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9f5b1486ddb49f9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red9b26c41c974e05"/>
 </x:worksheet>
 </file>
 
@@ -10166,7 +10166,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J128" s="14" t="str">
-        <x:v>READY</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K128" s="14" t="str">
         <x:v>IMP-AND-0100, IMP-AND-0102</x:v>
@@ -10205,7 +10205,7 @@
         <x:v>feature/android-services</x:v>
       </x:c>
       <x:c r="W128" s="14" t="str">
-        <x:v>DoR PASS 2026-09-10: DEC-G-013 APPROVED; contrato frontend data/mock APPROVED en Android doc 16; Figma base 239:132 y sección de estados 1818:410 (Base 1821:410; Selected 1818:411; Loading 1819:410; Submitting 1820:410; Success 1820:13372; Error 1820:13290; Offline 1820:13331). Fixture catálogo/contexto/mutation exactos; priceText solo presentación; Mapper/Domain/UI, TanStack Query/RemoteState y NetworkError definidos. Matriz DoR 15/15 PASS; sin gate adicional pendiente. DoD no iniciado: sin código, tests, feature branch ni cambios a IMP-AND-0100/0102.</x:v>
+        <x:v>DoR/DoD PASS 2026-09-10: Figma visual PASS (Base, Selected, Loading, Submitting, Success, Error, Offline); navegación Guest V3 y accesibilidad del alcance PASS; DTO → Mapper → Domain → Query/Mutation → UI PASS; doble submit y Home → Services → Back PASS; regresiones IMP-AND-0100/0102 PASS; WEB-3 PASS. Defecto footbar Success corregido y revalidado. lint/typecheck/check PASS; test PASS 8 suites/30 tests; Expo Doctor 21/21; export Android PASS; git diff --check PASS.</x:v>
       </x:c>
       <x:c r="X128" s="14"/>
       <x:c r="Y128" s="14"/>
@@ -11342,7 +11342,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1db797273d14a10"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79089500d904443e"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(web): implement booking guarantee and payment contracts, mappers, service and mocks (IMP-WEB-0109)
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -4541,7 +4541,7 @@
       </c>
       <c r="J29" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>EN_QA</t>
         </is>
       </c>
       <c r="K29" s="14" t="inlineStr">
@@ -4600,8 +4600,16 @@
           <t>feature/booking-payment-contract</t>
         </is>
       </c>
-      <c r="W29" s="14" t="str"/>
-      <c r="X29" s="14" t="str"/>
+      <c r="W29" s="14" t="inlineStr">
+        <is>
+          <t>feature/web4-sprint-1; vitest 30 tests PASS; npm run check PASS</t>
+        </is>
+      </c>
+      <c r="X29" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="Y29" s="14" t="str"/>
       <c r="Z29" s="14" t="str"/>
     </row>

</xml_diff>

<commit_message>
feat(web): implement shared StatusBadge component and unit tests (IMP-WEB-S401)
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -7465,7 +7465,7 @@
       </c>
       <c r="J55" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>EN_QA</t>
         </is>
       </c>
       <c r="K55" s="14" t="inlineStr">
@@ -7524,8 +7524,16 @@
           <t>feature/shared-status-badge</t>
         </is>
       </c>
-      <c r="W55" s="14" t="str"/>
-      <c r="X55" s="14" t="str"/>
+      <c r="W55" s="14" t="inlineStr">
+        <is>
+          <t>feature/web4-sprint-4; StatusBadge component + 4 tests PASS; npm run check PASS</t>
+        </is>
+      </c>
+      <c r="X55" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="Y55" s="14" t="str"/>
       <c r="Z55" s="14" t="str"/>
     </row>

</xml_diff>

<commit_message>
feat(web): implement advanced Folio domain, mappers, service, mocks and FolioDetailCard (IMP-WEB-0401)
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -7585,7 +7585,7 @@
       </c>
       <c r="J56" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>EN_QA</t>
         </is>
       </c>
       <c r="K56" s="14" t="inlineStr">
@@ -7644,8 +7644,16 @@
           <t>feature/folio-detail</t>
         </is>
       </c>
-      <c r="W56" s="14" t="str"/>
-      <c r="X56" s="14" t="str"/>
+      <c r="W56" s="14" t="inlineStr">
+        <is>
+          <t>feature/web4-sprint-4; Folio module + FolioDetailCard + 10 tests PASS; npm run check PASS</t>
+        </is>
+      </c>
+      <c r="X56" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="Y56" s="14" t="str"/>
       <c r="Z56" s="14" t="str"/>
     </row>

</xml_diff>

<commit_message>
feat(web): implement Folio charge routing, split operations and FolioSplitModal (IMP-WEB-0402)
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -7705,7 +7705,7 @@
       </c>
       <c r="J57" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>EN_QA</t>
         </is>
       </c>
       <c r="K57" s="14" t="inlineStr">
@@ -7764,8 +7764,16 @@
           <t>feature/folio-routing</t>
         </is>
       </c>
-      <c r="W57" s="14" t="str"/>
-      <c r="X57" s="14" t="str"/>
+      <c r="W57" s="14" t="inlineStr">
+        <is>
+          <t>feature/web4-sprint-4; Charge routing + FolioSplitModal + 17 tests PASS; npm run check PASS</t>
+        </is>
+      </c>
+      <c r="X57" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="Y57" s="14" t="str"/>
       <c r="Z57" s="14" t="str"/>
     </row>

</xml_diff>

<commit_message>
feat: implement payment refunds and add rate plan and availability matrix management modules
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -8385,7 +8385,7 @@
       </c>
       <c r="J63" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>EN_QA</t>
         </is>
       </c>
       <c r="K63" s="14" t="inlineStr">
@@ -8497,7 +8497,7 @@
       </c>
       <c r="J64" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>EN_QA</t>
         </is>
       </c>
       <c r="K64" s="14" t="inlineStr">
@@ -9617,7 +9617,7 @@
       </c>
       <c r="J74" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>EN_QA</t>
         </is>
       </c>
       <c r="K74" s="14" t="inlineStr">
@@ -9729,7 +9729,7 @@
       </c>
       <c r="J75" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>EN_QA</t>
         </is>
       </c>
       <c r="K75" s="14" t="inlineStr">

</xml_diff>

<commit_message>
docs(android): approve frontend-first feature contracts
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="Rb18b1d3e474b409a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="Rc27383600f8d482d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R205fb67c07e54c9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R174f0bcd7d834c1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Re7607aac63db443b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Re7252a74c7a54854"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R87ac0065fba946ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R1f8cbfa1315a42bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R9bfc85a08fbb49f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R45589663c03a4dcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R33d7b1cdca3042bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R36f0646809bf42ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4f26b5e607404998"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6a5aac43e6864b51"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -804,7 +804,7 @@
       </x:c>
       <x:c r="B6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_PROGRESO")</x:f>
@@ -812,7 +812,7 @@
       </x:c>
       <x:c r="D6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_QA")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"BLOQUEADA")</x:f>
@@ -820,7 +820,7 @@
       </x:c>
       <x:c r="F6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -888,7 +888,7 @@
       </x:c>
       <x:c r="G11" t="n">
         <x:f>COUNTIFS('01_Backlog'!C2:C142,E11,'01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -927,7 +927,7 @@
       </x:c>
       <x:c r="C14" s="12" t="n">
         <x:f>COUNTIFS('01_Backlog'!E2:E142,A14,'01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red9b26c41c974e05"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f5ef29bc84f4377"/>
 </x:worksheet>
 </file>
 
@@ -9930,7 +9930,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J125" s="14" t="str">
-        <x:v>EN_QA</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K125" s="14" t="str">
         <x:v>IMP-AND-0009</x:v>
@@ -10240,7 +10240,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J129" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>READY</x:v>
       </x:c>
       <x:c r="K129" s="14" t="str">
         <x:v>IMP-AND-0102</x:v>
@@ -10264,7 +10264,7 @@
         <x:v>No direct HK/Maintenance recipient; no PII logs.</x:v>
       </x:c>
       <x:c r="R129" s="14" t="str">
-        <x:v>Messaging contract reviewed.</x:v>
+        <x:v>Messaging frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S129" s="14" t="str">
         <x:v>Mapper + UI send/offline.</x:v>
@@ -10278,7 +10278,9 @@
       <x:c r="V129" s="14" t="str">
         <x:v>feature/android-chat</x:v>
       </x:c>
-      <x:c r="W129" s="14"/>
+      <x:c r="W129" s="14" t="str">
+        <x:v>DoR PASS: Messaging frontend/mock contract approved; Figma Chat 238:192 y 334:132 disponibles; Backend no requerido para implementación frontend-first.</x:v>
+      </x:c>
       <x:c r="X129" s="14"/>
       <x:c r="Y129" s="14"/>
       <x:c r="Z129" s="14"/>
@@ -10312,7 +10314,7 @@
         <x:v>MEDIA</x:v>
       </x:c>
       <x:c r="J130" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>READY</x:v>
       </x:c>
       <x:c r="K130" s="14" t="str">
         <x:v>IMP-AND-0102</x:v>
@@ -10336,7 +10338,7 @@
         <x:v>No financial assumptions fuera Figma; linked to stay/property.</x:v>
       </x:c>
       <x:c r="R130" s="14" t="str">
-        <x:v>Valet contract confirmed.</x:v>
+        <x:v>Valet frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S130" s="14" t="str">
         <x:v>UI tests.</x:v>
@@ -10350,7 +10352,9 @@
       <x:c r="V130" s="14" t="str">
         <x:v>feature/android-valet</x:v>
       </x:c>
-      <x:c r="W130" s="14"/>
+      <x:c r="W130" s="14" t="str">
+        <x:v>DoR PASS: Valet frontend/mock contract approved; Figma Valet 239:197 y 244:132 disponibles; Backend no requerido para implementación frontend-first.</x:v>
+      </x:c>
       <x:c r="X130" s="14"/>
       <x:c r="Y130" s="14"/>
       <x:c r="Z130" s="14"/>
@@ -10456,7 +10460,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J132" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>READY</x:v>
       </x:c>
       <x:c r="K132" s="14" t="str">
         <x:v>IMP-AND-0009</x:v>
@@ -10480,7 +10484,7 @@
         <x:v>No Staff auth; no provider JSON UI; mapper tests.</x:v>
       </x:c>
       <x:c r="R132" s="14" t="str">
-        <x:v>S0 complete.</x:v>
+        <x:v>Sprint 0 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S132" s="14" t="str">
         <x:v>Unit.</x:v>
@@ -10494,7 +10498,9 @@
       <x:c r="V132" s="14" t="str">
         <x:v>feature/android-account-contract</x:v>
       </x:c>
-      <x:c r="W132" s="14"/>
+      <x:c r="W132" s="14" t="str">
+        <x:v>DoR PASS: GuestAccount != GuestProfile; Account/Profile frontend/mock contract approved; Backend no requerido para implementación frontend-first.</x:v>
+      </x:c>
       <x:c r="X132" s="14"/>
       <x:c r="Y132" s="14"/>
       <x:c r="Z132" s="14"/>
@@ -10552,7 +10558,7 @@
         <x:v>Account/Profile separation; no secrets; save states correct.</x:v>
       </x:c>
       <x:c r="R133" s="14" t="str">
-        <x:v>0201 complete.</x:v>
+        <x:v>IMP-AND-0201 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S133" s="14" t="str">
         <x:v>UI tests.</x:v>
@@ -10600,7 +10606,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J134" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>READY</x:v>
       </x:c>
       <x:c r="K134" s="14" t="str">
         <x:v>IMP-AND-0102</x:v>
@@ -10624,7 +10630,7 @@
         <x:v>Finance no recalculated in UI; no sensitive file persisted; no provider raw data.</x:v>
       </x:c>
       <x:c r="R134" s="14" t="str">
-        <x:v>Folio/Fiscal mobile contract reviewed.</x:v>
+        <x:v>Checkout/Folio frontend/mock contract approved; representación simulada/frontend únicamente hasta integración Backend/fiscal.</x:v>
       </x:c>
       <x:c r="S134" s="14" t="str">
         <x:v>Mapper + UI/security.</x:v>
@@ -10638,7 +10644,9 @@
       <x:c r="V134" s="14" t="str">
         <x:v>feature/android-checkout-invoice</x:v>
       </x:c>
-      <x:c r="W134" s="14"/>
+      <x:c r="W134" s="14" t="str">
+        <x:v>DoR PASS: Checkout/Folio frontend/mock contract approved; implementación frontend simulada únicamente. No implica pago real, factura fiscal real ni integración FEL/SAT; Backend/fiscal se integra posteriormente.</x:v>
+      </x:c>
       <x:c r="X134" s="14"/>
       <x:c r="Y134" s="14"/>
       <x:c r="Z134" s="14"/>
@@ -10744,7 +10752,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J136" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>READY</x:v>
       </x:c>
       <x:c r="K136" s="14" t="str">
         <x:v>IMP-AND-0009</x:v>
@@ -10768,7 +10776,7 @@
         <x:v>CANCELLED/NO_SHOW no elegibles; ledger read-only.</x:v>
       </x:c>
       <x:c r="R136" s="14" t="str">
-        <x:v>Reward contract reviewed.</x:v>
+        <x:v>Rewards frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S136" s="14" t="str">
         <x:v>Mapper + UI.</x:v>
@@ -10782,7 +10790,9 @@
       <x:c r="V136" s="14" t="str">
         <x:v>feature/android-rewards</x:v>
       </x:c>
-      <x:c r="W136" s="14"/>
+      <x:c r="W136" s="14" t="str">
+        <x:v>DoR PASS: Rewards frontend/mock contract approved; Backend no requerido para implementación frontend-first.</x:v>
+      </x:c>
       <x:c r="X136" s="14"/>
       <x:c r="Y136" s="14"/>
       <x:c r="Z136" s="14"/>
@@ -10816,7 +10826,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J137" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>READY</x:v>
       </x:c>
       <x:c r="K137" s="14" t="str">
         <x:v>IMP-AND-0009</x:v>
@@ -10840,7 +10850,7 @@
         <x:v>Incompatible no combinable; reasons correct.</x:v>
       </x:c>
       <x:c r="R137" s="14" t="str">
-        <x:v>Promotion contract reviewed.</x:v>
+        <x:v>Promotions frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S137" s="14" t="str">
         <x:v>Mapper + UI.</x:v>
@@ -10854,7 +10864,9 @@
       <x:c r="V137" s="14" t="str">
         <x:v>feature/android-promotions</x:v>
       </x:c>
-      <x:c r="W137" s="14"/>
+      <x:c r="W137" s="14" t="str">
+        <x:v>DoR PASS: Promotions frontend/mock contract approved; Backend no requerido para implementación frontend-first.</x:v>
+      </x:c>
       <x:c r="X137" s="14"/>
       <x:c r="Y137" s="14"/>
       <x:c r="Z137" s="14"/>
@@ -10912,7 +10924,7 @@
         <x:v>No duplicated model; PII safe; save states correct.</x:v>
       </x:c>
       <x:c r="R138" s="14" t="str">
-        <x:v>Profile contract ready.</x:v>
+        <x:v>IMP-AND-0201 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S138" s="14" t="str">
         <x:v>UI tests.</x:v>
@@ -11342,7 +11354,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79089500d904443e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0194b67f07ef4824"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(android): implement guest chat flow
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R87ac0065fba946ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R1f8cbfa1315a42bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R9bfc85a08fbb49f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R45589663c03a4dcc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R33d7b1cdca3042bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R36f0646809bf42ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="Rcb67e75c10144d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R2929aa16abaf4e2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Rb5723a0abb9d4e59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R6a984ad7a64240c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Rd8c4553f7b3e4260"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R82ce537d3bb84822"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6a5aac43e6864b51"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rca15d1b49c284863"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -804,7 +804,7 @@
       </x:c>
       <x:c r="B6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_PROGRESO")</x:f>
@@ -820,7 +820,7 @@
       </x:c>
       <x:c r="F6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>30</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -888,7 +888,7 @@
       </x:c>
       <x:c r="G11" t="n">
         <x:f>COUNTIFS('01_Backlog'!C2:C142,E11,'01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -927,7 +927,7 @@
       </x:c>
       <x:c r="C14" s="12" t="n">
         <x:f>COUNTIFS('01_Backlog'!E2:E142,A14,'01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f5ef29bc84f4377"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R196ceb18ed2842e5"/>
 </x:worksheet>
 </file>
 
@@ -10240,7 +10240,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J129" s="14" t="str">
-        <x:v>READY</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K129" s="14" t="str">
         <x:v>IMP-AND-0102</x:v>
@@ -10279,7 +10279,7 @@
         <x:v>feature/android-chat</x:v>
       </x:c>
       <x:c r="W129" s="14" t="str">
-        <x:v>DoR PASS: Messaging frontend/mock contract approved; Figma Chat 238:192 y 334:132 disponibles; Backend no requerido para implementación frontend-first.</x:v>
+        <x:v>FINAL PASS 2026-09-11: QA visual/funcional aprobada (composer sobre teclado, footbar oculta/reaparece, flecha izquierda, trim/doble submit, success sin optimismo, draft limpio, mensajes consecutivos, historial y auto-scroll; error/offline conservan draft; sin auto-reply/queue; navegación Chat/Servicios/Valet/Cuenta PASS). WEB-3 review PASS. Técnico: test PASS 9 suites/40; Doctor 21/21 PASS; lint PASS; typecheck PASS; npm run check PASS; git diff --check PASS.</x:v>
       </x:c>
       <x:c r="X129" s="14"/>
       <x:c r="Y129" s="14"/>
@@ -11354,7 +11354,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0194b67f07ef4824"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb89dcb8fdd9406e"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(android): implement valet and transfer flow
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="Rcb67e75c10144d5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R2929aa16abaf4e2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Rb5723a0abb9d4e59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R6a984ad7a64240c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="Rd8c4553f7b3e4260"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R82ce537d3bb84822"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R399be9af763f48aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="Rf712b2289d2d487a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R238bbfe1e6214065"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="Rd15bd98b7e134e5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R35ba96d9d07b4a3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Rb64a3485fc7748a2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rca15d1b49c284863"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R34c19c81c4384092"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -804,7 +804,7 @@
       </x:c>
       <x:c r="B6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_PROGRESO")</x:f>
@@ -820,7 +820,7 @@
       </x:c>
       <x:c r="F6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -888,7 +888,7 @@
       </x:c>
       <x:c r="G11" t="n">
         <x:f>COUNTIFS('01_Backlog'!C2:C142,E11,'01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -927,7 +927,7 @@
       </x:c>
       <x:c r="C14" s="12" t="n">
         <x:f>COUNTIFS('01_Backlog'!E2:E142,A14,'01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R196ceb18ed2842e5"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48c1c06c42eb491d"/>
 </x:worksheet>
 </file>
 
@@ -10314,7 +10314,7 @@
         <x:v>MEDIA</x:v>
       </x:c>
       <x:c r="J130" s="14" t="str">
-        <x:v>READY</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K130" s="14" t="str">
         <x:v>IMP-AND-0102</x:v>
@@ -10353,7 +10353,7 @@
         <x:v>feature/android-valet</x:v>
       </x:c>
       <x:c r="W130" s="14" t="str">
-        <x:v>DoR PASS: Valet frontend/mock contract approved; Figma Valet 239:197 y 244:132 disponibles; Backend no requerido para implementación frontend-first.</x:v>
+        <x:v>FINAL PASS 2026-09-11: QA visual/funcional PASS; WEB-3 review PASS. Vehículo: selector/detalle local, solicitud mock y success centrado PASS. Corrección visual Services Success PASS. Traslado generalizado PASS: tipo HOTEL|PLACE, pickup PLACE condicional para regreso al Hotel, selector mock, distancia/duración mock y tarifa estimada Q40 + Q8/km PASS. Ver ruta en Maps con Linking PASS. Calendario/reloj nativos, Clock, lead time mínimo 30 minutos y revalidación antes de reservar/retry PASS; Backend futuro será la autoridad temporal definitiva. Validación técnica: lint PASS; Expo Doctor 21/21 PASS; typecheck PASS; test PASS 12 suites/68; npm run check PASS; Android export PASS; git diff --check PASS.</x:v>
       </x:c>
       <x:c r="X130" s="14"/>
       <x:c r="Y130" s="14"/>
@@ -11354,7 +11354,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb89dcb8fdd9406e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7f617e8a72e489c"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(android): freeze early journey V3 migration
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R399be9af763f48aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="Rf712b2289d2d487a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R238bbfe1e6214065"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="Rd15bd98b7e134e5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R35ba96d9d07b4a3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Rb64a3485fc7748a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="Rd7a7326eee72480b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="Ra4d691e2273c4750"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R7334b3f39bba4fa9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="Re331cf68db824811"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R738bb23a3b09480b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Rc29636f4ff364216"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R34c19c81c4384092"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc827b7375ffe4780"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -505,7 +505,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationBacklog" displayName="ImplementationBacklog" ref="A1:Z142" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationBacklog" displayName="ImplementationBacklog" ref="A1:Z151" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="26">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Sprint"/>
@@ -804,11 +804,11 @@
       </x:c>
       <x:c r="B6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_PROGRESO")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_QA")</x:f>
@@ -820,7 +820,7 @@
       </x:c>
       <x:c r="F6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -888,7 +888,7 @@
       </x:c>
       <x:c r="G11" t="n">
         <x:f>COUNTIFS('01_Backlog'!C2:C142,E11,'01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -927,7 +927,7 @@
       </x:c>
       <x:c r="C14" s="12" t="n">
         <x:f>COUNTIFS('01_Backlog'!E2:E142,A14,'01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48c1c06c42eb491d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f82350207b24f3e"/>
 </x:worksheet>
 </file>
 
@@ -10388,7 +10388,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J131" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>EN_PROGRESO</x:v>
       </x:c>
       <x:c r="K131" s="14" t="str">
         <x:v>IMP-AND-0102, IMP-AND-0103, IMP-AND-0104, IMP-AND-0105</x:v>
@@ -10426,80 +10426,82 @@
       <x:c r="V131" s="14" t="str">
         <x:v>test/android-stay-services</x:v>
       </x:c>
-      <x:c r="W131" s="14"/>
+      <x:c r="W131" s="14" t="str">
+        <x:v>QA técnica PASS preservada. EN_PROGRESO por hallazgos bloqueantes QA-AND-0106-01 (footbar V1/Stay aislado) y QA-AND-0106-02 (MOB-01 y MOB-03..07 sin migración V3). Ver IMP-AND-0107 / docs Android 23; reejecutar QA tras las migraciones.</x:v>
+      </x:c>
       <x:c r="X131" s="14"/>
       <x:c r="Y131" s="14"/>
       <x:c r="Z131" s="14"/>
     </x:row>
     <x:row r="132" ht="84" customHeight="1">
       <x:c r="A132" s="14" t="str">
-        <x:v>IMP-AND-0201</x:v>
+        <x:v>IMP-AND-0107</x:v>
       </x:c>
       <x:c r="B132" s="14" t="str">
-        <x:v>S2 Android Account</x:v>
+        <x:v>S1 Android Stay &amp; Services</x:v>
       </x:c>
       <x:c r="C132" s="14" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D132" s="14" t="str">
-        <x:v>Cuenta</x:v>
+        <x:v>Navegación</x:v>
       </x:c>
       <x:c r="E132" s="14" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F132" s="14" t="str">
-        <x:v>WEB-2</x:v>
+        <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G132" s="14" t="str">
-        <x:v>account</x:v>
+        <x:v>navigation</x:v>
       </x:c>
       <x:c r="H132" s="14" t="str">
-        <x:v>FEATURE</x:v>
+        <x:v>SHARED</x:v>
       </x:c>
       <x:c r="I132" s="14" t="str">
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J132" s="14" t="str">
-        <x:v>READY</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K132" s="14" t="str">
-        <x:v>IMP-AND-0009</x:v>
+        <x:v>QA-AND-0106-01, QA-AND-0106-02</x:v>
       </x:c>
       <x:c r="L132" s="14" t="str">
-        <x:v>Android 02 Cuenta, checkout y factura</x:v>
+        <x:v>Android Early Journey → V3</x:v>
       </x:c>
       <x:c r="M132" s="14" t="str">
-        <x:v>238:132</x:v>
+        <x:v>31:132 / 238:132</x:v>
       </x:c>
       <x:c r="N132" s="14" t="str">
-        <x:v>Account</x:v>
+        <x:v>MOB-01..07 → MOB-19..25</x:v>
       </x:c>
       <x:c r="O132" s="14" t="str">
-        <x:v>Crear Account/Profile contracts</x:v>
+        <x:v>Change Control + mapa Early Journey → V3</x:v>
       </x:c>
       <x:c r="P132" s="14" t="str">
-        <x:v>GuestAccount/Profile separados; remote-&gt;DTO-&gt;Mapper-&gt;Domain.</x:v>
+        <x:v>Decisiones, rutas, pantallas, dependencias y límites congelados.</x:v>
       </x:c>
       <x:c r="Q132" s="14" t="str">
-        <x:v>No Staff auth; no provider JSON UI; mapper tests.</x:v>
+        <x:v>Sin quinta tab, sin retorno V1, sin Backend ni pantallas.</x:v>
       </x:c>
       <x:c r="R132" s="14" t="str">
-        <x:v>Sprint 0 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
+        <x:v>Hallazgos QA documentados; matriz y gates definidos.</x:v>
       </x:c>
       <x:c r="S132" s="14" t="str">
-        <x:v>Unit.</x:v>
+        <x:v>Documentación y backlog sincronizados; revisión documental pendiente.</x:v>
       </x:c>
       <x:c r="T132" s="14" t="str">
-        <x:v>unit</x:v>
+        <x:v>docs/backlog review</x:v>
       </x:c>
       <x:c r="U132" s="14" t="str">
-        <x:v>account layers</x:v>
+        <x:v>Android S1 migration</x:v>
       </x:c>
       <x:c r="V132" s="14" t="str">
-        <x:v>feature/android-account-contract</x:v>
+        <x:v>qa/android-sprint-1</x:v>
       </x:c>
       <x:c r="W132" s="14" t="str">
-        <x:v>DoR PASS: GuestAccount != GuestProfile; Account/Profile frontend/mock contract approved; Backend no requerido para implementación frontend-first.</x:v>
+        <x:v>COMPLETADA: ANDROID-1 PASS; WEB-3 PASS; WEB-2 CONSULT PASS. Freeze Early Journey → V3 aprobado; rutas y parent-tab semantics aprobadas; orden 0109 → 0108 aprobado; único Account / Stay Hub aprobado; IMP-AND-0201 extiende IMP-AND-0109; sin quinta tab, sin navegación V1 productiva y sin Backend anticipado.</x:v>
       </x:c>
       <x:c r="X132" s="14"/>
       <x:c r="Y132" s="14"/>
@@ -10507,97 +10509,99 @@
     </x:row>
     <x:row r="133" ht="84" customHeight="1">
       <x:c r="A133" s="14" t="str">
-        <x:v>IMP-AND-0202</x:v>
+        <x:v>IMP-AND-0108</x:v>
       </x:c>
       <x:c r="B133" s="14" t="str">
-        <x:v>S2 Android Account</x:v>
+        <x:v>S1 Android Stay &amp; Services</x:v>
       </x:c>
       <x:c r="C133" s="14" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D133" s="14" t="str">
-        <x:v>Cuenta</x:v>
+        <x:v>Acceso</x:v>
       </x:c>
       <x:c r="E133" s="14" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F133" s="14" t="str">
-        <x:v>WEB-2</x:v>
+        <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G133" s="14" t="str">
-        <x:v>account</x:v>
+        <x:v>access</x:v>
       </x:c>
       <x:c r="H133" s="14" t="str">
         <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I133" s="14" t="str">
-        <x:v>ALTA</x:v>
+        <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J133" s="14" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K133" s="14" t="str">
-        <x:v>IMP-AND-0201</x:v>
+        <x:v>IMP-AND-0107, IMP-AND-0109</x:v>
       </x:c>
       <x:c r="L133" s="14" t="str">
-        <x:v>Android 02 Cuenta, checkout y factura</x:v>
+        <x:v>Android Early Journey → V3</x:v>
       </x:c>
       <x:c r="M133" s="14" t="str">
-        <x:v>238:132</x:v>
+        <x:v>31:133 / 238:132</x:v>
       </x:c>
       <x:c r="N133" s="14" t="str">
-        <x:v>Account/Profile</x:v>
+        <x:v>MOB-19 /access</x:v>
       </x:c>
       <x:c r="O133" s="14" t="str">
-        <x:v>Implementar cuenta/perfil</x:v>
+        <x:v>Migrar acceso/vinculación de reserva</x:v>
       </x:c>
       <x:c r="P133" s="14" t="str">
-        <x:v>Display/edit Profile; loading/error/offline; submit.</x:v>
+        <x:v>Ruta /access fuera de GuestNavigationShell.</x:v>
       </x:c>
       <x:c r="Q133" s="14" t="str">
-        <x:v>Account/Profile separation; no secrets; save states correct.</x:v>
+        <x:v>Sin auth real, Backend ni navegación V1.</x:v>
       </x:c>
       <x:c r="R133" s="14" t="str">
-        <x:v>IMP-AND-0201 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
+        <x:v>IMP-AND-0107 y IMP-AND-0109 COMPLETADA; Figma/contrato frontend/mock READY.</x:v>
       </x:c>
       <x:c r="S133" s="14" t="str">
-        <x:v>UI tests.</x:v>
+        <x:v>UI tests</x:v>
       </x:c>
       <x:c r="T133" s="14" t="str">
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U133" s="14" t="str">
-        <x:v>account/profile screens</x:v>
+        <x:v>access</x:v>
       </x:c>
       <x:c r="V133" s="14" t="str">
-        <x:v>feature/android-account-profile</x:v>
-      </x:c>
-      <x:c r="W133" s="14"/>
+        <x:v>feature/android-access-link</x:v>
+      </x:c>
+      <x:c r="W133" s="14" t="str">
+        <x:v>PENDIENTE: orden 0109 → 0108. Tras vinculación exitosa, /access → /account → Account / Stay Hub V3; /access permanece fuera de GuestNavigationShell.</x:v>
+      </x:c>
       <x:c r="X133" s="14"/>
       <x:c r="Y133" s="14"/>
       <x:c r="Z133" s="14"/>
     </x:row>
     <x:row r="134" ht="84" customHeight="1">
       <x:c r="A134" s="14" t="str">
-        <x:v>IMP-AND-0203</x:v>
+        <x:v>IMP-AND-0109</x:v>
       </x:c>
       <x:c r="B134" s="14" t="str">
-        <x:v>S2 Android Account</x:v>
+        <x:v>S1 Android Stay &amp; Services</x:v>
       </x:c>
       <x:c r="C134" s="14" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D134" s="14" t="str">
-        <x:v>Checkout/Factura</x:v>
+        <x:v>Cuenta / Estancia</x:v>
       </x:c>
       <x:c r="E134" s="14" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F134" s="14" t="str">
-        <x:v>WEB-4</x:v>
+        <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G134" s="14" t="str">
-        <x:v>checkout</x:v>
+        <x:v>account</x:v>
       </x:c>
       <x:c r="H134" s="14" t="str">
         <x:v>FEATURE</x:v>
@@ -10606,46 +10610,46 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J134" s="14" t="str">
-        <x:v>READY</x:v>
+        <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K134" s="14" t="str">
-        <x:v>IMP-AND-0102</x:v>
+        <x:v>IMP-AND-0107</x:v>
       </x:c>
       <x:c r="L134" s="14" t="str">
-        <x:v>Android 02 Cuenta, checkout y factura</x:v>
+        <x:v>Android Early Journey → V3</x:v>
       </x:c>
       <x:c r="M134" s="14" t="str">
-        <x:v>238:132</x:v>
+        <x:v>31:154 / 238:132</x:v>
       </x:c>
       <x:c r="N134" s="14" t="str">
-        <x:v>Checkout/Invoice</x:v>
+        <x:v>MOB-20 /account</x:v>
       </x:c>
       <x:c r="O134" s="14" t="str">
-        <x:v>Implementar checkout e invoice</x:v>
+        <x:v>Migrar Mi estadía a Account / Stay Hub</x:v>
       </x:c>
       <x:c r="P134" s="14" t="str">
-        <x:v>Charges/balance/status Folio read model; invoice ref/status/date/total; offline/error.</x:v>
+        <x:v>Cuenta activa en /account y rutas hijas; base de Stay Hub.</x:v>
       </x:c>
       <x:c r="Q134" s="14" t="str">
-        <x:v>Finance no recalculated in UI; no sensitive file persisted; no provider raw data.</x:v>
+        <x:v>No quinta tab ni segundo hub /account.</x:v>
       </x:c>
       <x:c r="R134" s="14" t="str">
-        <x:v>Checkout/Folio frontend/mock contract approved; representación simulada/frontend únicamente hasta integración Backend/fiscal.</x:v>
+        <x:v>IMP-AND-0107 COMPLETADA; Figma/contrato frontend/mock READY.</x:v>
       </x:c>
       <x:c r="S134" s="14" t="str">
-        <x:v>Mapper + UI/security.</x:v>
+        <x:v>UI tests</x:v>
       </x:c>
       <x:c r="T134" s="14" t="str">
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U134" s="14" t="str">
-        <x:v>checkout/invoice</x:v>
+        <x:v>account/stay hub</x:v>
       </x:c>
       <x:c r="V134" s="14" t="str">
-        <x:v>feature/android-checkout-invoice</x:v>
+        <x:v>feature/android-account-stay-hub</x:v>
       </x:c>
       <x:c r="W134" s="14" t="str">
-        <x:v>DoR PASS: Checkout/Folio frontend/mock contract approved; implementación frontend simulada únicamente. No implica pago real, factura fiscal real ni integración FEL/SAT; Backend/fiscal se integra posteriormente.</x:v>
+        <x:v>PENDIENTE: implementa primero el destino /account y el Account / Stay Hub V3 requerido para el post-success validable de IMP-AND-0108.</x:v>
       </x:c>
       <x:c r="X134" s="14"/>
       <x:c r="Y134" s="14"/>
@@ -10653,70 +10657,70 @@
     </x:row>
     <x:row r="135" ht="84" customHeight="1">
       <x:c r="A135" s="14" t="str">
-        <x:v>IMP-AND-0204</x:v>
+        <x:v>IMP-AND-0110</x:v>
       </x:c>
       <x:c r="B135" s="14" t="str">
-        <x:v>S2 Android Account</x:v>
+        <x:v>S1 Android Stay &amp; Services</x:v>
       </x:c>
       <x:c r="C135" s="14" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D135" s="14" t="str">
-        <x:v>QA</x:v>
+        <x:v>Servicios / Limpieza</x:v>
       </x:c>
       <x:c r="E135" s="14" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F135" s="14" t="str">
-        <x:v>WEB-2</x:v>
+        <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G135" s="14" t="str">
-        <x:v>account-checkout</x:v>
+        <x:v>services</x:v>
       </x:c>
       <x:c r="H135" s="14" t="str">
-        <x:v>QA</x:v>
+        <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I135" s="14" t="str">
-        <x:v>CRÍTICA</x:v>
+        <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J135" s="14" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K135" s="14" t="str">
-        <x:v>IMP-AND-0202, IMP-AND-0203</x:v>
+        <x:v>IMP-AND-0107, IMP-AND-0103</x:v>
       </x:c>
       <x:c r="L135" s="14" t="str">
-        <x:v>Android 02 Cuenta, checkout y factura</x:v>
+        <x:v>Android Early Journey → V3</x:v>
       </x:c>
       <x:c r="M135" s="14" t="str">
-        <x:v>238:132</x:v>
+        <x:v>31:191 / 238:132</x:v>
       </x:c>
       <x:c r="N135" s="14" t="str">
-        <x:v>Account/Checkout</x:v>
+        <x:v>MOB-21 /services/housekeeping</x:v>
       </x:c>
       <x:c r="O135" s="14" t="str">
-        <x:v>QA Cuenta/Checkout/Factura</x:v>
+        <x:v>Migrar Solicitar limpieza</x:v>
       </x:c>
       <x:c r="P135" s="14" t="str">
-        <x:v>Profile/checkout/invoice/states/navigation/contracts.</x:v>
+        <x:v>Servicios activa en /services/housekeeping.</x:v>
       </x:c>
       <x:c r="Q135" s="14" t="str">
-        <x:v>Guest/Staff separation; finance coherent; Figma parity.</x:v>
+        <x:v>Sin Backend ni duplicar GuestNavigationShell.</x:v>
       </x:c>
       <x:c r="R135" s="14" t="str">
-        <x:v>S2 done.</x:v>
+        <x:v>IMP-AND-0107 y IMP-AND-0103 COMPLETADA; contrato frontend/mock READY.</x:v>
       </x:c>
       <x:c r="S135" s="14" t="str">
-        <x:v>Android Global DoD.</x:v>
+        <x:v>UI tests</x:v>
       </x:c>
       <x:c r="T135" s="14" t="str">
-        <x:v>build/tests/manual</x:v>
+        <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U135" s="14" t="str">
-        <x:v>Android S2</x:v>
+        <x:v>services/housekeeping</x:v>
       </x:c>
       <x:c r="V135" s="14" t="str">
-        <x:v>test/android-account-checkout</x:v>
+        <x:v>feature/android-services-housekeeping</x:v>
       </x:c>
       <x:c r="W135" s="14"/>
       <x:c r="X135" s="14"/>
@@ -10725,25 +10729,25 @@
     </x:row>
     <x:row r="136" ht="84" customHeight="1">
       <x:c r="A136" s="14" t="str">
-        <x:v>IMP-AND-0301</x:v>
+        <x:v>IMP-AND-0111</x:v>
       </x:c>
       <x:c r="B136" s="14" t="str">
-        <x:v>S3 Android Loyalty</x:v>
+        <x:v>S1 Android Stay &amp; Services</x:v>
       </x:c>
       <x:c r="C136" s="14" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D136" s="14" t="str">
-        <x:v>Loyalty</x:v>
+        <x:v>Servicios / Room Service</x:v>
       </x:c>
       <x:c r="E136" s="14" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F136" s="14" t="str">
-        <x:v>WEB-2</x:v>
+        <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G136" s="14" t="str">
-        <x:v>rewards</x:v>
+        <x:v>services</x:v>
       </x:c>
       <x:c r="H136" s="14" t="str">
         <x:v>FEATURE</x:v>
@@ -10752,72 +10756,70 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J136" s="14" t="str">
-        <x:v>READY</x:v>
+        <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K136" s="14" t="str">
-        <x:v>IMP-AND-0009</x:v>
+        <x:v>IMP-AND-0107, IMP-AND-0103</x:v>
       </x:c>
       <x:c r="L136" s="14" t="str">
-        <x:v>Android 03 Loyalty, promociones y perfil</x:v>
+        <x:v>Android Early Journey → V3</x:v>
       </x:c>
       <x:c r="M136" s="14" t="str">
-        <x:v>238:132</x:v>
+        <x:v>31:221 / 238:132</x:v>
       </x:c>
       <x:c r="N136" s="14" t="str">
-        <x:v>Rewards</x:v>
+        <x:v>MOB-22 /services/room-service</x:v>
       </x:c>
       <x:c r="O136" s="14" t="str">
-        <x:v>Implementar Rewards</x:v>
+        <x:v>Migrar Room Service</x:v>
       </x:c>
       <x:c r="P136" s="14" t="str">
-        <x:v>Ledger/balance Domain cross-app; offline/error/empty.</x:v>
+        <x:v>Servicios activa en /services/room-service.</x:v>
       </x:c>
       <x:c r="Q136" s="14" t="str">
-        <x:v>CANCELLED/NO_SHOW no elegibles; ledger read-only.</x:v>
+        <x:v>Sin Backend ni duplicar GuestNavigationShell.</x:v>
       </x:c>
       <x:c r="R136" s="14" t="str">
-        <x:v>Rewards frontend/mock contract approved.</x:v>
+        <x:v>IMP-AND-0107 y IMP-AND-0103 COMPLETADA; contrato frontend/mock READY.</x:v>
       </x:c>
       <x:c r="S136" s="14" t="str">
-        <x:v>Mapper + UI.</x:v>
+        <x:v>UI tests</x:v>
       </x:c>
       <x:c r="T136" s="14" t="str">
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U136" s="14" t="str">
-        <x:v>rewards</x:v>
+        <x:v>services/room-service</x:v>
       </x:c>
       <x:c r="V136" s="14" t="str">
-        <x:v>feature/android-rewards</x:v>
-      </x:c>
-      <x:c r="W136" s="14" t="str">
-        <x:v>DoR PASS: Rewards frontend/mock contract approved; Backend no requerido para implementación frontend-first.</x:v>
-      </x:c>
+        <x:v>feature/android-services-room-service</x:v>
+      </x:c>
+      <x:c r="W136" s="14"/>
       <x:c r="X136" s="14"/>
       <x:c r="Y136" s="14"/>
       <x:c r="Z136" s="14"/>
     </x:row>
     <x:row r="137" ht="84" customHeight="1">
       <x:c r="A137" s="14" t="str">
-        <x:v>IMP-AND-0302</x:v>
+        <x:v>IMP-AND-0112</x:v>
       </x:c>
       <x:c r="B137" s="14" t="str">
-        <x:v>S3 Android Loyalty</x:v>
+        <x:v>S1 Android Stay &amp; Services</x:v>
       </x:c>
       <x:c r="C137" s="14" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D137" s="14" t="str">
-        <x:v>Promociones</x:v>
+        <x:v>Servicios / Solicitudes</x:v>
       </x:c>
       <x:c r="E137" s="14" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F137" s="14" t="str">
-        <x:v>WEB-2</x:v>
+        <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G137" s="14" t="str">
-        <x:v>promotions</x:v>
+        <x:v>services</x:v>
       </x:c>
       <x:c r="H137" s="14" t="str">
         <x:v>FEATURE</x:v>
@@ -10826,72 +10828,70 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J137" s="14" t="str">
-        <x:v>READY</x:v>
+        <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K137" s="14" t="str">
-        <x:v>IMP-AND-0009</x:v>
+        <x:v>IMP-AND-0107, IMP-AND-0103</x:v>
       </x:c>
       <x:c r="L137" s="14" t="str">
-        <x:v>Android 03 Loyalty, promociones y perfil</x:v>
+        <x:v>Android Early Journey → V3</x:v>
       </x:c>
       <x:c r="M137" s="14" t="str">
-        <x:v>238:132</x:v>
+        <x:v>31:264 / 238:132</x:v>
       </x:c>
       <x:c r="N137" s="14" t="str">
-        <x:v>Promotions</x:v>
+        <x:v>MOB-23 /services/requests</x:v>
       </x:c>
       <x:c r="O137" s="14" t="str">
-        <x:v>Implementar Promotions</x:v>
+        <x:v>Migrar Estado de solicitudes</x:v>
       </x:c>
       <x:c r="P137" s="14" t="str">
-        <x:v>Eligibility/vigencia/stacking reason; states.</x:v>
+        <x:v>Servicios activa en /services/requests.</x:v>
       </x:c>
       <x:c r="Q137" s="14" t="str">
-        <x:v>Incompatible no combinable; reasons correct.</x:v>
+        <x:v>Sin Backend ni duplicar GuestNavigationShell.</x:v>
       </x:c>
       <x:c r="R137" s="14" t="str">
-        <x:v>Promotions frontend/mock contract approved.</x:v>
+        <x:v>IMP-AND-0107 y IMP-AND-0103 COMPLETADA; contrato frontend/mock READY.</x:v>
       </x:c>
       <x:c r="S137" s="14" t="str">
-        <x:v>Mapper + UI.</x:v>
+        <x:v>UI tests</x:v>
       </x:c>
       <x:c r="T137" s="14" t="str">
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U137" s="14" t="str">
-        <x:v>promotions</x:v>
+        <x:v>services/requests</x:v>
       </x:c>
       <x:c r="V137" s="14" t="str">
-        <x:v>feature/android-promotions</x:v>
-      </x:c>
-      <x:c r="W137" s="14" t="str">
-        <x:v>DoR PASS: Promotions frontend/mock contract approved; Backend no requerido para implementación frontend-first.</x:v>
-      </x:c>
+        <x:v>feature/android-services-requests</x:v>
+      </x:c>
+      <x:c r="W137" s="14"/>
       <x:c r="X137" s="14"/>
       <x:c r="Y137" s="14"/>
       <x:c r="Z137" s="14"/>
     </x:row>
     <x:row r="138" ht="84" customHeight="1">
       <x:c r="A138" s="14" t="str">
-        <x:v>IMP-AND-0303</x:v>
+        <x:v>IMP-AND-0113</x:v>
       </x:c>
       <x:c r="B138" s="14" t="str">
-        <x:v>S3 Android Loyalty</x:v>
+        <x:v>S1 Android Stay &amp; Services</x:v>
       </x:c>
       <x:c r="C138" s="14" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D138" s="14" t="str">
-        <x:v>Perfil</x:v>
+        <x:v>Servicios / Amenidades</x:v>
       </x:c>
       <x:c r="E138" s="14" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F138" s="14" t="str">
-        <x:v>WEB-2</x:v>
+        <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G138" s="14" t="str">
-        <x:v>profile</x:v>
+        <x:v>services</x:v>
       </x:c>
       <x:c r="H138" s="14" t="str">
         <x:v>FEATURE</x:v>
@@ -10903,40 +10903,40 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K138" s="14" t="str">
-        <x:v>IMP-AND-0201</x:v>
+        <x:v>IMP-AND-0107, IMP-AND-0103</x:v>
       </x:c>
       <x:c r="L138" s="14" t="str">
-        <x:v>Android 03 Loyalty, promociones y perfil</x:v>
+        <x:v>Android Early Journey → V3</x:v>
       </x:c>
       <x:c r="M138" s="14" t="str">
-        <x:v>238:132</x:v>
+        <x:v>31:299 / 238:132</x:v>
       </x:c>
       <x:c r="N138" s="14" t="str">
-        <x:v>Profile</x:v>
+        <x:v>MOB-24 /services/amenities</x:v>
       </x:c>
       <x:c r="O138" s="14" t="str">
-        <x:v>Implementar perfil final</x:v>
+        <x:v>Migrar Amenidades</x:v>
       </x:c>
       <x:c r="P138" s="14" t="str">
-        <x:v>Figma layout/edit/states; reuse Account/Profile Domain.</x:v>
+        <x:v>Servicios activa en /services/amenities.</x:v>
       </x:c>
       <x:c r="Q138" s="14" t="str">
-        <x:v>No duplicated model; PII safe; save states correct.</x:v>
+        <x:v>Sin Backend ni duplicar GuestNavigationShell.</x:v>
       </x:c>
       <x:c r="R138" s="14" t="str">
-        <x:v>IMP-AND-0201 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
+        <x:v>IMP-AND-0107 y IMP-AND-0103 COMPLETADA; contrato frontend/mock READY.</x:v>
       </x:c>
       <x:c r="S138" s="14" t="str">
-        <x:v>UI tests.</x:v>
+        <x:v>UI tests</x:v>
       </x:c>
       <x:c r="T138" s="14" t="str">
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U138" s="14" t="str">
-        <x:v>profile</x:v>
+        <x:v>services/amenities</x:v>
       </x:c>
       <x:c r="V138" s="14" t="str">
-        <x:v>feature/android-profile</x:v>
+        <x:v>feature/android-services-amenities</x:v>
       </x:c>
       <x:c r="W138" s="14"/>
       <x:c r="X138" s="14"/>
@@ -10945,70 +10945,70 @@
     </x:row>
     <x:row r="139" ht="84" customHeight="1">
       <x:c r="A139" s="14" t="str">
-        <x:v>IMP-AND-0304</x:v>
+        <x:v>IMP-AND-0114</x:v>
       </x:c>
       <x:c r="B139" s="14" t="str">
-        <x:v>S3 Android Loyalty</x:v>
+        <x:v>S1 Android Stay &amp; Services</x:v>
       </x:c>
       <x:c r="C139" s="14" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D139" s="14" t="str">
-        <x:v>QA</x:v>
+        <x:v>Servicios / Información</x:v>
       </x:c>
       <x:c r="E139" s="14" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F139" s="14" t="str">
-        <x:v>WEB-2</x:v>
+        <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G139" s="14" t="str">
-        <x:v>loyalty-profile</x:v>
+        <x:v>services</x:v>
       </x:c>
       <x:c r="H139" s="14" t="str">
-        <x:v>QA</x:v>
+        <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I139" s="14" t="str">
-        <x:v>CRÍTICA</x:v>
+        <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J139" s="14" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K139" s="14" t="str">
-        <x:v>IMP-AND-0301, IMP-AND-0302, IMP-AND-0303</x:v>
+        <x:v>IMP-AND-0107, IMP-AND-0103</x:v>
       </x:c>
       <x:c r="L139" s="14" t="str">
-        <x:v>Android 03 Loyalty, promociones y perfil</x:v>
+        <x:v>Android Early Journey → V3</x:v>
       </x:c>
       <x:c r="M139" s="14" t="str">
-        <x:v>238:132</x:v>
+        <x:v>31:338 / 238:132</x:v>
       </x:c>
       <x:c r="N139" s="14" t="str">
-        <x:v>Rewards/Promos/Profile</x:v>
+        <x:v>MOB-25 /services/hotel-info</x:v>
       </x:c>
       <x:c r="O139" s="14" t="str">
-        <x:v>QA Loyalty/Profile</x:v>
+        <x:v>Migrar Información del hotel</x:v>
       </x:c>
       <x:c r="P139" s="14" t="str">
-        <x:v>Rewards/promotions/profile/offline/error/empty/navigation.</x:v>
+        <x:v>Servicios activa en /services/hotel-info.</x:v>
       </x:c>
       <x:c r="Q139" s="14" t="str">
-        <x:v>Cross-app semantics PASS; Figma parity; no DTO UI.</x:v>
+        <x:v>Sin Backend ni duplicar GuestNavigationShell.</x:v>
       </x:c>
       <x:c r="R139" s="14" t="str">
-        <x:v>S3 done.</x:v>
+        <x:v>IMP-AND-0107 y IMP-AND-0103 COMPLETADA; contrato frontend/mock READY.</x:v>
       </x:c>
       <x:c r="S139" s="14" t="str">
-        <x:v>Android Global DoD.</x:v>
+        <x:v>UI tests</x:v>
       </x:c>
       <x:c r="T139" s="14" t="str">
-        <x:v>build/tests/manual</x:v>
+        <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U139" s="14" t="str">
-        <x:v>Android S3</x:v>
+        <x:v>services/hotel-info</x:v>
       </x:c>
       <x:c r="V139" s="14" t="str">
-        <x:v>test/android-loyalty</x:v>
+        <x:v>feature/android-services-hotel-info</x:v>
       </x:c>
       <x:c r="W139" s="14"/>
       <x:c r="X139" s="14"/>
@@ -11017,16 +11017,16 @@
     </x:row>
     <x:row r="140" ht="84" customHeight="1">
       <x:c r="A140" s="14" t="str">
-        <x:v>IMP-AND-0401</x:v>
+        <x:v>IMP-AND-0201</x:v>
       </x:c>
       <x:c r="B140" s="14" t="str">
-        <x:v>S4 Android Release</x:v>
+        <x:v>S2 Android Account</x:v>
       </x:c>
       <x:c r="C140" s="14" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D140" s="14" t="str">
-        <x:v>Estados</x:v>
+        <x:v>Cuenta</x:v>
       </x:c>
       <x:c r="E140" s="14" t="str">
         <x:v>ANDROID-1</x:v>
@@ -11035,10 +11035,10 @@
         <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G140" s="14" t="str">
-        <x:v>ui-states</x:v>
+        <x:v>account</x:v>
       </x:c>
       <x:c r="H140" s="14" t="str">
-        <x:v>SHARED</x:v>
+        <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I140" s="14" t="str">
         <x:v>CRÍTICA</x:v>
@@ -11047,112 +11047,114 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K140" s="14" t="str">
-        <x:v>IMP-AND-0009</x:v>
+        <x:v>IMP-AND-0009, IMP-AND-0109</x:v>
       </x:c>
       <x:c r="L140" s="14" t="str">
-        <x:v>Android 04 Loading, error y offline</x:v>
+        <x:v>Android 02 Cuenta, checkout y factura</x:v>
       </x:c>
       <x:c r="M140" s="14" t="str">
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N140" s="14" t="str">
-        <x:v>Universal States</x:v>
+        <x:v>Account</x:v>
       </x:c>
       <x:c r="O140" s="14" t="str">
-        <x:v>Implementar Loading/Error/Empty/Offline shared</x:v>
+        <x:v>Crear Account/Profile contracts</x:v>
       </x:c>
       <x:c r="P140" s="14" t="str">
-        <x:v>Reusable state UI; retry callback; accessible; no business logic.</x:v>
+        <x:v>GuestAccount/Profile separados; extiende Account / Stay Hub existente; no duplica /account.</x:v>
       </x:c>
       <x:c r="Q140" s="14" t="str">
-        <x:v>Features reutilizan states; offline explicit; retry actionable.</x:v>
+        <x:v>No Staff auth; no provider JSON UI; mapper tests; sin segundo hub /account.</x:v>
       </x:c>
       <x:c r="R140" s="14" t="str">
-        <x:v>Figma states reviewed.</x:v>
+        <x:v>IMP-AND-0109 COMPLETADA; Sprint 0 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S140" s="14" t="str">
-        <x:v>UI tests.</x:v>
+        <x:v>Unit.</x:v>
       </x:c>
       <x:c r="T140" s="14" t="str">
-        <x:v>ui</x:v>
+        <x:v>unit</x:v>
       </x:c>
       <x:c r="U140" s="14" t="str">
-        <x:v>shared state UI</x:v>
+        <x:v>account layers</x:v>
       </x:c>
       <x:c r="V140" s="14" t="str">
-        <x:v>feature/android-universal-states</x:v>
-      </x:c>
-      <x:c r="W140" s="14"/>
+        <x:v>feature/android-account-contract</x:v>
+      </x:c>
+      <x:c r="W140" s="14" t="str">
+        <x:v>PENDIENTE: IMP-AND-0109 debe completar el Account / Stay Hub en /account. Account/Profile lo extiende sin crear un segundo hub ni duplicar la ruta.</x:v>
+      </x:c>
       <x:c r="X140" s="14"/>
       <x:c r="Y140" s="14"/>
       <x:c r="Z140" s="14"/>
     </x:row>
     <x:row r="141" ht="84" customHeight="1">
       <x:c r="A141" s="14" t="str">
-        <x:v>IMP-AND-0402</x:v>
+        <x:v>IMP-AND-0202</x:v>
       </x:c>
       <x:c r="B141" s="14" t="str">
-        <x:v>S4 Android Release</x:v>
+        <x:v>S2 Android Account</x:v>
       </x:c>
       <x:c r="C141" s="14" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D141" s="14" t="str">
-        <x:v>Estados</x:v>
+        <x:v>Cuenta</x:v>
       </x:c>
       <x:c r="E141" s="14" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F141" s="14" t="str">
-        <x:v>WEB-3</x:v>
+        <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G141" s="14" t="str">
-        <x:v>offline</x:v>
+        <x:v>account</x:v>
       </x:c>
       <x:c r="H141" s="14" t="str">
         <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I141" s="14" t="str">
-        <x:v>CRÍTICA</x:v>
+        <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J141" s="14" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K141" s="14" t="str">
-        <x:v>IMP-AND-0401, IMP-AND-0106, IMP-AND-0204, IMP-AND-0304</x:v>
+        <x:v>IMP-AND-0201</x:v>
       </x:c>
       <x:c r="L141" s="14" t="str">
-        <x:v>Android 04 Loading, error y offline</x:v>
+        <x:v>Android 02 Cuenta, checkout y factura</x:v>
       </x:c>
       <x:c r="M141" s="14" t="str">
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N141" s="14" t="str">
-        <x:v>All</x:v>
+        <x:v>Account/Profile</x:v>
       </x:c>
       <x:c r="O141" s="14" t="str">
-        <x:v>Integrar states universales</x:v>
+        <x:v>Implementar cuenta/perfil</x:v>
       </x:c>
       <x:c r="P141" s="14" t="str">
-        <x:v>Reemplazar estados ad-hoc; retry; stale indication donde aplica.</x:v>
+        <x:v>Display/edit Profile; loading/error/offline; submit.</x:v>
       </x:c>
       <x:c r="Q141" s="14" t="str">
-        <x:v>0 remote screen sin Loading/Error; Offline según Figma; no false success.</x:v>
+        <x:v>Account/Profile separation; no secrets; save states correct.</x:v>
       </x:c>
       <x:c r="R141" s="14" t="str">
-        <x:v>Feature screens done.</x:v>
+        <x:v>IMP-AND-0201 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S141" s="14" t="str">
-        <x:v>Regression states.</x:v>
+        <x:v>UI tests.</x:v>
       </x:c>
       <x:c r="T141" s="14" t="str">
-        <x:v>ui/manual</x:v>
+        <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U141" s="14" t="str">
-        <x:v>all Android</x:v>
+        <x:v>account/profile screens</x:v>
       </x:c>
       <x:c r="V141" s="14" t="str">
-        <x:v>feature/android-state-integration</x:v>
+        <x:v>feature/android-account-profile</x:v>
       </x:c>
       <x:c r="W141" s="14"/>
       <x:c r="X141" s="14"/>
@@ -11161,82 +11163,84 @@
     </x:row>
     <x:row r="142" ht="84" customHeight="1">
       <x:c r="A142" s="14" t="str">
-        <x:v>IMP-AND-0403</x:v>
+        <x:v>IMP-AND-0203</x:v>
       </x:c>
       <x:c r="B142" s="14" t="str">
-        <x:v>S4 Android Release</x:v>
+        <x:v>S2 Android Account</x:v>
       </x:c>
       <x:c r="C142" s="14" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D142" s="14" t="str">
-        <x:v>QA</x:v>
+        <x:v>Checkout/Factura</x:v>
       </x:c>
       <x:c r="E142" s="14" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F142" s="14" t="str">
-        <x:v>WEB-2</x:v>
+        <x:v>WEB-4</x:v>
       </x:c>
       <x:c r="G142" s="14" t="str">
-        <x:v>accessibility</x:v>
+        <x:v>checkout</x:v>
       </x:c>
       <x:c r="H142" s="14" t="str">
-        <x:v>QA</x:v>
+        <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I142" s="14" t="str">
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J142" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>READY</x:v>
       </x:c>
       <x:c r="K142" s="14" t="str">
-        <x:v>IMP-AND-0402</x:v>
+        <x:v>IMP-AND-0102</x:v>
       </x:c>
       <x:c r="L142" s="14" t="str">
-        <x:v>Android final regression</x:v>
+        <x:v>Android 02 Cuenta, checkout y factura</x:v>
       </x:c>
       <x:c r="M142" s="14" t="str">
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N142" s="14" t="str">
-        <x:v>All</x:v>
+        <x:v>Checkout/Invoice</x:v>
       </x:c>
       <x:c r="O142" s="14" t="str">
-        <x:v>Auditoría accesibilidad Android</x:v>
+        <x:v>Implementar checkout e invoice</x:v>
       </x:c>
       <x:c r="P142" s="14" t="str">
-        <x:v>TalkBack/labels/targets/contrast/focus/auth/errors.</x:v>
+        <x:v>Charges/balance/status Folio read model; invoice ref/status/date/total; offline/error.</x:v>
       </x:c>
       <x:c r="Q142" s="14" t="str">
-        <x:v>0 critical/high accessibility defects; primary journeys operable.</x:v>
+        <x:v>Finance no recalculated in UI; no sensitive file persisted; no provider raw data.</x:v>
       </x:c>
       <x:c r="R142" s="14" t="str">
-        <x:v>Features done.</x:v>
+        <x:v>Checkout/Folio frontend/mock contract approved; representación simulada/frontend únicamente hasta integración Backend/fiscal.</x:v>
       </x:c>
       <x:c r="S142" s="14" t="str">
-        <x:v>A11y PASS.</x:v>
+        <x:v>Mapper + UI/security.</x:v>
       </x:c>
       <x:c r="T142" s="14" t="str">
-        <x:v>manual/tooling</x:v>
+        <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U142" s="14" t="str">
-        <x:v>whole Android</x:v>
+        <x:v>checkout/invoice</x:v>
       </x:c>
       <x:c r="V142" s="14" t="str">
-        <x:v>test/android-a11y</x:v>
-      </x:c>
-      <x:c r="W142" s="14"/>
+        <x:v>feature/android-checkout-invoice</x:v>
+      </x:c>
+      <x:c r="W142" s="14" t="str">
+        <x:v>DoR PASS: Checkout/Folio frontend/mock contract approved; implementación frontend simulada únicamente. No implica pago real, factura fiscal real ni integración FEL/SAT; Backend/fiscal se integra posteriormente.</x:v>
+      </x:c>
       <x:c r="X142" s="14"/>
       <x:c r="Y142" s="14"/>
       <x:c r="Z142" s="14"/>
     </x:row>
     <x:row r="143">
       <x:c r="A143" t="str">
-        <x:v>IMP-AND-0404</x:v>
+        <x:v>IMP-AND-0204</x:v>
       </x:c>
       <x:c r="B143" t="str">
-        <x:v>S4 Android Release</x:v>
+        <x:v>S2 Android Account</x:v>
       </x:c>
       <x:c r="C143" t="str">
         <x:v>ANDROID</x:v>
@@ -11248,10 +11252,10 @@
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F143" t="str">
-        <x:v>WEB-3</x:v>
+        <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G143" t="str">
-        <x:v>release</x:v>
+        <x:v>account-checkout</x:v>
       </x:c>
       <x:c r="H143" t="str">
         <x:v>QA</x:v>
@@ -11263,45 +11267,581 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K143" t="str">
-        <x:v>IMP-AND-0403</x:v>
+        <x:v>IMP-AND-0202, IMP-AND-0203</x:v>
       </x:c>
       <x:c r="L143" t="str">
-        <x:v>Android final regression</x:v>
+        <x:v>Android 02 Cuenta, checkout y factura</x:v>
       </x:c>
       <x:c r="M143" t="str">
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N143" t="str">
-        <x:v>All</x:v>
+        <x:v>Account/Checkout</x:v>
       </x:c>
       <x:c r="O143" t="str">
-        <x:v>Regresión final Android</x:v>
+        <x:v>QA Cuenta/Checkout/Factura</x:v>
       </x:c>
       <x:c r="P143" t="str">
-        <x:v>Build/tests/navigation/states/contracts/no DTO UI/no secrets.</x:v>
+        <x:v>Profile/checkout/invoice/states/navigation/contracts.</x:v>
       </x:c>
       <x:c r="Q143" t="str">
-        <x:v>0 critical/high; all checks PASS; release candidate.</x:v>
+        <x:v>Guest/Staff separation; finance coherent; Figma parity.</x:v>
       </x:c>
       <x:c r="R143" t="str">
-        <x:v>All Android tasks done.</x:v>
+        <x:v>S2 done.</x:v>
       </x:c>
       <x:c r="S143" t="str">
-        <x:v>Release DoD PASS.</x:v>
+        <x:v>Android Global DoD.</x:v>
       </x:c>
       <x:c r="T143" t="str">
         <x:v>build/tests/manual</x:v>
       </x:c>
       <x:c r="U143" t="str">
-        <x:v>whole Android</x:v>
+        <x:v>Android S2</x:v>
       </x:c>
       <x:c r="V143" t="str">
-        <x:v>release/android-rc</x:v>
+        <x:v>test/android-account-checkout</x:v>
       </x:c>
       <x:c r="W143"/>
       <x:c r="X143"/>
       <x:c r="Y143"/>
       <x:c r="Z143"/>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" t="str">
+        <x:v>IMP-AND-0301</x:v>
+      </x:c>
+      <x:c r="B144" t="str">
+        <x:v>S3 Android Loyalty</x:v>
+      </x:c>
+      <x:c r="C144" t="str">
+        <x:v>ANDROID</x:v>
+      </x:c>
+      <x:c r="D144" t="str">
+        <x:v>Loyalty</x:v>
+      </x:c>
+      <x:c r="E144" t="str">
+        <x:v>ANDROID-1</x:v>
+      </x:c>
+      <x:c r="F144" t="str">
+        <x:v>WEB-2</x:v>
+      </x:c>
+      <x:c r="G144" t="str">
+        <x:v>rewards</x:v>
+      </x:c>
+      <x:c r="H144" t="str">
+        <x:v>FEATURE</x:v>
+      </x:c>
+      <x:c r="I144" t="str">
+        <x:v>ALTA</x:v>
+      </x:c>
+      <x:c r="J144" t="str">
+        <x:v>READY</x:v>
+      </x:c>
+      <x:c r="K144" t="str">
+        <x:v>IMP-AND-0009</x:v>
+      </x:c>
+      <x:c r="L144" t="str">
+        <x:v>Android 03 Loyalty, promociones y perfil</x:v>
+      </x:c>
+      <x:c r="M144" t="str">
+        <x:v>238:132</x:v>
+      </x:c>
+      <x:c r="N144" t="str">
+        <x:v>Rewards</x:v>
+      </x:c>
+      <x:c r="O144" t="str">
+        <x:v>Implementar Rewards</x:v>
+      </x:c>
+      <x:c r="P144" t="str">
+        <x:v>Ledger/balance Domain cross-app; offline/error/empty.</x:v>
+      </x:c>
+      <x:c r="Q144" t="str">
+        <x:v>CANCELLED/NO_SHOW no elegibles; ledger read-only.</x:v>
+      </x:c>
+      <x:c r="R144" t="str">
+        <x:v>Rewards frontend/mock contract approved.</x:v>
+      </x:c>
+      <x:c r="S144" t="str">
+        <x:v>Mapper + UI.</x:v>
+      </x:c>
+      <x:c r="T144" t="str">
+        <x:v>unit/ui</x:v>
+      </x:c>
+      <x:c r="U144" t="str">
+        <x:v>rewards</x:v>
+      </x:c>
+      <x:c r="V144" t="str">
+        <x:v>feature/android-rewards</x:v>
+      </x:c>
+      <x:c r="W144" t="str">
+        <x:v>DoR PASS: Rewards frontend/mock contract approved; Backend no requerido para implementación frontend-first.</x:v>
+      </x:c>
+      <x:c r="X144"/>
+      <x:c r="Y144"/>
+      <x:c r="Z144"/>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" t="str">
+        <x:v>IMP-AND-0302</x:v>
+      </x:c>
+      <x:c r="B145" t="str">
+        <x:v>S3 Android Loyalty</x:v>
+      </x:c>
+      <x:c r="C145" t="str">
+        <x:v>ANDROID</x:v>
+      </x:c>
+      <x:c r="D145" t="str">
+        <x:v>Promociones</x:v>
+      </x:c>
+      <x:c r="E145" t="str">
+        <x:v>ANDROID-1</x:v>
+      </x:c>
+      <x:c r="F145" t="str">
+        <x:v>WEB-2</x:v>
+      </x:c>
+      <x:c r="G145" t="str">
+        <x:v>promotions</x:v>
+      </x:c>
+      <x:c r="H145" t="str">
+        <x:v>FEATURE</x:v>
+      </x:c>
+      <x:c r="I145" t="str">
+        <x:v>ALTA</x:v>
+      </x:c>
+      <x:c r="J145" t="str">
+        <x:v>READY</x:v>
+      </x:c>
+      <x:c r="K145" t="str">
+        <x:v>IMP-AND-0009</x:v>
+      </x:c>
+      <x:c r="L145" t="str">
+        <x:v>Android 03 Loyalty, promociones y perfil</x:v>
+      </x:c>
+      <x:c r="M145" t="str">
+        <x:v>238:132</x:v>
+      </x:c>
+      <x:c r="N145" t="str">
+        <x:v>Promotions</x:v>
+      </x:c>
+      <x:c r="O145" t="str">
+        <x:v>Implementar Promotions</x:v>
+      </x:c>
+      <x:c r="P145" t="str">
+        <x:v>Eligibility/vigencia/stacking reason; states.</x:v>
+      </x:c>
+      <x:c r="Q145" t="str">
+        <x:v>Incompatible no combinable; reasons correct.</x:v>
+      </x:c>
+      <x:c r="R145" t="str">
+        <x:v>Promotions frontend/mock contract approved.</x:v>
+      </x:c>
+      <x:c r="S145" t="str">
+        <x:v>Mapper + UI.</x:v>
+      </x:c>
+      <x:c r="T145" t="str">
+        <x:v>unit/ui</x:v>
+      </x:c>
+      <x:c r="U145" t="str">
+        <x:v>promotions</x:v>
+      </x:c>
+      <x:c r="V145" t="str">
+        <x:v>feature/android-promotions</x:v>
+      </x:c>
+      <x:c r="W145" t="str">
+        <x:v>DoR PASS: Promotions frontend/mock contract approved; Backend no requerido para implementación frontend-first.</x:v>
+      </x:c>
+      <x:c r="X145"/>
+      <x:c r="Y145"/>
+      <x:c r="Z145"/>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" t="str">
+        <x:v>IMP-AND-0303</x:v>
+      </x:c>
+      <x:c r="B146" t="str">
+        <x:v>S3 Android Loyalty</x:v>
+      </x:c>
+      <x:c r="C146" t="str">
+        <x:v>ANDROID</x:v>
+      </x:c>
+      <x:c r="D146" t="str">
+        <x:v>Perfil</x:v>
+      </x:c>
+      <x:c r="E146" t="str">
+        <x:v>ANDROID-1</x:v>
+      </x:c>
+      <x:c r="F146" t="str">
+        <x:v>WEB-2</x:v>
+      </x:c>
+      <x:c r="G146" t="str">
+        <x:v>profile</x:v>
+      </x:c>
+      <x:c r="H146" t="str">
+        <x:v>FEATURE</x:v>
+      </x:c>
+      <x:c r="I146" t="str">
+        <x:v>ALTA</x:v>
+      </x:c>
+      <x:c r="J146" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="K146" t="str">
+        <x:v>IMP-AND-0201</x:v>
+      </x:c>
+      <x:c r="L146" t="str">
+        <x:v>Android 03 Loyalty, promociones y perfil</x:v>
+      </x:c>
+      <x:c r="M146" t="str">
+        <x:v>238:132</x:v>
+      </x:c>
+      <x:c r="N146" t="str">
+        <x:v>Profile</x:v>
+      </x:c>
+      <x:c r="O146" t="str">
+        <x:v>Implementar perfil final</x:v>
+      </x:c>
+      <x:c r="P146" t="str">
+        <x:v>Figma layout/edit/states; reuse Account/Profile Domain.</x:v>
+      </x:c>
+      <x:c r="Q146" t="str">
+        <x:v>No duplicated model; PII safe; save states correct.</x:v>
+      </x:c>
+      <x:c r="R146" t="str">
+        <x:v>IMP-AND-0201 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
+      </x:c>
+      <x:c r="S146" t="str">
+        <x:v>UI tests.</x:v>
+      </x:c>
+      <x:c r="T146" t="str">
+        <x:v>unit/ui</x:v>
+      </x:c>
+      <x:c r="U146" t="str">
+        <x:v>profile</x:v>
+      </x:c>
+      <x:c r="V146" t="str">
+        <x:v>feature/android-profile</x:v>
+      </x:c>
+      <x:c r="W146"/>
+      <x:c r="X146"/>
+      <x:c r="Y146"/>
+      <x:c r="Z146"/>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" t="str">
+        <x:v>IMP-AND-0304</x:v>
+      </x:c>
+      <x:c r="B147" t="str">
+        <x:v>S3 Android Loyalty</x:v>
+      </x:c>
+      <x:c r="C147" t="str">
+        <x:v>ANDROID</x:v>
+      </x:c>
+      <x:c r="D147" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="E147" t="str">
+        <x:v>ANDROID-1</x:v>
+      </x:c>
+      <x:c r="F147" t="str">
+        <x:v>WEB-2</x:v>
+      </x:c>
+      <x:c r="G147" t="str">
+        <x:v>loyalty-profile</x:v>
+      </x:c>
+      <x:c r="H147" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="I147" t="str">
+        <x:v>CRÍTICA</x:v>
+      </x:c>
+      <x:c r="J147" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="K147" t="str">
+        <x:v>IMP-AND-0301, IMP-AND-0302, IMP-AND-0303</x:v>
+      </x:c>
+      <x:c r="L147" t="str">
+        <x:v>Android 03 Loyalty, promociones y perfil</x:v>
+      </x:c>
+      <x:c r="M147" t="str">
+        <x:v>238:132</x:v>
+      </x:c>
+      <x:c r="N147" t="str">
+        <x:v>Rewards/Promos/Profile</x:v>
+      </x:c>
+      <x:c r="O147" t="str">
+        <x:v>QA Loyalty/Profile</x:v>
+      </x:c>
+      <x:c r="P147" t="str">
+        <x:v>Rewards/promotions/profile/offline/error/empty/navigation.</x:v>
+      </x:c>
+      <x:c r="Q147" t="str">
+        <x:v>Cross-app semantics PASS; Figma parity; no DTO UI.</x:v>
+      </x:c>
+      <x:c r="R147" t="str">
+        <x:v>S3 done.</x:v>
+      </x:c>
+      <x:c r="S147" t="str">
+        <x:v>Android Global DoD.</x:v>
+      </x:c>
+      <x:c r="T147" t="str">
+        <x:v>build/tests/manual</x:v>
+      </x:c>
+      <x:c r="U147" t="str">
+        <x:v>Android S3</x:v>
+      </x:c>
+      <x:c r="V147" t="str">
+        <x:v>test/android-loyalty</x:v>
+      </x:c>
+      <x:c r="W147"/>
+      <x:c r="X147"/>
+      <x:c r="Y147"/>
+      <x:c r="Z147"/>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" t="str">
+        <x:v>IMP-AND-0401</x:v>
+      </x:c>
+      <x:c r="B148" t="str">
+        <x:v>S4 Android Release</x:v>
+      </x:c>
+      <x:c r="C148" t="str">
+        <x:v>ANDROID</x:v>
+      </x:c>
+      <x:c r="D148" t="str">
+        <x:v>Estados</x:v>
+      </x:c>
+      <x:c r="E148" t="str">
+        <x:v>ANDROID-1</x:v>
+      </x:c>
+      <x:c r="F148" t="str">
+        <x:v>WEB-2</x:v>
+      </x:c>
+      <x:c r="G148" t="str">
+        <x:v>ui-states</x:v>
+      </x:c>
+      <x:c r="H148" t="str">
+        <x:v>SHARED</x:v>
+      </x:c>
+      <x:c r="I148" t="str">
+        <x:v>CRÍTICA</x:v>
+      </x:c>
+      <x:c r="J148" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="K148" t="str">
+        <x:v>IMP-AND-0009</x:v>
+      </x:c>
+      <x:c r="L148" t="str">
+        <x:v>Android 04 Loading, error y offline</x:v>
+      </x:c>
+      <x:c r="M148" t="str">
+        <x:v>238:132</x:v>
+      </x:c>
+      <x:c r="N148" t="str">
+        <x:v>Universal States</x:v>
+      </x:c>
+      <x:c r="O148" t="str">
+        <x:v>Implementar Loading/Error/Empty/Offline shared</x:v>
+      </x:c>
+      <x:c r="P148" t="str">
+        <x:v>Reusable state UI; retry callback; accessible; no business logic.</x:v>
+      </x:c>
+      <x:c r="Q148" t="str">
+        <x:v>Features reutilizan states; offline explicit; retry actionable.</x:v>
+      </x:c>
+      <x:c r="R148" t="str">
+        <x:v>Figma states reviewed.</x:v>
+      </x:c>
+      <x:c r="S148" t="str">
+        <x:v>UI tests.</x:v>
+      </x:c>
+      <x:c r="T148" t="str">
+        <x:v>ui</x:v>
+      </x:c>
+      <x:c r="U148" t="str">
+        <x:v>shared state UI</x:v>
+      </x:c>
+      <x:c r="V148" t="str">
+        <x:v>feature/android-universal-states</x:v>
+      </x:c>
+      <x:c r="W148"/>
+      <x:c r="X148"/>
+      <x:c r="Y148"/>
+      <x:c r="Z148"/>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" t="str">
+        <x:v>IMP-AND-0402</x:v>
+      </x:c>
+      <x:c r="B149" t="str">
+        <x:v>S4 Android Release</x:v>
+      </x:c>
+      <x:c r="C149" t="str">
+        <x:v>ANDROID</x:v>
+      </x:c>
+      <x:c r="D149" t="str">
+        <x:v>Estados</x:v>
+      </x:c>
+      <x:c r="E149" t="str">
+        <x:v>ANDROID-1</x:v>
+      </x:c>
+      <x:c r="F149" t="str">
+        <x:v>WEB-3</x:v>
+      </x:c>
+      <x:c r="G149" t="str">
+        <x:v>offline</x:v>
+      </x:c>
+      <x:c r="H149" t="str">
+        <x:v>FEATURE</x:v>
+      </x:c>
+      <x:c r="I149" t="str">
+        <x:v>CRÍTICA</x:v>
+      </x:c>
+      <x:c r="J149" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="K149" t="str">
+        <x:v>IMP-AND-0401, IMP-AND-0106, IMP-AND-0204, IMP-AND-0304</x:v>
+      </x:c>
+      <x:c r="L149" t="str">
+        <x:v>Android 04 Loading, error y offline</x:v>
+      </x:c>
+      <x:c r="M149" t="str">
+        <x:v>238:132</x:v>
+      </x:c>
+      <x:c r="N149" t="str">
+        <x:v>All</x:v>
+      </x:c>
+      <x:c r="O149" t="str">
+        <x:v>Integrar states universales</x:v>
+      </x:c>
+      <x:c r="P149" t="str">
+        <x:v>Reemplazar estados ad-hoc; retry; stale indication donde aplica.</x:v>
+      </x:c>
+      <x:c r="Q149" t="str">
+        <x:v>0 remote screen sin Loading/Error; Offline según Figma; no false success.</x:v>
+      </x:c>
+      <x:c r="R149" t="str">
+        <x:v>Feature screens done.</x:v>
+      </x:c>
+      <x:c r="S149" t="str">
+        <x:v>Regression states.</x:v>
+      </x:c>
+      <x:c r="T149" t="str">
+        <x:v>ui/manual</x:v>
+      </x:c>
+      <x:c r="U149" t="str">
+        <x:v>all Android</x:v>
+      </x:c>
+      <x:c r="V149" t="str">
+        <x:v>feature/android-state-integration</x:v>
+      </x:c>
+      <x:c r="W149"/>
+      <x:c r="X149"/>
+      <x:c r="Y149"/>
+      <x:c r="Z149"/>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" t="str">
+        <x:v>IMP-AND-0403</x:v>
+      </x:c>
+      <x:c r="B150" t="str">
+        <x:v>S4 Android Release</x:v>
+      </x:c>
+      <x:c r="C150" t="str">
+        <x:v>ANDROID</x:v>
+      </x:c>
+      <x:c r="D150" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="E150" t="str">
+        <x:v>ANDROID-1</x:v>
+      </x:c>
+      <x:c r="F150" t="str">
+        <x:v>WEB-2</x:v>
+      </x:c>
+      <x:c r="G150" t="str">
+        <x:v>accessibility</x:v>
+      </x:c>
+      <x:c r="H150" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="I150" t="str">
+        <x:v>CRÍTICA</x:v>
+      </x:c>
+      <x:c r="J150" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="K150" t="str">
+        <x:v>IMP-AND-0402</x:v>
+      </x:c>
+      <x:c r="L150" t="str">
+        <x:v>Android final regression</x:v>
+      </x:c>
+      <x:c r="M150" t="str">
+        <x:v>238:132</x:v>
+      </x:c>
+      <x:c r="N150" t="str">
+        <x:v>All</x:v>
+      </x:c>
+      <x:c r="O150" t="str">
+        <x:v>Auditoría accesibilidad Android</x:v>
+      </x:c>
+      <x:c r="P150" t="str">
+        <x:v>TalkBack/labels/targets/contrast/focus/auth/errors.</x:v>
+      </x:c>
+      <x:c r="Q150" t="str">
+        <x:v>0 critical/high accessibility defects; primary journeys operable.</x:v>
+      </x:c>
+      <x:c r="R150" t="str">
+        <x:v>Features done.</x:v>
+      </x:c>
+      <x:c r="S150" t="str">
+        <x:v>A11y PASS.</x:v>
+      </x:c>
+      <x:c r="T150" t="str">
+        <x:v>manual/tooling</x:v>
+      </x:c>
+      <x:c r="U150" t="str">
+        <x:v>whole Android</x:v>
+      </x:c>
+      <x:c r="V150" t="str">
+        <x:v>test/android-a11y</x:v>
+      </x:c>
+      <x:c r="W150"/>
+      <x:c r="X150"/>
+      <x:c r="Y150"/>
+      <x:c r="Z150"/>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151"/>
+      <x:c r="B151"/>
+      <x:c r="C151"/>
+      <x:c r="D151"/>
+      <x:c r="E151"/>
+      <x:c r="F151"/>
+      <x:c r="G151"/>
+      <x:c r="H151"/>
+      <x:c r="I151"/>
+      <x:c r="J151"/>
+      <x:c r="K151"/>
+      <x:c r="L151"/>
+      <x:c r="M151"/>
+      <x:c r="N151"/>
+      <x:c r="O151"/>
+      <x:c r="P151"/>
+      <x:c r="Q151"/>
+      <x:c r="R151"/>
+      <x:c r="S151"/>
+      <x:c r="T151"/>
+      <x:c r="U151"/>
+      <x:c r="V151"/>
+      <x:c r="W151"/>
+      <x:c r="X151"/>
+      <x:c r="Y151"/>
+      <x:c r="Z151"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="J2:J142">
@@ -11354,7 +11894,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7f617e8a72e489c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94603eacc9674bf4"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(android): add account stay hub
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="Rd7a7326eee72480b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="Ra4d691e2273c4750"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R7334b3f39bba4fa9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="Re331cf68db824811"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R738bb23a3b09480b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="Rc29636f4ff364216"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="Rf691f4a8d3154469"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R56c7217556a54047"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R5db3950fd0534926"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R98de94fc11b740b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R0e7b2d66a2314c9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R0fcac7f181f8400e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc827b7375ffe4780"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0cdad5b969064b4a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -804,7 +804,7 @@
       </x:c>
       <x:c r="B6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_PROGRESO")</x:f>
@@ -820,7 +820,7 @@
       </x:c>
       <x:c r="F6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -888,7 +888,7 @@
       </x:c>
       <x:c r="G11" t="n">
         <x:f>COUNTIFS('01_Backlog'!C2:C142,E11,'01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -927,7 +927,7 @@
       </x:c>
       <x:c r="C14" s="12" t="n">
         <x:f>COUNTIFS('01_Backlog'!E2:E142,A14,'01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f82350207b24f3e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fc7866a04874f6d"/>
 </x:worksheet>
 </file>
 
@@ -10610,16 +10610,16 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J134" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K134" s="14" t="str">
         <x:v>IMP-AND-0107</x:v>
       </x:c>
       <x:c r="L134" s="14" t="str">
-        <x:v>Android Early Journey → V3</x:v>
+        <x:v>Android V3 Account / Stay Hub</x:v>
       </x:c>
       <x:c r="M134" s="14" t="str">
-        <x:v>31:154 / 238:132</x:v>
+        <x:v>1839:410 / 1839:411 / 1839:443 / 1839:458 / 1839:473</x:v>
       </x:c>
       <x:c r="N134" s="14" t="str">
         <x:v>MOB-20 /account</x:v>
@@ -10634,7 +10634,7 @@
         <x:v>No quinta tab ni segundo hub /account.</x:v>
       </x:c>
       <x:c r="R134" s="14" t="str">
-        <x:v>IMP-AND-0107 COMPLETADA; Figma/contrato frontend/mock READY.</x:v>
+        <x:v>IMP-AND-0107 COMPLETADA; Figma 1839:410 y estados aprobados; 24_ACCOUNT_STAY_HUB_CONTRACT.md APPROVED.</x:v>
       </x:c>
       <x:c r="S134" s="14" t="str">
         <x:v>UI tests</x:v>
@@ -10649,7 +10649,7 @@
         <x:v>feature/android-account-stay-hub</x:v>
       </x:c>
       <x:c r="W134" s="14" t="str">
-        <x:v>PENDIENTE: implementa primero el destino /account y el Account / Stay Hub V3 requerido para el post-success validable de IMP-AND-0108.</x:v>
+        <x:v>COMPLETADA: /account implementado como Account / Stay Hub V3 canónico. Cuenta enabled y activa en /account y /account/*; StayHomeScreen y footer V1 retirados; root → /account. Reutiliza ReservationStay. Base/Loading/Error/Offline/retry y room nullable cubiertos. REMOTE_STATUS crudo no visible en UI; status preservado opaco en dominio. QA manual PASS; WEB-2 PASS; lint PASS; typecheck PASS; Expo Doctor 21/21 PASS; test 12 suites / 65 tests PASS; Android export PASS; npm run check PASS; git diff --check PASS.</x:v>
       </x:c>
       <x:c r="X134" s="14"/>
       <x:c r="Y134" s="14"/>
@@ -11017,16 +11017,16 @@
     </x:row>
     <x:row r="140" ht="84" customHeight="1">
       <x:c r="A140" s="14" t="str">
-        <x:v>IMP-AND-0201</x:v>
+        <x:v>IMP-AND-0115</x:v>
       </x:c>
       <x:c r="B140" s="14" t="str">
-        <x:v>S2 Android Account</x:v>
+        <x:v>S1 Android Stay &amp; Services</x:v>
       </x:c>
       <x:c r="C140" s="14" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D140" s="14" t="str">
-        <x:v>Cuenta</x:v>
+        <x:v>Cuenta / Actividad de la estadía</x:v>
       </x:c>
       <x:c r="E140" s="14" t="str">
         <x:v>ANDROID-1</x:v>
@@ -11041,57 +11041,57 @@
         <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I140" s="14" t="str">
-        <x:v>CRÍTICA</x:v>
+        <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J140" s="14" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K140" s="14" t="str">
-        <x:v>IMP-AND-0009, IMP-AND-0109</x:v>
+        <x:v>IMP-AND-0109, IMP-AND-0112, IMP-AND-0105</x:v>
       </x:c>
       <x:c r="L140" s="14" t="str">
-        <x:v>Android 02 Cuenta, checkout y factura</x:v>
-      </x:c>
-      <x:c r="M140" s="14" t="str">
-        <x:v>238:132</x:v>
-      </x:c>
+        <x:v>Pendiente de fuente visual aprobada</x:v>
+      </x:c>
+      <x:c r="M140" s="14"/>
       <x:c r="N140" s="14" t="str">
-        <x:v>Account</x:v>
+        <x:v>Account / actividad</x:v>
       </x:c>
       <x:c r="O140" s="14" t="str">
-        <x:v>Crear Account/Profile contracts</x:v>
+        <x:v>Extender Account / Stay Hub con resumen de actividad de la estadía</x:v>
       </x:c>
       <x:c r="P140" s="14" t="str">
-        <x:v>GuestAccount/Profile separados; extiende Account / Stay Hub existente; no duplica /account.</x:v>
+        <x:v>Definir frontera agregada de actividad antes de UI; incluir solicitudes de servicios, housekeeping, room service, valet y traslados solo cuando corresponda.</x:v>
       </x:c>
       <x:c r="Q140" s="14" t="str">
-        <x:v>No Staff auth; no provider JSON UI; mapper tests; sin segundo hub /account.</x:v>
+        <x:v>Account no es owner de Services ni Valet; UI no consume DTOs ni fixtures directos de esos módulos.</x:v>
       </x:c>
       <x:c r="R140" s="14" t="str">
-        <x:v>IMP-AND-0109 COMPLETADA; Sprint 0 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
+        <x:v>IMP-AND-0109, IMP-AND-0112 e IMP-AND-0105 COMPLETADA; fuente visual y frontera agregada de actividad aprobadas.</x:v>
       </x:c>
       <x:c r="S140" s="14" t="str">
-        <x:v>Unit.</x:v>
+        <x:v>Contrato agregado, tests y UI PASS; sin duplicar dominios ni consumir DTOs/fixtures de Services o Valet.</x:v>
       </x:c>
       <x:c r="T140" s="14" t="str">
-        <x:v>unit</x:v>
+        <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U140" s="14" t="str">
-        <x:v>account layers</x:v>
+        <x:v>account activity aggregate</x:v>
       </x:c>
       <x:c r="V140" s="14" t="str">
-        <x:v>feature/android-account-contract</x:v>
+        <x:v>feature/android-account-stay-activity</x:v>
       </x:c>
       <x:c r="W140" s="14" t="str">
-        <x:v>PENDIENTE: IMP-AND-0109 debe completar el Account / Stay Hub en /account. Account/Profile lo extiende sin crear un segundo hub ni duplicar la ruta.</x:v>
+        <x:v>PENDIENTE: no implementada. Debe ejecutarse después de las capacidades base de solicitudes de Services.</x:v>
       </x:c>
       <x:c r="X140" s="14"/>
       <x:c r="Y140" s="14"/>
-      <x:c r="Z140" s="14"/>
+      <x:c r="Z140" s="14" t="str">
+        <x:v>No iniciar sin fuente visual y contrato agregado aprobados.</x:v>
+      </x:c>
     </x:row>
     <x:row r="141" ht="84" customHeight="1">
       <x:c r="A141" s="14" t="str">
-        <x:v>IMP-AND-0202</x:v>
+        <x:v>IMP-AND-0201</x:v>
       </x:c>
       <x:c r="B141" s="14" t="str">
         <x:v>S2 Android Account</x:v>
@@ -11115,13 +11115,13 @@
         <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I141" s="14" t="str">
-        <x:v>ALTA</x:v>
+        <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J141" s="14" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K141" s="14" t="str">
-        <x:v>IMP-AND-0201</x:v>
+        <x:v>IMP-AND-0009, IMP-AND-0109</x:v>
       </x:c>
       <x:c r="L141" s="14" t="str">
         <x:v>Android 02 Cuenta, checkout y factura</x:v>
@@ -11130,40 +11130,42 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N141" s="14" t="str">
-        <x:v>Account/Profile</x:v>
+        <x:v>Account</x:v>
       </x:c>
       <x:c r="O141" s="14" t="str">
-        <x:v>Implementar cuenta/perfil</x:v>
+        <x:v>Crear Account/Profile contracts</x:v>
       </x:c>
       <x:c r="P141" s="14" t="str">
-        <x:v>Display/edit Profile; loading/error/offline; submit.</x:v>
+        <x:v>GuestAccount/Profile separados; extiende Account / Stay Hub existente; no duplica /account.</x:v>
       </x:c>
       <x:c r="Q141" s="14" t="str">
-        <x:v>Account/Profile separation; no secrets; save states correct.</x:v>
+        <x:v>No Staff auth; no provider JSON UI; mapper tests; sin segundo hub /account.</x:v>
       </x:c>
       <x:c r="R141" s="14" t="str">
-        <x:v>IMP-AND-0201 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
+        <x:v>IMP-AND-0109 COMPLETADA; Sprint 0 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S141" s="14" t="str">
-        <x:v>UI tests.</x:v>
+        <x:v>Unit.</x:v>
       </x:c>
       <x:c r="T141" s="14" t="str">
-        <x:v>unit/ui</x:v>
+        <x:v>unit</x:v>
       </x:c>
       <x:c r="U141" s="14" t="str">
-        <x:v>account/profile screens</x:v>
+        <x:v>account layers</x:v>
       </x:c>
       <x:c r="V141" s="14" t="str">
-        <x:v>feature/android-account-profile</x:v>
-      </x:c>
-      <x:c r="W141" s="14"/>
+        <x:v>feature/android-account-contract</x:v>
+      </x:c>
+      <x:c r="W141" s="14" t="str">
+        <x:v>PENDIENTE: IMP-AND-0109 debe completar el Account / Stay Hub en /account. Account/Profile lo extiende sin crear un segundo hub ni duplicar la ruta.</x:v>
+      </x:c>
       <x:c r="X141" s="14"/>
       <x:c r="Y141" s="14"/>
       <x:c r="Z141" s="14"/>
     </x:row>
     <x:row r="142" ht="84" customHeight="1">
       <x:c r="A142" s="14" t="str">
-        <x:v>IMP-AND-0203</x:v>
+        <x:v>IMP-AND-0202</x:v>
       </x:c>
       <x:c r="B142" s="14" t="str">
         <x:v>S2 Android Account</x:v>
@@ -11172,28 +11174,28 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D142" s="14" t="str">
-        <x:v>Checkout/Factura</x:v>
+        <x:v>Cuenta</x:v>
       </x:c>
       <x:c r="E142" s="14" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F142" s="14" t="str">
-        <x:v>WEB-4</x:v>
+        <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G142" s="14" t="str">
-        <x:v>checkout</x:v>
+        <x:v>account</x:v>
       </x:c>
       <x:c r="H142" s="14" t="str">
         <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I142" s="14" t="str">
-        <x:v>CRÍTICA</x:v>
+        <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J142" s="14" t="str">
-        <x:v>READY</x:v>
+        <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K142" s="14" t="str">
-        <x:v>IMP-AND-0102</x:v>
+        <x:v>IMP-AND-0201</x:v>
       </x:c>
       <x:c r="L142" s="14" t="str">
         <x:v>Android 02 Cuenta, checkout y factura</x:v>
@@ -11202,42 +11204,40 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N142" s="14" t="str">
-        <x:v>Checkout/Invoice</x:v>
+        <x:v>Account/Profile</x:v>
       </x:c>
       <x:c r="O142" s="14" t="str">
-        <x:v>Implementar checkout e invoice</x:v>
+        <x:v>Implementar cuenta/perfil</x:v>
       </x:c>
       <x:c r="P142" s="14" t="str">
-        <x:v>Charges/balance/status Folio read model; invoice ref/status/date/total; offline/error.</x:v>
+        <x:v>Display/edit Profile; loading/error/offline; submit.</x:v>
       </x:c>
       <x:c r="Q142" s="14" t="str">
-        <x:v>Finance no recalculated in UI; no sensitive file persisted; no provider raw data.</x:v>
+        <x:v>Account/Profile separation; no secrets; save states correct.</x:v>
       </x:c>
       <x:c r="R142" s="14" t="str">
-        <x:v>Checkout/Folio frontend/mock contract approved; representación simulada/frontend únicamente hasta integración Backend/fiscal.</x:v>
+        <x:v>IMP-AND-0201 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S142" s="14" t="str">
-        <x:v>Mapper + UI/security.</x:v>
+        <x:v>UI tests.</x:v>
       </x:c>
       <x:c r="T142" s="14" t="str">
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U142" s="14" t="str">
-        <x:v>checkout/invoice</x:v>
+        <x:v>account/profile screens</x:v>
       </x:c>
       <x:c r="V142" s="14" t="str">
-        <x:v>feature/android-checkout-invoice</x:v>
-      </x:c>
-      <x:c r="W142" s="14" t="str">
-        <x:v>DoR PASS: Checkout/Folio frontend/mock contract approved; implementación frontend simulada únicamente. No implica pago real, factura fiscal real ni integración FEL/SAT; Backend/fiscal se integra posteriormente.</x:v>
-      </x:c>
+        <x:v>feature/android-account-profile</x:v>
+      </x:c>
+      <x:c r="W142" s="14"/>
       <x:c r="X142" s="14"/>
       <x:c r="Y142" s="14"/>
       <x:c r="Z142" s="14"/>
     </x:row>
     <x:row r="143">
       <x:c r="A143" t="str">
-        <x:v>IMP-AND-0204</x:v>
+        <x:v>IMP-AND-0203</x:v>
       </x:c>
       <x:c r="B143" t="str">
         <x:v>S2 Android Account</x:v>
@@ -11246,28 +11246,28 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D143" t="str">
-        <x:v>QA</x:v>
+        <x:v>Checkout/Factura</x:v>
       </x:c>
       <x:c r="E143" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F143" t="str">
-        <x:v>WEB-2</x:v>
+        <x:v>WEB-4</x:v>
       </x:c>
       <x:c r="G143" t="str">
-        <x:v>account-checkout</x:v>
+        <x:v>checkout</x:v>
       </x:c>
       <x:c r="H143" t="str">
-        <x:v>QA</x:v>
+        <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I143" t="str">
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J143" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>READY</x:v>
       </x:c>
       <x:c r="K143" t="str">
-        <x:v>IMP-AND-0202, IMP-AND-0203</x:v>
+        <x:v>IMP-AND-0102</x:v>
       </x:c>
       <x:c r="L143" t="str">
         <x:v>Android 02 Cuenta, checkout y factura</x:v>
@@ -11276,49 +11276,51 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N143" t="str">
-        <x:v>Account/Checkout</x:v>
+        <x:v>Checkout/Invoice</x:v>
       </x:c>
       <x:c r="O143" t="str">
-        <x:v>QA Cuenta/Checkout/Factura</x:v>
+        <x:v>Implementar checkout e invoice</x:v>
       </x:c>
       <x:c r="P143" t="str">
-        <x:v>Profile/checkout/invoice/states/navigation/contracts.</x:v>
+        <x:v>Charges/balance/status Folio read model; invoice ref/status/date/total; offline/error.</x:v>
       </x:c>
       <x:c r="Q143" t="str">
-        <x:v>Guest/Staff separation; finance coherent; Figma parity.</x:v>
+        <x:v>Finance no recalculated in UI; no sensitive file persisted; no provider raw data.</x:v>
       </x:c>
       <x:c r="R143" t="str">
-        <x:v>S2 done.</x:v>
+        <x:v>Checkout/Folio frontend/mock contract approved; representación simulada/frontend únicamente hasta integración Backend/fiscal.</x:v>
       </x:c>
       <x:c r="S143" t="str">
-        <x:v>Android Global DoD.</x:v>
+        <x:v>Mapper + UI/security.</x:v>
       </x:c>
       <x:c r="T143" t="str">
-        <x:v>build/tests/manual</x:v>
+        <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U143" t="str">
-        <x:v>Android S2</x:v>
+        <x:v>checkout/invoice</x:v>
       </x:c>
       <x:c r="V143" t="str">
-        <x:v>test/android-account-checkout</x:v>
-      </x:c>
-      <x:c r="W143"/>
+        <x:v>feature/android-checkout-invoice</x:v>
+      </x:c>
+      <x:c r="W143" t="str">
+        <x:v>DoR PASS: Checkout/Folio frontend/mock contract approved; implementación frontend simulada únicamente. No implica pago real, factura fiscal real ni integración FEL/SAT; Backend/fiscal se integra posteriormente.</x:v>
+      </x:c>
       <x:c r="X143"/>
       <x:c r="Y143"/>
       <x:c r="Z143"/>
     </x:row>
     <x:row r="144">
       <x:c r="A144" t="str">
-        <x:v>IMP-AND-0301</x:v>
+        <x:v>IMP-AND-0204</x:v>
       </x:c>
       <x:c r="B144" t="str">
-        <x:v>S3 Android Loyalty</x:v>
+        <x:v>S2 Android Account</x:v>
       </x:c>
       <x:c r="C144" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D144" t="str">
-        <x:v>Loyalty</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="E144" t="str">
         <x:v>ANDROID-1</x:v>
@@ -11327,63 +11329,61 @@
         <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G144" t="str">
-        <x:v>rewards</x:v>
+        <x:v>account-checkout</x:v>
       </x:c>
       <x:c r="H144" t="str">
-        <x:v>FEATURE</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="I144" t="str">
-        <x:v>ALTA</x:v>
+        <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J144" t="str">
-        <x:v>READY</x:v>
+        <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K144" t="str">
-        <x:v>IMP-AND-0009</x:v>
+        <x:v>IMP-AND-0202, IMP-AND-0203</x:v>
       </x:c>
       <x:c r="L144" t="str">
-        <x:v>Android 03 Loyalty, promociones y perfil</x:v>
+        <x:v>Android 02 Cuenta, checkout y factura</x:v>
       </x:c>
       <x:c r="M144" t="str">
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N144" t="str">
-        <x:v>Rewards</x:v>
+        <x:v>Account/Checkout</x:v>
       </x:c>
       <x:c r="O144" t="str">
-        <x:v>Implementar Rewards</x:v>
+        <x:v>QA Cuenta/Checkout/Factura</x:v>
       </x:c>
       <x:c r="P144" t="str">
-        <x:v>Ledger/balance Domain cross-app; offline/error/empty.</x:v>
+        <x:v>Profile/checkout/invoice/states/navigation/contracts.</x:v>
       </x:c>
       <x:c r="Q144" t="str">
-        <x:v>CANCELLED/NO_SHOW no elegibles; ledger read-only.</x:v>
+        <x:v>Guest/Staff separation; finance coherent; Figma parity.</x:v>
       </x:c>
       <x:c r="R144" t="str">
-        <x:v>Rewards frontend/mock contract approved.</x:v>
+        <x:v>S2 done.</x:v>
       </x:c>
       <x:c r="S144" t="str">
-        <x:v>Mapper + UI.</x:v>
+        <x:v>Android Global DoD.</x:v>
       </x:c>
       <x:c r="T144" t="str">
-        <x:v>unit/ui</x:v>
+        <x:v>build/tests/manual</x:v>
       </x:c>
       <x:c r="U144" t="str">
-        <x:v>rewards</x:v>
+        <x:v>Android S2</x:v>
       </x:c>
       <x:c r="V144" t="str">
-        <x:v>feature/android-rewards</x:v>
-      </x:c>
-      <x:c r="W144" t="str">
-        <x:v>DoR PASS: Rewards frontend/mock contract approved; Backend no requerido para implementación frontend-first.</x:v>
-      </x:c>
+        <x:v>test/android-account-checkout</x:v>
+      </x:c>
+      <x:c r="W144"/>
       <x:c r="X144"/>
       <x:c r="Y144"/>
       <x:c r="Z144"/>
     </x:row>
     <x:row r="145">
       <x:c r="A145" t="str">
-        <x:v>IMP-AND-0302</x:v>
+        <x:v>IMP-AND-0301</x:v>
       </x:c>
       <x:c r="B145" t="str">
         <x:v>S3 Android Loyalty</x:v>
@@ -11392,7 +11392,7 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D145" t="str">
-        <x:v>Promociones</x:v>
+        <x:v>Loyalty</x:v>
       </x:c>
       <x:c r="E145" t="str">
         <x:v>ANDROID-1</x:v>
@@ -11401,7 +11401,7 @@
         <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G145" t="str">
-        <x:v>promotions</x:v>
+        <x:v>rewards</x:v>
       </x:c>
       <x:c r="H145" t="str">
         <x:v>FEATURE</x:v>
@@ -11422,19 +11422,19 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N145" t="str">
-        <x:v>Promotions</x:v>
+        <x:v>Rewards</x:v>
       </x:c>
       <x:c r="O145" t="str">
-        <x:v>Implementar Promotions</x:v>
+        <x:v>Implementar Rewards</x:v>
       </x:c>
       <x:c r="P145" t="str">
-        <x:v>Eligibility/vigencia/stacking reason; states.</x:v>
+        <x:v>Ledger/balance Domain cross-app; offline/error/empty.</x:v>
       </x:c>
       <x:c r="Q145" t="str">
-        <x:v>Incompatible no combinable; reasons correct.</x:v>
+        <x:v>CANCELLED/NO_SHOW no elegibles; ledger read-only.</x:v>
       </x:c>
       <x:c r="R145" t="str">
-        <x:v>Promotions frontend/mock contract approved.</x:v>
+        <x:v>Rewards frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S145" t="str">
         <x:v>Mapper + UI.</x:v>
@@ -11443,13 +11443,13 @@
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U145" t="str">
-        <x:v>promotions</x:v>
+        <x:v>rewards</x:v>
       </x:c>
       <x:c r="V145" t="str">
-        <x:v>feature/android-promotions</x:v>
+        <x:v>feature/android-rewards</x:v>
       </x:c>
       <x:c r="W145" t="str">
-        <x:v>DoR PASS: Promotions frontend/mock contract approved; Backend no requerido para implementación frontend-first.</x:v>
+        <x:v>DoR PASS: Rewards frontend/mock contract approved; Backend no requerido para implementación frontend-first.</x:v>
       </x:c>
       <x:c r="X145"/>
       <x:c r="Y145"/>
@@ -11457,7 +11457,7 @@
     </x:row>
     <x:row r="146">
       <x:c r="A146" t="str">
-        <x:v>IMP-AND-0303</x:v>
+        <x:v>IMP-AND-0302</x:v>
       </x:c>
       <x:c r="B146" t="str">
         <x:v>S3 Android Loyalty</x:v>
@@ -11466,7 +11466,7 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D146" t="str">
-        <x:v>Perfil</x:v>
+        <x:v>Promociones</x:v>
       </x:c>
       <x:c r="E146" t="str">
         <x:v>ANDROID-1</x:v>
@@ -11475,7 +11475,7 @@
         <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G146" t="str">
-        <x:v>profile</x:v>
+        <x:v>promotions</x:v>
       </x:c>
       <x:c r="H146" t="str">
         <x:v>FEATURE</x:v>
@@ -11484,10 +11484,10 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J146" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>READY</x:v>
       </x:c>
       <x:c r="K146" t="str">
-        <x:v>IMP-AND-0201</x:v>
+        <x:v>IMP-AND-0009</x:v>
       </x:c>
       <x:c r="L146" t="str">
         <x:v>Android 03 Loyalty, promociones y perfil</x:v>
@@ -11496,40 +11496,42 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N146" t="str">
-        <x:v>Profile</x:v>
+        <x:v>Promotions</x:v>
       </x:c>
       <x:c r="O146" t="str">
-        <x:v>Implementar perfil final</x:v>
+        <x:v>Implementar Promotions</x:v>
       </x:c>
       <x:c r="P146" t="str">
-        <x:v>Figma layout/edit/states; reuse Account/Profile Domain.</x:v>
+        <x:v>Eligibility/vigencia/stacking reason; states.</x:v>
       </x:c>
       <x:c r="Q146" t="str">
-        <x:v>No duplicated model; PII safe; save states correct.</x:v>
+        <x:v>Incompatible no combinable; reasons correct.</x:v>
       </x:c>
       <x:c r="R146" t="str">
-        <x:v>IMP-AND-0201 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
+        <x:v>Promotions frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S146" t="str">
-        <x:v>UI tests.</x:v>
+        <x:v>Mapper + UI.</x:v>
       </x:c>
       <x:c r="T146" t="str">
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U146" t="str">
-        <x:v>profile</x:v>
+        <x:v>promotions</x:v>
       </x:c>
       <x:c r="V146" t="str">
-        <x:v>feature/android-profile</x:v>
-      </x:c>
-      <x:c r="W146"/>
+        <x:v>feature/android-promotions</x:v>
+      </x:c>
+      <x:c r="W146" t="str">
+        <x:v>DoR PASS: Promotions frontend/mock contract approved; Backend no requerido para implementación frontend-first.</x:v>
+      </x:c>
       <x:c r="X146"/>
       <x:c r="Y146"/>
       <x:c r="Z146"/>
     </x:row>
     <x:row r="147">
       <x:c r="A147" t="str">
-        <x:v>IMP-AND-0304</x:v>
+        <x:v>IMP-AND-0303</x:v>
       </x:c>
       <x:c r="B147" t="str">
         <x:v>S3 Android Loyalty</x:v>
@@ -11538,7 +11540,7 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D147" t="str">
-        <x:v>QA</x:v>
+        <x:v>Perfil</x:v>
       </x:c>
       <x:c r="E147" t="str">
         <x:v>ANDROID-1</x:v>
@@ -11547,19 +11549,19 @@
         <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G147" t="str">
-        <x:v>loyalty-profile</x:v>
+        <x:v>profile</x:v>
       </x:c>
       <x:c r="H147" t="str">
-        <x:v>QA</x:v>
+        <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I147" t="str">
-        <x:v>CRÍTICA</x:v>
+        <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J147" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K147" t="str">
-        <x:v>IMP-AND-0301, IMP-AND-0302, IMP-AND-0303</x:v>
+        <x:v>IMP-AND-0201</x:v>
       </x:c>
       <x:c r="L147" t="str">
         <x:v>Android 03 Loyalty, promociones y perfil</x:v>
@@ -11568,31 +11570,31 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N147" t="str">
-        <x:v>Rewards/Promos/Profile</x:v>
+        <x:v>Profile</x:v>
       </x:c>
       <x:c r="O147" t="str">
-        <x:v>QA Loyalty/Profile</x:v>
+        <x:v>Implementar perfil final</x:v>
       </x:c>
       <x:c r="P147" t="str">
-        <x:v>Rewards/promotions/profile/offline/error/empty/navigation.</x:v>
+        <x:v>Figma layout/edit/states; reuse Account/Profile Domain.</x:v>
       </x:c>
       <x:c r="Q147" t="str">
-        <x:v>Cross-app semantics PASS; Figma parity; no DTO UI.</x:v>
+        <x:v>No duplicated model; PII safe; save states correct.</x:v>
       </x:c>
       <x:c r="R147" t="str">
-        <x:v>S3 done.</x:v>
+        <x:v>IMP-AND-0201 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S147" t="str">
-        <x:v>Android Global DoD.</x:v>
+        <x:v>UI tests.</x:v>
       </x:c>
       <x:c r="T147" t="str">
-        <x:v>build/tests/manual</x:v>
+        <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U147" t="str">
-        <x:v>Android S3</x:v>
+        <x:v>profile</x:v>
       </x:c>
       <x:c r="V147" t="str">
-        <x:v>test/android-loyalty</x:v>
+        <x:v>feature/android-profile</x:v>
       </x:c>
       <x:c r="W147"/>
       <x:c r="X147"/>
@@ -11601,16 +11603,16 @@
     </x:row>
     <x:row r="148">
       <x:c r="A148" t="str">
-        <x:v>IMP-AND-0401</x:v>
+        <x:v>IMP-AND-0304</x:v>
       </x:c>
       <x:c r="B148" t="str">
-        <x:v>S4 Android Release</x:v>
+        <x:v>S3 Android Loyalty</x:v>
       </x:c>
       <x:c r="C148" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D148" t="str">
-        <x:v>Estados</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="E148" t="str">
         <x:v>ANDROID-1</x:v>
@@ -11619,10 +11621,10 @@
         <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G148" t="str">
-        <x:v>ui-states</x:v>
+        <x:v>loyalty-profile</x:v>
       </x:c>
       <x:c r="H148" t="str">
-        <x:v>SHARED</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="I148" t="str">
         <x:v>CRÍTICA</x:v>
@@ -11631,40 +11633,40 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K148" t="str">
-        <x:v>IMP-AND-0009</x:v>
+        <x:v>IMP-AND-0301, IMP-AND-0302, IMP-AND-0303</x:v>
       </x:c>
       <x:c r="L148" t="str">
-        <x:v>Android 04 Loading, error y offline</x:v>
+        <x:v>Android 03 Loyalty, promociones y perfil</x:v>
       </x:c>
       <x:c r="M148" t="str">
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N148" t="str">
-        <x:v>Universal States</x:v>
+        <x:v>Rewards/Promos/Profile</x:v>
       </x:c>
       <x:c r="O148" t="str">
-        <x:v>Implementar Loading/Error/Empty/Offline shared</x:v>
+        <x:v>QA Loyalty/Profile</x:v>
       </x:c>
       <x:c r="P148" t="str">
-        <x:v>Reusable state UI; retry callback; accessible; no business logic.</x:v>
+        <x:v>Rewards/promotions/profile/offline/error/empty/navigation.</x:v>
       </x:c>
       <x:c r="Q148" t="str">
-        <x:v>Features reutilizan states; offline explicit; retry actionable.</x:v>
+        <x:v>Cross-app semantics PASS; Figma parity; no DTO UI.</x:v>
       </x:c>
       <x:c r="R148" t="str">
-        <x:v>Figma states reviewed.</x:v>
+        <x:v>S3 done.</x:v>
       </x:c>
       <x:c r="S148" t="str">
-        <x:v>UI tests.</x:v>
+        <x:v>Android Global DoD.</x:v>
       </x:c>
       <x:c r="T148" t="str">
-        <x:v>ui</x:v>
+        <x:v>build/tests/manual</x:v>
       </x:c>
       <x:c r="U148" t="str">
-        <x:v>shared state UI</x:v>
+        <x:v>Android S3</x:v>
       </x:c>
       <x:c r="V148" t="str">
-        <x:v>feature/android-universal-states</x:v>
+        <x:v>test/android-loyalty</x:v>
       </x:c>
       <x:c r="W148"/>
       <x:c r="X148"/>
@@ -11673,7 +11675,7 @@
     </x:row>
     <x:row r="149">
       <x:c r="A149" t="str">
-        <x:v>IMP-AND-0402</x:v>
+        <x:v>IMP-AND-0401</x:v>
       </x:c>
       <x:c r="B149" t="str">
         <x:v>S4 Android Release</x:v>
@@ -11688,13 +11690,13 @@
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F149" t="str">
-        <x:v>WEB-3</x:v>
+        <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G149" t="str">
-        <x:v>offline</x:v>
+        <x:v>ui-states</x:v>
       </x:c>
       <x:c r="H149" t="str">
-        <x:v>FEATURE</x:v>
+        <x:v>SHARED</x:v>
       </x:c>
       <x:c r="I149" t="str">
         <x:v>CRÍTICA</x:v>
@@ -11703,7 +11705,7 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K149" t="str">
-        <x:v>IMP-AND-0401, IMP-AND-0106, IMP-AND-0204, IMP-AND-0304</x:v>
+        <x:v>IMP-AND-0009</x:v>
       </x:c>
       <x:c r="L149" t="str">
         <x:v>Android 04 Loading, error y offline</x:v>
@@ -11712,31 +11714,31 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N149" t="str">
-        <x:v>All</x:v>
+        <x:v>Universal States</x:v>
       </x:c>
       <x:c r="O149" t="str">
-        <x:v>Integrar states universales</x:v>
+        <x:v>Implementar Loading/Error/Empty/Offline shared</x:v>
       </x:c>
       <x:c r="P149" t="str">
-        <x:v>Reemplazar estados ad-hoc; retry; stale indication donde aplica.</x:v>
+        <x:v>Reusable state UI; retry callback; accessible; no business logic.</x:v>
       </x:c>
       <x:c r="Q149" t="str">
-        <x:v>0 remote screen sin Loading/Error; Offline según Figma; no false success.</x:v>
+        <x:v>Features reutilizan states; offline explicit; retry actionable.</x:v>
       </x:c>
       <x:c r="R149" t="str">
-        <x:v>Feature screens done.</x:v>
+        <x:v>Figma states reviewed.</x:v>
       </x:c>
       <x:c r="S149" t="str">
-        <x:v>Regression states.</x:v>
+        <x:v>UI tests.</x:v>
       </x:c>
       <x:c r="T149" t="str">
-        <x:v>ui/manual</x:v>
+        <x:v>ui</x:v>
       </x:c>
       <x:c r="U149" t="str">
-        <x:v>all Android</x:v>
+        <x:v>shared state UI</x:v>
       </x:c>
       <x:c r="V149" t="str">
-        <x:v>feature/android-state-integration</x:v>
+        <x:v>feature/android-universal-states</x:v>
       </x:c>
       <x:c r="W149"/>
       <x:c r="X149"/>
@@ -11745,7 +11747,7 @@
     </x:row>
     <x:row r="150">
       <x:c r="A150" t="str">
-        <x:v>IMP-AND-0403</x:v>
+        <x:v>IMP-AND-0402</x:v>
       </x:c>
       <x:c r="B150" t="str">
         <x:v>S4 Android Release</x:v>
@@ -11754,19 +11756,19 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D150" t="str">
-        <x:v>QA</x:v>
+        <x:v>Estados</x:v>
       </x:c>
       <x:c r="E150" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F150" t="str">
-        <x:v>WEB-2</x:v>
+        <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G150" t="str">
-        <x:v>accessibility</x:v>
+        <x:v>offline</x:v>
       </x:c>
       <x:c r="H150" t="str">
-        <x:v>QA</x:v>
+        <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I150" t="str">
         <x:v>CRÍTICA</x:v>
@@ -11775,10 +11777,10 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K150" t="str">
-        <x:v>IMP-AND-0402</x:v>
+        <x:v>IMP-AND-0401, IMP-AND-0106, IMP-AND-0204, IMP-AND-0304</x:v>
       </x:c>
       <x:c r="L150" t="str">
-        <x:v>Android final regression</x:v>
+        <x:v>Android 04 Loading, error y offline</x:v>
       </x:c>
       <x:c r="M150" t="str">
         <x:v>238:132</x:v>
@@ -11787,28 +11789,28 @@
         <x:v>All</x:v>
       </x:c>
       <x:c r="O150" t="str">
-        <x:v>Auditoría accesibilidad Android</x:v>
+        <x:v>Integrar states universales</x:v>
       </x:c>
       <x:c r="P150" t="str">
-        <x:v>TalkBack/labels/targets/contrast/focus/auth/errors.</x:v>
+        <x:v>Reemplazar estados ad-hoc; retry; stale indication donde aplica.</x:v>
       </x:c>
       <x:c r="Q150" t="str">
-        <x:v>0 critical/high accessibility defects; primary journeys operable.</x:v>
+        <x:v>0 remote screen sin Loading/Error; Offline según Figma; no false success.</x:v>
       </x:c>
       <x:c r="R150" t="str">
-        <x:v>Features done.</x:v>
+        <x:v>Feature screens done.</x:v>
       </x:c>
       <x:c r="S150" t="str">
-        <x:v>A11y PASS.</x:v>
+        <x:v>Regression states.</x:v>
       </x:c>
       <x:c r="T150" t="str">
-        <x:v>manual/tooling</x:v>
+        <x:v>ui/manual</x:v>
       </x:c>
       <x:c r="U150" t="str">
-        <x:v>whole Android</x:v>
+        <x:v>all Android</x:v>
       </x:c>
       <x:c r="V150" t="str">
-        <x:v>test/android-a11y</x:v>
+        <x:v>feature/android-state-integration</x:v>
       </x:c>
       <x:c r="W150"/>
       <x:c r="X150"/>
@@ -11816,32 +11818,104 @@
       <x:c r="Z150"/>
     </x:row>
     <x:row r="151">
-      <x:c r="A151"/>
-      <x:c r="B151"/>
-      <x:c r="C151"/>
-      <x:c r="D151"/>
-      <x:c r="E151"/>
-      <x:c r="F151"/>
-      <x:c r="G151"/>
-      <x:c r="H151"/>
-      <x:c r="I151"/>
-      <x:c r="J151"/>
-      <x:c r="K151"/>
-      <x:c r="L151"/>
-      <x:c r="M151"/>
-      <x:c r="N151"/>
-      <x:c r="O151"/>
-      <x:c r="P151"/>
-      <x:c r="Q151"/>
-      <x:c r="R151"/>
-      <x:c r="S151"/>
-      <x:c r="T151"/>
-      <x:c r="U151"/>
-      <x:c r="V151"/>
+      <x:c r="A151" t="str">
+        <x:v>IMP-AND-0403</x:v>
+      </x:c>
+      <x:c r="B151" t="str">
+        <x:v>S4 Android Release</x:v>
+      </x:c>
+      <x:c r="C151" t="str">
+        <x:v>ANDROID</x:v>
+      </x:c>
+      <x:c r="D151" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="E151" t="str">
+        <x:v>ANDROID-1</x:v>
+      </x:c>
+      <x:c r="F151" t="str">
+        <x:v>WEB-2</x:v>
+      </x:c>
+      <x:c r="G151" t="str">
+        <x:v>accessibility</x:v>
+      </x:c>
+      <x:c r="H151" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="I151" t="str">
+        <x:v>CRÍTICA</x:v>
+      </x:c>
+      <x:c r="J151" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="K151" t="str">
+        <x:v>IMP-AND-0402</x:v>
+      </x:c>
+      <x:c r="L151" t="str">
+        <x:v>Android final regression</x:v>
+      </x:c>
+      <x:c r="M151" t="str">
+        <x:v>238:132</x:v>
+      </x:c>
+      <x:c r="N151" t="str">
+        <x:v>All</x:v>
+      </x:c>
+      <x:c r="O151" t="str">
+        <x:v>Auditoría accesibilidad Android</x:v>
+      </x:c>
+      <x:c r="P151" t="str">
+        <x:v>TalkBack/labels/targets/contrast/focus/auth/errors.</x:v>
+      </x:c>
+      <x:c r="Q151" t="str">
+        <x:v>0 critical/high accessibility defects; primary journeys operable.</x:v>
+      </x:c>
+      <x:c r="R151" t="str">
+        <x:v>Features done.</x:v>
+      </x:c>
+      <x:c r="S151" t="str">
+        <x:v>A11y PASS.</x:v>
+      </x:c>
+      <x:c r="T151" t="str">
+        <x:v>manual/tooling</x:v>
+      </x:c>
+      <x:c r="U151" t="str">
+        <x:v>whole Android</x:v>
+      </x:c>
+      <x:c r="V151" t="str">
+        <x:v>test/android-a11y</x:v>
+      </x:c>
       <x:c r="W151"/>
       <x:c r="X151"/>
       <x:c r="Y151"/>
       <x:c r="Z151"/>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152"/>
+      <x:c r="B152"/>
+      <x:c r="C152"/>
+      <x:c r="D152"/>
+      <x:c r="E152"/>
+      <x:c r="F152"/>
+      <x:c r="G152"/>
+      <x:c r="H152"/>
+      <x:c r="I152"/>
+      <x:c r="J152"/>
+      <x:c r="K152"/>
+      <x:c r="L152"/>
+      <x:c r="M152"/>
+      <x:c r="N152"/>
+      <x:c r="O152"/>
+      <x:c r="P152"/>
+      <x:c r="Q152"/>
+      <x:c r="R152"/>
+      <x:c r="S152"/>
+      <x:c r="T152"/>
+      <x:c r="U152"/>
+      <x:c r="V152"/>
+      <x:c r="W152"/>
+      <x:c r="X152"/>
+      <x:c r="Y152"/>
+      <x:c r="Z152"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="J2:J142">
@@ -11894,7 +11968,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94603eacc9674bf4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d25c96ec7a847c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(android): add reservation access flow
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="Rf691f4a8d3154469"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R56c7217556a54047"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="R5db3950fd0534926"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R98de94fc11b740b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R0e7b2d66a2314c9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R0fcac7f181f8400e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R3a3285a3c04c4518"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Backlog" sheetId="2" r:id="R7733a08f33014757"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Owners" sheetId="3" r:id="Rd08c76b98a534a25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Workflow_DoR_DoD" sheetId="4" r:id="R65bd6eefd86f408f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Figma_Map" sheetId="5" r:id="R6821f31e486f424b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Consistency_Audit" sheetId="6" r:id="R8d4e80d9fd6a44c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0cdad5b969064b4a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re828dda5078b4690"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -820,7 +820,7 @@
       </x:c>
       <x:c r="F6" s="41" t="n">
         <x:f>COUNTIF('01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -888,7 +888,7 @@
       </x:c>
       <x:c r="G11" t="n">
         <x:f>COUNTIFS('01_Backlog'!C2:C142,E11,'01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -1047,7 +1047,7 @@
     <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fc7866a04874f6d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43a7b7f5a2c24540"/>
 </x:worksheet>
 </file>
 
@@ -10536,16 +10536,16 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J133" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K133" s="14" t="str">
         <x:v>IMP-AND-0107, IMP-AND-0109</x:v>
       </x:c>
       <x:c r="L133" s="14" t="str">
-        <x:v>Android Early Journey → V3</x:v>
+        <x:v>Android V3 Access / Vincular reserva</x:v>
       </x:c>
       <x:c r="M133" s="14" t="str">
-        <x:v>31:133 / 238:132</x:v>
+        <x:v>1841:410 / 1841:411 / 1841:431 / 1841:453 / 1841:476 / 1841:496 / 1841:516</x:v>
       </x:c>
       <x:c r="N133" s="14" t="str">
         <x:v>MOB-19 /access</x:v>
@@ -10560,7 +10560,7 @@
         <x:v>Sin auth real, Backend ni navegación V1.</x:v>
       </x:c>
       <x:c r="R133" s="14" t="str">
-        <x:v>IMP-AND-0107 y IMP-AND-0109 COMPLETADA; Figma/contrato frontend/mock READY.</x:v>
+        <x:v>IMP-AND-0107 y IMP-AND-0109 COMPLETADAS; Figma 1841:410 y 25_ACCESS_CONTRACT.md APPROVED; campos, validación, root y success congelados.</x:v>
       </x:c>
       <x:c r="S133" s="14" t="str">
         <x:v>UI tests</x:v>
@@ -10575,7 +10575,10 @@
         <x:v>feature/android-access-link</x:v>
       </x:c>
       <x:c r="W133" s="14" t="str">
-        <x:v>PENDIENTE: orden 0109 → 0108. Tras vinculación exitosa, /access → /account → Account / Stay Hub V3; /access permanece fuera de GuestNavigationShell.</x:v>
+        <x:v>READY: Figma 1841:410 aprobado; contrato frontend/mock 25_ACCESS_CONTRACT.md APPROVED. Campos: código de reserva + correo. Root / → /access aprobado; success usa router.replace(/account). Sin auth, persistencia ni Backend.
+EN_QA: /access y root → /access implementados; código + correo con validación local; MockAccessService + TanStack Mutation; reserva no encontrada, error, offline y submitting cubiertos; success usa router.replace(/account). lint PASS; Expo Doctor 21/21 PASS; typecheck PASS; test PASS (13 suites / 72 tests); export Android PASS; npm run check PASS; git diff --check PASS. Pendiente QA manual y revisión WEB-3.
+QA-AND-0108: teclado corregido con KeyboardAvoidingView height en Android y ScrollView al foco; copy anti-enumeración corregido. ReservationNotFoundError permanece interno; UI usa copy genérico. Tests actualizados; 13 suites / 72 tests PASS; lint PASS; typecheck PASS; npm run check PASS; git diff --check PASS. IMP-AND-0108 permanece EN_QA.
+COMPLETADA: / → /access; /access fuera de GuestNavigationShell; código de reserva + correo; validación local; KeyboardAvoidingView y formulario accesible con teclado; TanStack Mutation; MockAccessService; ReservationNotFoundError interno; copy genérico anti-enumeración; Error genérico separado; NetworkError/Offline separado; submitting y doble submit bloqueado; router.replace(/account). QA manual PASS; WEB-3 PASS; test PASS (13 suites / 72 tests); lint PASS; typecheck PASS; Expo Doctor 21/21 PASS; Android export PASS; git diff --check PASS.</x:v>
       </x:c>
       <x:c r="X133" s="14"/>
       <x:c r="Y133" s="14"/>
@@ -11091,16 +11094,16 @@
     </x:row>
     <x:row r="141" ht="84" customHeight="1">
       <x:c r="A141" s="14" t="str">
-        <x:v>IMP-AND-0201</x:v>
+        <x:v>IMP-AND-0116</x:v>
       </x:c>
       <x:c r="B141" s="14" t="str">
-        <x:v>S2 Android Account</x:v>
+        <x:v>S1 Android Stay &amp; Services</x:v>
       </x:c>
       <x:c r="C141" s="14" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D141" s="14" t="str">
-        <x:v>Cuenta</x:v>
+        <x:v>Cuenta / Desvincular reserva y cambiar estadía</x:v>
       </x:c>
       <x:c r="E141" s="14" t="str">
         <x:v>ANDROID-1</x:v>
@@ -11115,57 +11118,57 @@
         <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I141" s="14" t="str">
-        <x:v>CRÍTICA</x:v>
+        <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J141" s="14" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K141" s="14" t="str">
-        <x:v>IMP-AND-0009, IMP-AND-0109</x:v>
+        <x:v>IMP-AND-0108, IMP-AND-0109, contexto/sesión real de reserva vinculada (pendiente)</x:v>
       </x:c>
       <x:c r="L141" s="14" t="str">
-        <x:v>Android 02 Cuenta, checkout y factura</x:v>
-      </x:c>
-      <x:c r="M141" s="14" t="str">
-        <x:v>238:132</x:v>
-      </x:c>
+        <x:v>Pendiente de fuente visual aprobada</x:v>
+      </x:c>
+      <x:c r="M141" s="14"/>
       <x:c r="N141" s="14" t="str">
-        <x:v>Account</x:v>
+        <x:v>/account</x:v>
       </x:c>
       <x:c r="O141" s="14" t="str">
-        <x:v>Crear Account/Profile contracts</x:v>
+        <x:v>Permitir desvincular la reserva del dispositivo y vincular otra estadía</x:v>
       </x:c>
       <x:c r="P141" s="14" t="str">
-        <x:v>GuestAccount/Profile separados; extiende Account / Stay Hub existente; no duplica /account.</x:v>
+        <x:v>Desde Cuenta: acción, confirmación, limpiar solo contexto/session local, invalidar caches asociadas cuando corresponda, router.replace(/access) y reflejar la nueva estadía.</x:v>
       </x:c>
       <x:c r="Q141" s="14" t="str">
-        <x:v>No Staff auth; no provider JSON UI; mapper tests; sin segundo hub /account.</x:v>
+        <x:v>No cancela reservas ni solicitudes; no borra datos Backend. Account no consume DTOs/fixtures directos de otros módulos.</x:v>
       </x:c>
       <x:c r="R141" s="14" t="str">
-        <x:v>IMP-AND-0109 COMPLETADA; Sprint 0 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
+        <x:v>IMP-AND-0108 e IMP-AND-0109 COMPLETADAS; fuente visual, contrato de contexto/sesión real y estrategia de cache aprobados.</x:v>
       </x:c>
       <x:c r="S141" s="14" t="str">
-        <x:v>Unit.</x:v>
+        <x:v>Flujo de confirmación, limpieza de contexto, caches y nueva estadía validados; sin auth/Backend inventados.</x:v>
       </x:c>
       <x:c r="T141" s="14" t="str">
-        <x:v>unit</x:v>
+        <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U141" s="14" t="str">
-        <x:v>account layers</x:v>
+        <x:v>account linked-reservation context</x:v>
       </x:c>
       <x:c r="V141" s="14" t="str">
-        <x:v>feature/android-account-contract</x:v>
+        <x:v>feature/android-account-unlink-reservation</x:v>
       </x:c>
       <x:c r="W141" s="14" t="str">
-        <x:v>PENDIENTE: IMP-AND-0109 debe completar el Account / Stay Hub en /account. Account/Profile lo extiende sin crear un segundo hub ni duplicar la ruta.</x:v>
+        <x:v>PENDIENTE: no implementada. No existe aún contexto/session real de reserva vinculada.</x:v>
       </x:c>
       <x:c r="X141" s="14"/>
       <x:c r="Y141" s="14"/>
-      <x:c r="Z141" s="14"/>
+      <x:c r="Z141" s="14" t="str">
+        <x:v>No iniciar hasta que exista y se apruebe la capacidad de contexto/sesión real de reserva vinculada.</x:v>
+      </x:c>
     </x:row>
     <x:row r="142" ht="84" customHeight="1">
       <x:c r="A142" s="14" t="str">
-        <x:v>IMP-AND-0202</x:v>
+        <x:v>IMP-AND-0201</x:v>
       </x:c>
       <x:c r="B142" s="14" t="str">
         <x:v>S2 Android Account</x:v>
@@ -11189,13 +11192,13 @@
         <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I142" s="14" t="str">
-        <x:v>ALTA</x:v>
+        <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J142" s="14" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K142" s="14" t="str">
-        <x:v>IMP-AND-0201</x:v>
+        <x:v>IMP-AND-0009, IMP-AND-0109</x:v>
       </x:c>
       <x:c r="L142" s="14" t="str">
         <x:v>Android 02 Cuenta, checkout y factura</x:v>
@@ -11204,40 +11207,42 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N142" s="14" t="str">
-        <x:v>Account/Profile</x:v>
+        <x:v>Account</x:v>
       </x:c>
       <x:c r="O142" s="14" t="str">
-        <x:v>Implementar cuenta/perfil</x:v>
+        <x:v>Crear Account/Profile contracts</x:v>
       </x:c>
       <x:c r="P142" s="14" t="str">
-        <x:v>Display/edit Profile; loading/error/offline; submit.</x:v>
+        <x:v>GuestAccount/Profile separados; extiende Account / Stay Hub existente; no duplica /account.</x:v>
       </x:c>
       <x:c r="Q142" s="14" t="str">
-        <x:v>Account/Profile separation; no secrets; save states correct.</x:v>
+        <x:v>No Staff auth; no provider JSON UI; mapper tests; sin segundo hub /account.</x:v>
       </x:c>
       <x:c r="R142" s="14" t="str">
-        <x:v>IMP-AND-0201 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
+        <x:v>IMP-AND-0109 COMPLETADA; Sprint 0 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S142" s="14" t="str">
-        <x:v>UI tests.</x:v>
+        <x:v>Unit.</x:v>
       </x:c>
       <x:c r="T142" s="14" t="str">
-        <x:v>unit/ui</x:v>
+        <x:v>unit</x:v>
       </x:c>
       <x:c r="U142" s="14" t="str">
-        <x:v>account/profile screens</x:v>
+        <x:v>account layers</x:v>
       </x:c>
       <x:c r="V142" s="14" t="str">
-        <x:v>feature/android-account-profile</x:v>
-      </x:c>
-      <x:c r="W142" s="14"/>
+        <x:v>feature/android-account-contract</x:v>
+      </x:c>
+      <x:c r="W142" s="14" t="str">
+        <x:v>PENDIENTE: IMP-AND-0109 debe completar el Account / Stay Hub en /account. Account/Profile lo extiende sin crear un segundo hub ni duplicar la ruta.</x:v>
+      </x:c>
       <x:c r="X142" s="14"/>
       <x:c r="Y142" s="14"/>
       <x:c r="Z142" s="14"/>
     </x:row>
     <x:row r="143">
       <x:c r="A143" t="str">
-        <x:v>IMP-AND-0203</x:v>
+        <x:v>IMP-AND-0202</x:v>
       </x:c>
       <x:c r="B143" t="str">
         <x:v>S2 Android Account</x:v>
@@ -11246,28 +11251,28 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D143" t="str">
-        <x:v>Checkout/Factura</x:v>
+        <x:v>Cuenta</x:v>
       </x:c>
       <x:c r="E143" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F143" t="str">
-        <x:v>WEB-4</x:v>
+        <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G143" t="str">
-        <x:v>checkout</x:v>
+        <x:v>account</x:v>
       </x:c>
       <x:c r="H143" t="str">
         <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I143" t="str">
-        <x:v>CRÍTICA</x:v>
+        <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J143" t="str">
-        <x:v>READY</x:v>
+        <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K143" t="str">
-        <x:v>IMP-AND-0102</x:v>
+        <x:v>IMP-AND-0201</x:v>
       </x:c>
       <x:c r="L143" t="str">
         <x:v>Android 02 Cuenta, checkout y factura</x:v>
@@ -11276,42 +11281,40 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N143" t="str">
-        <x:v>Checkout/Invoice</x:v>
+        <x:v>Account/Profile</x:v>
       </x:c>
       <x:c r="O143" t="str">
-        <x:v>Implementar checkout e invoice</x:v>
+        <x:v>Implementar cuenta/perfil</x:v>
       </x:c>
       <x:c r="P143" t="str">
-        <x:v>Charges/balance/status Folio read model; invoice ref/status/date/total; offline/error.</x:v>
+        <x:v>Display/edit Profile; loading/error/offline; submit.</x:v>
       </x:c>
       <x:c r="Q143" t="str">
-        <x:v>Finance no recalculated in UI; no sensitive file persisted; no provider raw data.</x:v>
+        <x:v>Account/Profile separation; no secrets; save states correct.</x:v>
       </x:c>
       <x:c r="R143" t="str">
-        <x:v>Checkout/Folio frontend/mock contract approved; representación simulada/frontend únicamente hasta integración Backend/fiscal.</x:v>
+        <x:v>IMP-AND-0201 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S143" t="str">
-        <x:v>Mapper + UI/security.</x:v>
+        <x:v>UI tests.</x:v>
       </x:c>
       <x:c r="T143" t="str">
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U143" t="str">
-        <x:v>checkout/invoice</x:v>
+        <x:v>account/profile screens</x:v>
       </x:c>
       <x:c r="V143" t="str">
-        <x:v>feature/android-checkout-invoice</x:v>
-      </x:c>
-      <x:c r="W143" t="str">
-        <x:v>DoR PASS: Checkout/Folio frontend/mock contract approved; implementación frontend simulada únicamente. No implica pago real, factura fiscal real ni integración FEL/SAT; Backend/fiscal se integra posteriormente.</x:v>
-      </x:c>
+        <x:v>feature/android-account-profile</x:v>
+      </x:c>
+      <x:c r="W143"/>
       <x:c r="X143"/>
       <x:c r="Y143"/>
       <x:c r="Z143"/>
     </x:row>
     <x:row r="144">
       <x:c r="A144" t="str">
-        <x:v>IMP-AND-0204</x:v>
+        <x:v>IMP-AND-0203</x:v>
       </x:c>
       <x:c r="B144" t="str">
         <x:v>S2 Android Account</x:v>
@@ -11320,28 +11323,28 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D144" t="str">
-        <x:v>QA</x:v>
+        <x:v>Checkout/Factura</x:v>
       </x:c>
       <x:c r="E144" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F144" t="str">
-        <x:v>WEB-2</x:v>
+        <x:v>WEB-4</x:v>
       </x:c>
       <x:c r="G144" t="str">
-        <x:v>account-checkout</x:v>
+        <x:v>checkout</x:v>
       </x:c>
       <x:c r="H144" t="str">
-        <x:v>QA</x:v>
+        <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I144" t="str">
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J144" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>READY</x:v>
       </x:c>
       <x:c r="K144" t="str">
-        <x:v>IMP-AND-0202, IMP-AND-0203</x:v>
+        <x:v>IMP-AND-0102</x:v>
       </x:c>
       <x:c r="L144" t="str">
         <x:v>Android 02 Cuenta, checkout y factura</x:v>
@@ -11350,49 +11353,51 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N144" t="str">
-        <x:v>Account/Checkout</x:v>
+        <x:v>Checkout/Invoice</x:v>
       </x:c>
       <x:c r="O144" t="str">
-        <x:v>QA Cuenta/Checkout/Factura</x:v>
+        <x:v>Implementar checkout e invoice</x:v>
       </x:c>
       <x:c r="P144" t="str">
-        <x:v>Profile/checkout/invoice/states/navigation/contracts.</x:v>
+        <x:v>Charges/balance/status Folio read model; invoice ref/status/date/total; offline/error.</x:v>
       </x:c>
       <x:c r="Q144" t="str">
-        <x:v>Guest/Staff separation; finance coherent; Figma parity.</x:v>
+        <x:v>Finance no recalculated in UI; no sensitive file persisted; no provider raw data.</x:v>
       </x:c>
       <x:c r="R144" t="str">
-        <x:v>S2 done.</x:v>
+        <x:v>Checkout/Folio frontend/mock contract approved; representación simulada/frontend únicamente hasta integración Backend/fiscal.</x:v>
       </x:c>
       <x:c r="S144" t="str">
-        <x:v>Android Global DoD.</x:v>
+        <x:v>Mapper + UI/security.</x:v>
       </x:c>
       <x:c r="T144" t="str">
-        <x:v>build/tests/manual</x:v>
+        <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U144" t="str">
-        <x:v>Android S2</x:v>
+        <x:v>checkout/invoice</x:v>
       </x:c>
       <x:c r="V144" t="str">
-        <x:v>test/android-account-checkout</x:v>
-      </x:c>
-      <x:c r="W144"/>
+        <x:v>feature/android-checkout-invoice</x:v>
+      </x:c>
+      <x:c r="W144" t="str">
+        <x:v>DoR PASS: Checkout/Folio frontend/mock contract approved; implementación frontend simulada únicamente. No implica pago real, factura fiscal real ni integración FEL/SAT; Backend/fiscal se integra posteriormente.</x:v>
+      </x:c>
       <x:c r="X144"/>
       <x:c r="Y144"/>
       <x:c r="Z144"/>
     </x:row>
     <x:row r="145">
       <x:c r="A145" t="str">
-        <x:v>IMP-AND-0301</x:v>
+        <x:v>IMP-AND-0204</x:v>
       </x:c>
       <x:c r="B145" t="str">
-        <x:v>S3 Android Loyalty</x:v>
+        <x:v>S2 Android Account</x:v>
       </x:c>
       <x:c r="C145" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D145" t="str">
-        <x:v>Loyalty</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="E145" t="str">
         <x:v>ANDROID-1</x:v>
@@ -11401,63 +11406,61 @@
         <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G145" t="str">
-        <x:v>rewards</x:v>
+        <x:v>account-checkout</x:v>
       </x:c>
       <x:c r="H145" t="str">
-        <x:v>FEATURE</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="I145" t="str">
-        <x:v>ALTA</x:v>
+        <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J145" t="str">
-        <x:v>READY</x:v>
+        <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K145" t="str">
-        <x:v>IMP-AND-0009</x:v>
+        <x:v>IMP-AND-0202, IMP-AND-0203</x:v>
       </x:c>
       <x:c r="L145" t="str">
-        <x:v>Android 03 Loyalty, promociones y perfil</x:v>
+        <x:v>Android 02 Cuenta, checkout y factura</x:v>
       </x:c>
       <x:c r="M145" t="str">
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N145" t="str">
-        <x:v>Rewards</x:v>
+        <x:v>Account/Checkout</x:v>
       </x:c>
       <x:c r="O145" t="str">
-        <x:v>Implementar Rewards</x:v>
+        <x:v>QA Cuenta/Checkout/Factura</x:v>
       </x:c>
       <x:c r="P145" t="str">
-        <x:v>Ledger/balance Domain cross-app; offline/error/empty.</x:v>
+        <x:v>Profile/checkout/invoice/states/navigation/contracts.</x:v>
       </x:c>
       <x:c r="Q145" t="str">
-        <x:v>CANCELLED/NO_SHOW no elegibles; ledger read-only.</x:v>
+        <x:v>Guest/Staff separation; finance coherent; Figma parity.</x:v>
       </x:c>
       <x:c r="R145" t="str">
-        <x:v>Rewards frontend/mock contract approved.</x:v>
+        <x:v>S2 done.</x:v>
       </x:c>
       <x:c r="S145" t="str">
-        <x:v>Mapper + UI.</x:v>
+        <x:v>Android Global DoD.</x:v>
       </x:c>
       <x:c r="T145" t="str">
-        <x:v>unit/ui</x:v>
+        <x:v>build/tests/manual</x:v>
       </x:c>
       <x:c r="U145" t="str">
-        <x:v>rewards</x:v>
+        <x:v>Android S2</x:v>
       </x:c>
       <x:c r="V145" t="str">
-        <x:v>feature/android-rewards</x:v>
-      </x:c>
-      <x:c r="W145" t="str">
-        <x:v>DoR PASS: Rewards frontend/mock contract approved; Backend no requerido para implementación frontend-first.</x:v>
-      </x:c>
+        <x:v>test/android-account-checkout</x:v>
+      </x:c>
+      <x:c r="W145"/>
       <x:c r="X145"/>
       <x:c r="Y145"/>
       <x:c r="Z145"/>
     </x:row>
     <x:row r="146">
       <x:c r="A146" t="str">
-        <x:v>IMP-AND-0302</x:v>
+        <x:v>IMP-AND-0301</x:v>
       </x:c>
       <x:c r="B146" t="str">
         <x:v>S3 Android Loyalty</x:v>
@@ -11466,7 +11469,7 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D146" t="str">
-        <x:v>Promociones</x:v>
+        <x:v>Loyalty</x:v>
       </x:c>
       <x:c r="E146" t="str">
         <x:v>ANDROID-1</x:v>
@@ -11475,7 +11478,7 @@
         <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G146" t="str">
-        <x:v>promotions</x:v>
+        <x:v>rewards</x:v>
       </x:c>
       <x:c r="H146" t="str">
         <x:v>FEATURE</x:v>
@@ -11496,19 +11499,19 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N146" t="str">
-        <x:v>Promotions</x:v>
+        <x:v>Rewards</x:v>
       </x:c>
       <x:c r="O146" t="str">
-        <x:v>Implementar Promotions</x:v>
+        <x:v>Implementar Rewards</x:v>
       </x:c>
       <x:c r="P146" t="str">
-        <x:v>Eligibility/vigencia/stacking reason; states.</x:v>
+        <x:v>Ledger/balance Domain cross-app; offline/error/empty.</x:v>
       </x:c>
       <x:c r="Q146" t="str">
-        <x:v>Incompatible no combinable; reasons correct.</x:v>
+        <x:v>CANCELLED/NO_SHOW no elegibles; ledger read-only.</x:v>
       </x:c>
       <x:c r="R146" t="str">
-        <x:v>Promotions frontend/mock contract approved.</x:v>
+        <x:v>Rewards frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S146" t="str">
         <x:v>Mapper + UI.</x:v>
@@ -11517,13 +11520,13 @@
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U146" t="str">
-        <x:v>promotions</x:v>
+        <x:v>rewards</x:v>
       </x:c>
       <x:c r="V146" t="str">
-        <x:v>feature/android-promotions</x:v>
+        <x:v>feature/android-rewards</x:v>
       </x:c>
       <x:c r="W146" t="str">
-        <x:v>DoR PASS: Promotions frontend/mock contract approved; Backend no requerido para implementación frontend-first.</x:v>
+        <x:v>DoR PASS: Rewards frontend/mock contract approved; Backend no requerido para implementación frontend-first.</x:v>
       </x:c>
       <x:c r="X146"/>
       <x:c r="Y146"/>
@@ -11531,7 +11534,7 @@
     </x:row>
     <x:row r="147">
       <x:c r="A147" t="str">
-        <x:v>IMP-AND-0303</x:v>
+        <x:v>IMP-AND-0302</x:v>
       </x:c>
       <x:c r="B147" t="str">
         <x:v>S3 Android Loyalty</x:v>
@@ -11540,7 +11543,7 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D147" t="str">
-        <x:v>Perfil</x:v>
+        <x:v>Promociones</x:v>
       </x:c>
       <x:c r="E147" t="str">
         <x:v>ANDROID-1</x:v>
@@ -11549,7 +11552,7 @@
         <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G147" t="str">
-        <x:v>profile</x:v>
+        <x:v>promotions</x:v>
       </x:c>
       <x:c r="H147" t="str">
         <x:v>FEATURE</x:v>
@@ -11558,10 +11561,10 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J147" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>READY</x:v>
       </x:c>
       <x:c r="K147" t="str">
-        <x:v>IMP-AND-0201</x:v>
+        <x:v>IMP-AND-0009</x:v>
       </x:c>
       <x:c r="L147" t="str">
         <x:v>Android 03 Loyalty, promociones y perfil</x:v>
@@ -11570,40 +11573,42 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N147" t="str">
-        <x:v>Profile</x:v>
+        <x:v>Promotions</x:v>
       </x:c>
       <x:c r="O147" t="str">
-        <x:v>Implementar perfil final</x:v>
+        <x:v>Implementar Promotions</x:v>
       </x:c>
       <x:c r="P147" t="str">
-        <x:v>Figma layout/edit/states; reuse Account/Profile Domain.</x:v>
+        <x:v>Eligibility/vigencia/stacking reason; states.</x:v>
       </x:c>
       <x:c r="Q147" t="str">
-        <x:v>No duplicated model; PII safe; save states correct.</x:v>
+        <x:v>Incompatible no combinable; reasons correct.</x:v>
       </x:c>
       <x:c r="R147" t="str">
-        <x:v>IMP-AND-0201 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
+        <x:v>Promotions frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S147" t="str">
-        <x:v>UI tests.</x:v>
+        <x:v>Mapper + UI.</x:v>
       </x:c>
       <x:c r="T147" t="str">
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U147" t="str">
-        <x:v>profile</x:v>
+        <x:v>promotions</x:v>
       </x:c>
       <x:c r="V147" t="str">
-        <x:v>feature/android-profile</x:v>
-      </x:c>
-      <x:c r="W147"/>
+        <x:v>feature/android-promotions</x:v>
+      </x:c>
+      <x:c r="W147" t="str">
+        <x:v>DoR PASS: Promotions frontend/mock contract approved; Backend no requerido para implementación frontend-first.</x:v>
+      </x:c>
       <x:c r="X147"/>
       <x:c r="Y147"/>
       <x:c r="Z147"/>
     </x:row>
     <x:row r="148">
       <x:c r="A148" t="str">
-        <x:v>IMP-AND-0304</x:v>
+        <x:v>IMP-AND-0303</x:v>
       </x:c>
       <x:c r="B148" t="str">
         <x:v>S3 Android Loyalty</x:v>
@@ -11612,7 +11617,7 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D148" t="str">
-        <x:v>QA</x:v>
+        <x:v>Perfil</x:v>
       </x:c>
       <x:c r="E148" t="str">
         <x:v>ANDROID-1</x:v>
@@ -11621,19 +11626,19 @@
         <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G148" t="str">
-        <x:v>loyalty-profile</x:v>
+        <x:v>profile</x:v>
       </x:c>
       <x:c r="H148" t="str">
-        <x:v>QA</x:v>
+        <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I148" t="str">
-        <x:v>CRÍTICA</x:v>
+        <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J148" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K148" t="str">
-        <x:v>IMP-AND-0301, IMP-AND-0302, IMP-AND-0303</x:v>
+        <x:v>IMP-AND-0201</x:v>
       </x:c>
       <x:c r="L148" t="str">
         <x:v>Android 03 Loyalty, promociones y perfil</x:v>
@@ -11642,31 +11647,31 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N148" t="str">
-        <x:v>Rewards/Promos/Profile</x:v>
+        <x:v>Profile</x:v>
       </x:c>
       <x:c r="O148" t="str">
-        <x:v>QA Loyalty/Profile</x:v>
+        <x:v>Implementar perfil final</x:v>
       </x:c>
       <x:c r="P148" t="str">
-        <x:v>Rewards/promotions/profile/offline/error/empty/navigation.</x:v>
+        <x:v>Figma layout/edit/states; reuse Account/Profile Domain.</x:v>
       </x:c>
       <x:c r="Q148" t="str">
-        <x:v>Cross-app semantics PASS; Figma parity; no DTO UI.</x:v>
+        <x:v>No duplicated model; PII safe; save states correct.</x:v>
       </x:c>
       <x:c r="R148" t="str">
-        <x:v>S3 done.</x:v>
+        <x:v>IMP-AND-0201 COMPLETADA; Account/Profile frontend/mock contract approved.</x:v>
       </x:c>
       <x:c r="S148" t="str">
-        <x:v>Android Global DoD.</x:v>
+        <x:v>UI tests.</x:v>
       </x:c>
       <x:c r="T148" t="str">
-        <x:v>build/tests/manual</x:v>
+        <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U148" t="str">
-        <x:v>Android S3</x:v>
+        <x:v>profile</x:v>
       </x:c>
       <x:c r="V148" t="str">
-        <x:v>test/android-loyalty</x:v>
+        <x:v>feature/android-profile</x:v>
       </x:c>
       <x:c r="W148"/>
       <x:c r="X148"/>
@@ -11675,16 +11680,16 @@
     </x:row>
     <x:row r="149">
       <x:c r="A149" t="str">
-        <x:v>IMP-AND-0401</x:v>
+        <x:v>IMP-AND-0304</x:v>
       </x:c>
       <x:c r="B149" t="str">
-        <x:v>S4 Android Release</x:v>
+        <x:v>S3 Android Loyalty</x:v>
       </x:c>
       <x:c r="C149" t="str">
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D149" t="str">
-        <x:v>Estados</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="E149" t="str">
         <x:v>ANDROID-1</x:v>
@@ -11693,10 +11698,10 @@
         <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G149" t="str">
-        <x:v>ui-states</x:v>
+        <x:v>loyalty-profile</x:v>
       </x:c>
       <x:c r="H149" t="str">
-        <x:v>SHARED</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="I149" t="str">
         <x:v>CRÍTICA</x:v>
@@ -11705,40 +11710,40 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K149" t="str">
-        <x:v>IMP-AND-0009</x:v>
+        <x:v>IMP-AND-0301, IMP-AND-0302, IMP-AND-0303</x:v>
       </x:c>
       <x:c r="L149" t="str">
-        <x:v>Android 04 Loading, error y offline</x:v>
+        <x:v>Android 03 Loyalty, promociones y perfil</x:v>
       </x:c>
       <x:c r="M149" t="str">
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N149" t="str">
-        <x:v>Universal States</x:v>
+        <x:v>Rewards/Promos/Profile</x:v>
       </x:c>
       <x:c r="O149" t="str">
-        <x:v>Implementar Loading/Error/Empty/Offline shared</x:v>
+        <x:v>QA Loyalty/Profile</x:v>
       </x:c>
       <x:c r="P149" t="str">
-        <x:v>Reusable state UI; retry callback; accessible; no business logic.</x:v>
+        <x:v>Rewards/promotions/profile/offline/error/empty/navigation.</x:v>
       </x:c>
       <x:c r="Q149" t="str">
-        <x:v>Features reutilizan states; offline explicit; retry actionable.</x:v>
+        <x:v>Cross-app semantics PASS; Figma parity; no DTO UI.</x:v>
       </x:c>
       <x:c r="R149" t="str">
-        <x:v>Figma states reviewed.</x:v>
+        <x:v>S3 done.</x:v>
       </x:c>
       <x:c r="S149" t="str">
-        <x:v>UI tests.</x:v>
+        <x:v>Android Global DoD.</x:v>
       </x:c>
       <x:c r="T149" t="str">
-        <x:v>ui</x:v>
+        <x:v>build/tests/manual</x:v>
       </x:c>
       <x:c r="U149" t="str">
-        <x:v>shared state UI</x:v>
+        <x:v>Android S3</x:v>
       </x:c>
       <x:c r="V149" t="str">
-        <x:v>feature/android-universal-states</x:v>
+        <x:v>test/android-loyalty</x:v>
       </x:c>
       <x:c r="W149"/>
       <x:c r="X149"/>
@@ -11747,7 +11752,7 @@
     </x:row>
     <x:row r="150">
       <x:c r="A150" t="str">
-        <x:v>IMP-AND-0402</x:v>
+        <x:v>IMP-AND-0401</x:v>
       </x:c>
       <x:c r="B150" t="str">
         <x:v>S4 Android Release</x:v>
@@ -11762,13 +11767,13 @@
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F150" t="str">
-        <x:v>WEB-3</x:v>
+        <x:v>WEB-2</x:v>
       </x:c>
       <x:c r="G150" t="str">
-        <x:v>offline</x:v>
+        <x:v>ui-states</x:v>
       </x:c>
       <x:c r="H150" t="str">
-        <x:v>FEATURE</x:v>
+        <x:v>SHARED</x:v>
       </x:c>
       <x:c r="I150" t="str">
         <x:v>CRÍTICA</x:v>
@@ -11777,7 +11782,7 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K150" t="str">
-        <x:v>IMP-AND-0401, IMP-AND-0106, IMP-AND-0204, IMP-AND-0304</x:v>
+        <x:v>IMP-AND-0009</x:v>
       </x:c>
       <x:c r="L150" t="str">
         <x:v>Android 04 Loading, error y offline</x:v>
@@ -11786,31 +11791,31 @@
         <x:v>238:132</x:v>
       </x:c>
       <x:c r="N150" t="str">
-        <x:v>All</x:v>
+        <x:v>Universal States</x:v>
       </x:c>
       <x:c r="O150" t="str">
-        <x:v>Integrar states universales</x:v>
+        <x:v>Implementar Loading/Error/Empty/Offline shared</x:v>
       </x:c>
       <x:c r="P150" t="str">
-        <x:v>Reemplazar estados ad-hoc; retry; stale indication donde aplica.</x:v>
+        <x:v>Reusable state UI; retry callback; accessible; no business logic.</x:v>
       </x:c>
       <x:c r="Q150" t="str">
-        <x:v>0 remote screen sin Loading/Error; Offline según Figma; no false success.</x:v>
+        <x:v>Features reutilizan states; offline explicit; retry actionable.</x:v>
       </x:c>
       <x:c r="R150" t="str">
-        <x:v>Feature screens done.</x:v>
+        <x:v>Figma states reviewed.</x:v>
       </x:c>
       <x:c r="S150" t="str">
-        <x:v>Regression states.</x:v>
+        <x:v>UI tests.</x:v>
       </x:c>
       <x:c r="T150" t="str">
-        <x:v>ui/manual</x:v>
+        <x:v>ui</x:v>
       </x:c>
       <x:c r="U150" t="str">
-        <x:v>all Android</x:v>
+        <x:v>shared state UI</x:v>
       </x:c>
       <x:c r="V150" t="str">
-        <x:v>feature/android-state-integration</x:v>
+        <x:v>feature/android-universal-states</x:v>
       </x:c>
       <x:c r="W150"/>
       <x:c r="X150"/>
@@ -11819,7 +11824,7 @@
     </x:row>
     <x:row r="151">
       <x:c r="A151" t="str">
-        <x:v>IMP-AND-0403</x:v>
+        <x:v>IMP-AND-0402</x:v>
       </x:c>
       <x:c r="B151" t="str">
         <x:v>S4 Android Release</x:v>
@@ -11828,19 +11833,19 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D151" t="str">
-        <x:v>QA</x:v>
+        <x:v>Estados</x:v>
       </x:c>
       <x:c r="E151" t="str">
         <x:v>ANDROID-1</x:v>
       </x:c>
       <x:c r="F151" t="str">
-        <x:v>WEB-2</x:v>
+        <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G151" t="str">
-        <x:v>accessibility</x:v>
+        <x:v>offline</x:v>
       </x:c>
       <x:c r="H151" t="str">
-        <x:v>QA</x:v>
+        <x:v>FEATURE</x:v>
       </x:c>
       <x:c r="I151" t="str">
         <x:v>CRÍTICA</x:v>
@@ -11849,10 +11854,10 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="K151" t="str">
-        <x:v>IMP-AND-0402</x:v>
+        <x:v>IMP-AND-0401, IMP-AND-0106, IMP-AND-0204, IMP-AND-0304</x:v>
       </x:c>
       <x:c r="L151" t="str">
-        <x:v>Android final regression</x:v>
+        <x:v>Android 04 Loading, error y offline</x:v>
       </x:c>
       <x:c r="M151" t="str">
         <x:v>238:132</x:v>
@@ -11861,28 +11866,28 @@
         <x:v>All</x:v>
       </x:c>
       <x:c r="O151" t="str">
-        <x:v>Auditoría accesibilidad Android</x:v>
+        <x:v>Integrar states universales</x:v>
       </x:c>
       <x:c r="P151" t="str">
-        <x:v>TalkBack/labels/targets/contrast/focus/auth/errors.</x:v>
+        <x:v>Reemplazar estados ad-hoc; retry; stale indication donde aplica.</x:v>
       </x:c>
       <x:c r="Q151" t="str">
-        <x:v>0 critical/high accessibility defects; primary journeys operable.</x:v>
+        <x:v>0 remote screen sin Loading/Error; Offline según Figma; no false success.</x:v>
       </x:c>
       <x:c r="R151" t="str">
-        <x:v>Features done.</x:v>
+        <x:v>Feature screens done.</x:v>
       </x:c>
       <x:c r="S151" t="str">
-        <x:v>A11y PASS.</x:v>
+        <x:v>Regression states.</x:v>
       </x:c>
       <x:c r="T151" t="str">
-        <x:v>manual/tooling</x:v>
+        <x:v>ui/manual</x:v>
       </x:c>
       <x:c r="U151" t="str">
-        <x:v>whole Android</x:v>
+        <x:v>all Android</x:v>
       </x:c>
       <x:c r="V151" t="str">
-        <x:v>test/android-a11y</x:v>
+        <x:v>feature/android-state-integration</x:v>
       </x:c>
       <x:c r="W151"/>
       <x:c r="X151"/>
@@ -11890,28 +11895,72 @@
       <x:c r="Z151"/>
     </x:row>
     <x:row r="152">
-      <x:c r="A152"/>
-      <x:c r="B152"/>
-      <x:c r="C152"/>
-      <x:c r="D152"/>
-      <x:c r="E152"/>
-      <x:c r="F152"/>
-      <x:c r="G152"/>
-      <x:c r="H152"/>
-      <x:c r="I152"/>
-      <x:c r="J152"/>
-      <x:c r="K152"/>
-      <x:c r="L152"/>
-      <x:c r="M152"/>
-      <x:c r="N152"/>
-      <x:c r="O152"/>
-      <x:c r="P152"/>
-      <x:c r="Q152"/>
-      <x:c r="R152"/>
-      <x:c r="S152"/>
-      <x:c r="T152"/>
-      <x:c r="U152"/>
-      <x:c r="V152"/>
+      <x:c r="A152" t="str">
+        <x:v>IMP-AND-0403</x:v>
+      </x:c>
+      <x:c r="B152" t="str">
+        <x:v>S4 Android Release</x:v>
+      </x:c>
+      <x:c r="C152" t="str">
+        <x:v>ANDROID</x:v>
+      </x:c>
+      <x:c r="D152" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="E152" t="str">
+        <x:v>ANDROID-1</x:v>
+      </x:c>
+      <x:c r="F152" t="str">
+        <x:v>WEB-2</x:v>
+      </x:c>
+      <x:c r="G152" t="str">
+        <x:v>accessibility</x:v>
+      </x:c>
+      <x:c r="H152" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="I152" t="str">
+        <x:v>CRÍTICA</x:v>
+      </x:c>
+      <x:c r="J152" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="K152" t="str">
+        <x:v>IMP-AND-0402</x:v>
+      </x:c>
+      <x:c r="L152" t="str">
+        <x:v>Android final regression</x:v>
+      </x:c>
+      <x:c r="M152" t="str">
+        <x:v>238:132</x:v>
+      </x:c>
+      <x:c r="N152" t="str">
+        <x:v>All</x:v>
+      </x:c>
+      <x:c r="O152" t="str">
+        <x:v>Auditoría accesibilidad Android</x:v>
+      </x:c>
+      <x:c r="P152" t="str">
+        <x:v>TalkBack/labels/targets/contrast/focus/auth/errors.</x:v>
+      </x:c>
+      <x:c r="Q152" t="str">
+        <x:v>0 critical/high accessibility defects; primary journeys operable.</x:v>
+      </x:c>
+      <x:c r="R152" t="str">
+        <x:v>Features done.</x:v>
+      </x:c>
+      <x:c r="S152" t="str">
+        <x:v>A11y PASS.</x:v>
+      </x:c>
+      <x:c r="T152" t="str">
+        <x:v>manual/tooling</x:v>
+      </x:c>
+      <x:c r="U152" t="str">
+        <x:v>whole Android</x:v>
+      </x:c>
+      <x:c r="V152" t="str">
+        <x:v>test/android-a11y</x:v>
+      </x:c>
       <x:c r="W152"/>
       <x:c r="X152"/>
       <x:c r="Y152"/>
@@ -11968,7 +12017,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d25c96ec7a847c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re253c62bf646485b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(android): add housekeeping request flow
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -10687,7 +10687,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J135" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K135" s="14" t="str">
         <x:v>IMP-AND-0107, IMP-AND-0103</x:v>
@@ -10725,7 +10725,9 @@
       <x:c r="V135" s="14" t="str">
         <x:v>feature/android-services-housekeeping</x:v>
       </x:c>
-      <x:c r="W135" s="14"/>
+      <x:c r="W135" s="14" t="str">
+        <x:v>COMPLETADA: ruta /services/housekeeping, query ReservationStay y HousekeepingService mock con TanStack Mutation; QA manual PASS; revisión WEB-3 PASS; lint PASS; typecheck PASS; test PASS; Expo Doctor PASS; Android export PASS; git diff --check PASS. Catálogos QA frontend/mock provisionales; sin Backend ni IDs.</x:v>
+      </x:c>
       <x:c r="X135" s="14"/>
       <x:c r="Y135" s="14"/>
       <x:c r="Z135" s="14"/>

</xml_diff>

<commit_message>
feat(android): add room service flow
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -10761,7 +10761,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J136" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K136" s="14" t="str">
         <x:v>IMP-AND-0107, IMP-AND-0103</x:v>
@@ -10799,7 +10799,9 @@
       <x:c r="V136" s="14" t="str">
         <x:v>feature/android-services-room-service</x:v>
       </x:c>
-      <x:c r="W136" s="14"/>
+      <x:c r="W136" s="14" t="str">
+        <x:v>COMPLETADA: /services/room-service con catálogo y precios frontend/mock, carrito local, deliveryTime frontend/mock y RoomServiceService sustituible. QA automático PASS (lint, typecheck, 16 suites / 101 tests, Expo Doctor 21/21, Android export y Metro); QA manual PASS; revisión WEB-3 PASS. Sin Backend ni IDs de Stay/Reservation/Room; tracking y Mis solicitudes fuera de alcance.</x:v>
+      </x:c>
       <x:c r="X136" s="14"/>
       <x:c r="Y136" s="14"/>
       <x:c r="Z136" s="14"/>

</xml_diff>

<commit_message>
feat(android): add session service requests
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -10835,7 +10835,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J137" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K137" s="14" t="str">
         <x:v>IMP-AND-0107, IMP-AND-0103</x:v>
@@ -10873,7 +10873,9 @@
       <x:c r="V137" s="14" t="str">
         <x:v>feature/android-services-requests</x:v>
       </x:c>
-      <x:c r="W137" s="14"/>
+      <x:c r="W137" s="14" t="str">
+        <x:v>QA automático PASS; QA manual PASS; WEB-3 PASS.</x:v>
+      </x:c>
       <x:c r="X137" s="14"/>
       <x:c r="Y137" s="14"/>
       <x:c r="Z137" s="14"/>

</xml_diff>

<commit_message>
feat(android): add amenities and unify service request UX
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -10909,7 +10909,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J138" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K138" s="14" t="str">
         <x:v>IMP-AND-0107, IMP-AND-0103</x:v>
@@ -10947,7 +10947,9 @@
       <x:c r="V138" s="14" t="str">
         <x:v>feature/android-services-amenities</x:v>
       </x:c>
-      <x:c r="W138" s="14"/>
+      <x:c r="W138" s="14">
+        <x:v>DoR PASS; QA automático PASS; QA manual PASS; WEB-3 PASS.</x:v>
+      </x:c>
       <x:c r="X138" s="14"/>
       <x:c r="Y138" s="14"/>
       <x:c r="Z138" s="14"/>

</xml_diff>

<commit_message>
feat(android): add hotel hub and update guest navigation
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -10965,7 +10965,7 @@
         <x:v>ANDROID</x:v>
       </x:c>
       <x:c r="D139" s="14" t="str">
-        <x:v>Servicios / Información</x:v>
+        <x:v>Hotel</x:v>
       </x:c>
       <x:c r="E139" s="14" t="str">
         <x:v>ANDROID-1</x:v>
@@ -10974,7 +10974,7 @@
         <x:v>WEB-3</x:v>
       </x:c>
       <x:c r="G139" s="14" t="str">
-        <x:v>services</x:v>
+        <x:v>hotel, navigation</x:v>
       </x:c>
       <x:c r="H139" s="14" t="str">
         <x:v>FEATURE</x:v>
@@ -10983,7 +10983,7 @@
         <x:v>ALTA</x:v>
       </x:c>
       <x:c r="J139" s="14" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K139" s="14" t="str">
         <x:v>IMP-AND-0107, IMP-AND-0103</x:v>
@@ -10995,16 +10995,16 @@
         <x:v>31:338 / 238:132</x:v>
       </x:c>
       <x:c r="N139" s="14" t="str">
-        <x:v>MOB-25 /services/hotel-info</x:v>
+        <x:v>MOB-25 /hotel</x:v>
       </x:c>
       <x:c r="O139" s="14" t="str">
-        <x:v>Migrar Información del hotel</x:v>
+        <x:v>Hotel independiente y shell Guest</x:v>
       </x:c>
       <x:c r="P139" s="14" t="str">
-        <x:v>Servicios activa en /services/hotel-info.</x:v>
+        <x:v>Hotel activa en /hotel; Chat flotante y drawer.</x:v>
       </x:c>
       <x:c r="Q139" s="14" t="str">
-        <x:v>Sin Backend ni duplicar GuestNavigationShell.</x:v>
+        <x:v>Perfil frontend/mock demo; sin Backend, Stay ni solicitudes.</x:v>
       </x:c>
       <x:c r="R139" s="14" t="str">
         <x:v>IMP-AND-0107 y IMP-AND-0103 COMPLETADA; contrato frontend/mock READY.</x:v>
@@ -11016,12 +11016,14 @@
         <x:v>unit/ui</x:v>
       </x:c>
       <x:c r="U139" s="14" t="str">
-        <x:v>services/hotel-info</x:v>
+        <x:v>/hotel</x:v>
       </x:c>
       <x:c r="V139" s="14" t="str">
-        <x:v>feature/android-services-hotel-info</x:v>
-      </x:c>
-      <x:c r="W139" s="14"/>
+        <x:v>feature/android-hotel-info</x:v>
+      </x:c>
+      <x:c r="W139" s="14">
+        <x:v>DoR PASS; QA automático PASS; QA manual PASS; WEB-3 PASS.</x:v>
+      </x:c>
       <x:c r="X139" s="14"/>
       <x:c r="Y139" s="14"/>
       <x:c r="Z139" s="14"/>

</xml_diff>

<commit_message>
test(android): close stay and services sprint QA
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -10388,7 +10388,7 @@
         <x:v>CRÍTICA</x:v>
       </x:c>
       <x:c r="J131" s="14" t="str">
-        <x:v>EN_PROGRESO</x:v>
+        <x:v>COMPLETADA</x:v>
       </x:c>
       <x:c r="K131" s="14" t="str">
         <x:v>IMP-AND-0102, IMP-AND-0103, IMP-AND-0104, IMP-AND-0105</x:v>
@@ -10427,7 +10427,7 @@
         <x:v>test/android-stay-services</x:v>
       </x:c>
       <x:c r="W131" s="14" t="str">
-        <x:v>QA técnica PASS preservada. EN_PROGRESO por hallazgos bloqueantes QA-AND-0106-01 (footbar V1/Stay aislado) y QA-AND-0106-02 (MOB-01 y MOB-03..07 sin migración V3). Ver IMP-AND-0107 / docs Android 23; reejecutar QA tras las migraciones.</x:v>
+        <x:v>Android Global DoD PASS; QA técnica PASS; QA manual PASS; WEB-3 PASS. QA-AND-0106-01 RESUELTO (shell V3 única, Inicio en /account). QA-AND-0106-02 RESUELTO (IMP-AND-0107 y 0108..0114 COMPLETADAS).</x:v>
       </x:c>
       <x:c r="X131" s="14"/>
       <x:c r="Y131" s="14"/>

</xml_diff>

<commit_message>
feat(web/reservations): implement No-show flow (IMP-WEB-0304)
No-show pipeline following the cancellation pattern (PROVISIONAL contract):
- reservation-no-show.dto.ts: preview/apply PROVISIONAL contract
- reservation-no-show.mapper.ts + tests
- reservation.service: previewNoShow, applyNoShow + service tests
- use-reservation-no-show hook (preview + apply mutations) + tests
- reservation-no-show component (policy/cutoff/charge + ConfirmDialog) + tests
- ConfirmDialog: busyLabel support (default 'Cancelando…')
- detail header: 'Marcar no-show' button for NO_SHOW_PENDING + tests
- index.ts: exports NoShowPreview/NoShowResult
- MSW dev fixtures: no-show-preview/no-show handlers + NO_SHOW_PENDING detail
- Backlog row 49: PENDIENTE -> EN_QA
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -6789,7 +6789,7 @@
       </c>
       <c r="J49" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>EN_QA</t>
         </is>
       </c>
       <c r="K49" s="14" t="inlineStr">
@@ -6849,7 +6849,11 @@
         </is>
       </c>
       <c r="W49" s="14" t="str"/>
-      <c r="X49" s="14" t="str"/>
+      <c r="X49" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
       <c r="Y49" s="14" t="str"/>
       <c r="Z49" s="14" t="str"/>
     </row>

</xml_diff>

<commit_message>
feat(web/stays): implement Room Move flow (IMP-WEB-0306)
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -7021,7 +7021,7 @@
       </c>
       <c r="J51" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>EN_QA</t>
         </is>
       </c>
       <c r="K51" s="14" t="inlineStr">
@@ -7081,7 +7081,11 @@
         </is>
       </c>
       <c r="W51" s="14" t="str"/>
-      <c r="X51" s="14" t="str"/>
+      <c r="X51" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
       <c r="Y51" s="14" t="str"/>
       <c r="Z51" s="14" t="str"/>
     </row>

</xml_diff>

<commit_message>
feat(android): add rewards guest experience
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -11501,7 +11501,7 @@
         <v>ALTA</v>
       </c>
       <c r="J146" t="str">
-        <v>READY</v>
+        <v>COMPLETADA</v>
       </c>
       <c r="K146" t="str">
         <v>IMP-AND-0009</v>
@@ -11540,7 +11540,7 @@
         <v>feature/android-rewards</v>
       </c>
       <c r="W146" t="str">
-        <v>DoR PASS: Rewards frontend/mock contract approved; Backend no requerido para implementación frontend-first.</v>
+        <v>DoR PASS. Automated QA PASS: lint, typecheck, 212 tests, Expo Doctor 21/21, Android export and Metro /status. Manual QA PASS. WEB-2 PASS. Frontend/mock only; Backend no requerido.</v>
       </c>
       <c r="X146"/>
       <c r="Y146"/>

</xml_diff>

<commit_message>
feat(android): add promotions guest experience
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -11575,7 +11575,7 @@
         <v>ALTA</v>
       </c>
       <c r="J147" t="str">
-        <v>READY</v>
+        <v>COMPLETADA</v>
       </c>
       <c r="K147" t="str">
         <v>IMP-AND-0009</v>
@@ -11614,7 +11614,7 @@
         <v>feature/android-promotions</v>
       </c>
       <c r="W147" t="str">
-        <v>DoR PASS: Promotions frontend/mock contract approved; Backend no requerido para implementación frontend-first.</v>
+        <v>DoR PASS. Automated QA PASS: lint, typecheck, 223 tests, Expo Doctor 21/21, Android export and Metro /status. Manual QA PASS. WEB-2 PASS. Frontend/mock only; Backend no requerido.</v>
       </c>
       <c r="X147"/>
       <c r="Y147"/>

</xml_diff>

<commit_message>
feat(android): add account profile contracts
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -11205,7 +11205,7 @@
         <v>CRÍTICA</v>
       </c>
       <c r="J142" s="14" t="str">
-        <v>PENDIENTE</v>
+        <v>COMPLETADA</v>
       </c>
       <c r="K142" s="14" t="str">
         <v>IMP-AND-0009, IMP-AND-0109</v>
@@ -11244,7 +11244,7 @@
         <v>feature/android-account-contract</v>
       </c>
       <c r="W142" s="14" t="str">
-        <v>PENDIENTE: IMP-AND-0109 debe completar el Account / Stay Hub en /account. Account/Profile lo extiende sin crear un segundo hub ni duplicar la ruta.</v>
+        <v>DoR PASS. Automated QA PASS: lint, typecheck, 231 tests, Expo Doctor 21/21, Android export and Metro /status. Manual QA PASS: contract inspection and controlled mock/session behavior. WEB-2 PASS: contract implementation review. Account/Profile frontend/mock contract APPROVED; no Backend requerido. Extiende /account sin segundo hub.</v>
       </c>
       <c r="X142" s="14"/>
       <c r="Y142" s="14"/>

</xml_diff>

<commit_message>
docs(android): resolve account profile ownership
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -11279,7 +11279,7 @@
         <v>ALTA</v>
       </c>
       <c r="J143" t="str">
-        <v>PENDIENTE</v>
+        <v>READY</v>
       </c>
       <c r="K143" t="str">
         <v>IMP-AND-0201</v>
@@ -11317,7 +11317,9 @@
       <c r="V143" t="str">
         <v>feature/android-account-profile</v>
       </c>
-      <c r="W143"/>
+      <c r="W143" s="14" t="str">
+        <v>DoR PASS. Change Control 31: Account owns canonical /account/profile; drawer CUENTA &gt; Perfil; Back /account. Automated QA PENDING. Manual QA PENDING. WEB-2 PENDING. Frontend/mock session-only; no Backend ni persistencia.</v>
+      </c>
       <c r="X143"/>
       <c r="Y143"/>
       <c r="Z143"/>
@@ -11687,7 +11689,9 @@
       <c r="V148" t="str">
         <v>feature/android-profile</v>
       </c>
-      <c r="W148"/>
+      <c r="W148" s="14" t="str">
+        <v>PENDIENTE permitido por XLSX. ABSORBIDA POR IMP-AND-0202 — NO IMPLEMENTAR. Change Control 31: no segunda ProfileScreen, route, domain, service, Query/Mutation ni fuente de verdad.</v>
+      </c>
       <c r="X148"/>
       <c r="Y148"/>
       <c r="Z148"/>
@@ -11724,7 +11728,7 @@
         <v>PENDIENTE</v>
       </c>
       <c r="K149" t="str">
-        <v>IMP-AND-0301, IMP-AND-0302, IMP-AND-0303</v>
+        <v>IMP-AND-0301, IMP-AND-0302, IMP-AND-0202</v>
       </c>
       <c r="L149" t="str">
         <v>Android 03 Loyalty, promociones y perfil</v>
@@ -11759,7 +11763,9 @@
       <c r="V149" t="str">
         <v>test/android-loyalty</v>
       </c>
-      <c r="W149"/>
+      <c r="W149" s="14" t="str">
+        <v>Change Control 31: dependencia de Profile sustituida por IMP-AND-0202, implementación canónica. Permanece PENDIENTE hasta completar 0202.</v>
+      </c>
       <c r="X149"/>
       <c r="Y149"/>
       <c r="Z149"/>

</xml_diff>

<commit_message>
docs(android): define auth reservation context
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -11279,7 +11279,7 @@
         <v>ALTA</v>
       </c>
       <c r="J143" t="str">
-        <v>READY</v>
+        <v>EN_PROGRESO</v>
       </c>
       <c r="K143" t="str">
         <v>IMP-AND-0201</v>
@@ -11318,7 +11318,7 @@
         <v>feature/android-account-profile</v>
       </c>
       <c r="W143" s="14" t="str">
-        <v>DoR PASS. Change Control 31: Account owns canonical /account/profile; drawer CUENTA &gt; Perfil; Back /account. Automated QA PENDING. Manual QA PENDING. WEB-2 PENDING. Frontend/mock session-only; no Backend ni persistencia.</v>
+        <v>DoR PASS. Change Control 31/32: Profile permanece en Account y vuelve a EN_PROGRESO para mover Perfil a la primera acción del drawer y mantener Profile visible detrás de la confirmación dirty. QA automática PENDING; Manual QA PENDING; WEB-2 PENDING. Foundation auth/reservas/contexto activo pendiente; sin Backend ni persistencia.</v>
       </c>
       <c r="X143"/>
       <c r="Y143"/>

</xml_diff>

<commit_message>
feat(android): implement account profile
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -11279,7 +11279,7 @@
         <v>ALTA</v>
       </c>
       <c r="J143" t="str">
-        <v>EN_PROGRESO</v>
+        <v>COMPLETADA</v>
       </c>
       <c r="K143" t="str">
         <v>IMP-AND-0201</v>
@@ -11318,7 +11318,7 @@
         <v>feature/android-account-profile</v>
       </c>
       <c r="W143" s="14" t="str">
-        <v>DoR PASS. Change Control 31/32: Profile permanece en Account y vuelve a EN_PROGRESO para mover Perfil a la primera acción del drawer y mantener Profile visible detrás de la confirmación dirty. QA automática PENDING; Manual QA PENDING; WEB-2 PENDING. Foundation auth/reservas/contexto activo pendiente; sin Backend ni persistencia.</v>
+        <v>DoR PASS. QA automática PASS: lint, typecheck, 28 suites / 242 tests, Expo Doctor 21/21, export Android y Metro. Manual QA PASS; WEB-2 PASS. Change Control 31/32 aplicado: Perfil primera acción del drawer y confirmación dirty con Profile visible. Foundation auth/reservas/contexto activo pendiente; sin Backend ni persistencia.</v>
       </c>
       <c r="X143"/>
       <c r="Y143"/>

</xml_diff>

<commit_message>
feat(android): add guest auth and reservation context foundation
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -505,7 +505,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationBacklog" displayName="ImplementationBacklog" ref="A1:Z151" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationBacklog" displayName="ImplementationBacklog" ref="A1:Z156" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="26">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Sprint"/>
@@ -730,325 +730,325 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="18" t="str">
-        <x:v>Backlog de Implementación — PMS Hotel Boutique</x:v>
-      </x:c>
-      <x:c r="B1" s="18"/>
-      <x:c r="C1" s="18"/>
-      <x:c r="D1" s="18"/>
-      <x:c r="E1" s="18"/>
-      <x:c r="F1" s="18"/>
-      <x:c r="G1" s="18"/>
-      <x:c r="H1" s="18"/>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="18"/>
-      <x:c r="B2" s="18"/>
-      <x:c r="C2" s="18"/>
-      <x:c r="D2" s="18"/>
-      <x:c r="E2" s="18"/>
-      <x:c r="F2" s="18"/>
-      <x:c r="G2" s="18"/>
-      <x:c r="H2" s="18"/>
-    </x:row>
-    <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="26" t="str">
-        <x:v>Fuente oficial de trabajo para WEB-1..4 y ANDROID-1. Archivo canónico: docs/Backlog_Implementacion_PMS_V1.xlsx. No avanzar una tarea dependiente hasta que sus dependencias estén COMPLETADAS y el DoD haya pasado QA.</x:v>
-      </x:c>
-      <x:c r="B3" s="26"/>
-      <x:c r="C3" s="26"/>
-      <x:c r="D3" s="26"/>
-      <x:c r="E3" s="26"/>
-      <x:c r="F3" s="26"/>
-      <x:c r="G3" s="26"/>
-      <x:c r="H3" s="26"/>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="34" t="str">
-        <x:v>Total tareas</x:v>
-      </x:c>
-      <x:c r="B5" s="34" t="str">
-        <x:v>READY</x:v>
-      </x:c>
-      <x:c r="C5" s="34" t="str">
-        <x:v>En progreso</x:v>
-      </x:c>
-      <x:c r="D5" s="34" t="str">
-        <x:v>En QA</x:v>
-      </x:c>
-      <x:c r="E5" s="34" t="str">
-        <x:v>Bloqueadas</x:v>
-      </x:c>
-      <x:c r="F5" s="34" t="str">
-        <x:v>Completadas</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="32" customHeight="1">
-      <x:c r="A6" s="41" t="n">
-        <x:f>COUNTA('01_Backlog'!A2:A142)</x:f>
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="B6" s="41" t="n">
-        <x:f>COUNTIF('01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C6" s="41" t="n">
-        <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_PROGRESO")</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D6" s="41" t="n">
-        <x:f>COUNTIF('01_Backlog'!J2:J142,"EN_QA")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E6" s="41" t="n">
-        <x:f>COUNTIF('01_Backlog'!J2:J142,"BLOQUEADA")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F6" s="41" t="n">
-        <x:f>COUNTIF('01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>35</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="6" t="str">
-        <x:v>Owner</x:v>
-      </x:c>
-      <x:c r="B9" s="6" t="str">
-        <x:v>Total asignadas</x:v>
-      </x:c>
-      <x:c r="C9" s="6" t="str">
-        <x:v>Estado inicial READY</x:v>
-      </x:c>
-      <x:c r="E9" s="6" t="str">
-        <x:v>Aplicación</x:v>
-      </x:c>
-      <x:c r="F9" s="6" t="str">
-        <x:v>Total</x:v>
-      </x:c>
-      <x:c r="G9" s="6" t="str">
-        <x:v>Completadas</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="24" customHeight="1">
-      <x:c r="A10" s="12" t="str">
-        <x:v>WEB-1</x:v>
-      </x:c>
-      <x:c r="B10" s="12" t="n">
-        <x:f>COUNTIF('01_Backlog'!E2:E142,A10)</x:f>
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C10" s="12" t="n">
-        <x:f>COUNTIFS('01_Backlog'!E2:E142,A10,'01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E10" t="str">
-        <x:v>WEB</x:v>
-      </x:c>
-      <x:c r="F10" t="n">
-        <x:f>COUNTIF('01_Backlog'!C2:C142,E10)</x:f>
-        <x:v>114</x:v>
-      </x:c>
-      <x:c r="G10" t="n">
-        <x:f>COUNTIFS('01_Backlog'!C2:C142,E10,'01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>17</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="24" customHeight="1">
-      <x:c r="A11" s="12" t="str">
-        <x:v>WEB-2</x:v>
-      </x:c>
-      <x:c r="B11" s="12" t="n">
-        <x:f>COUNTIF('01_Backlog'!E2:E142,A11)</x:f>
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="C11" s="12" t="n">
-        <x:f>COUNTIFS('01_Backlog'!E2:E142,A11,'01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E11" t="str">
-        <x:v>ANDROID</x:v>
-      </x:c>
-      <x:c r="F11" t="n">
-        <x:f>COUNTIF('01_Backlog'!C2:C142,E11)</x:f>
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="G11" t="n">
-        <x:f>COUNTIFS('01_Backlog'!C2:C142,E11,'01_Backlog'!J2:J142,"COMPLETADA")</x:f>
-        <x:v>18</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="24" customHeight="1">
-      <x:c r="A12" s="12" t="str">
-        <x:v>WEB-3</x:v>
-      </x:c>
-      <x:c r="B12" s="12" t="n">
-        <x:f>COUNTIF('01_Backlog'!E2:E142,A12)</x:f>
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="C12" s="12" t="n">
-        <x:f>COUNTIFS('01_Backlog'!E2:E142,A12,'01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="24" customHeight="1">
-      <x:c r="A13" s="12" t="str">
-        <x:v>WEB-4</x:v>
-      </x:c>
-      <x:c r="B13" s="12" t="n">
-        <x:f>COUNTIF('01_Backlog'!E2:E142,A13)</x:f>
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="C13" s="12" t="n">
-        <x:f>COUNTIFS('01_Backlog'!E2:E142,A13,'01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="12" t="str">
-        <x:v>ANDROID-1</x:v>
-      </x:c>
-      <x:c r="B14" s="12" t="n">
-        <x:f>COUNTIF('01_Backlog'!E2:E142,A14)</x:f>
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="C14" s="12" t="n">
-        <x:f>COUNTIFS('01_Backlog'!E2:E142,A14,'01_Backlog'!J2:J142,"READY")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="6" t="str">
-        <x:v>Flujo obligatorio</x:v>
-      </x:c>
-      <x:c r="B17" s="6"/>
-      <x:c r="C17" s="6"/>
-      <x:c r="D17" s="6"/>
-      <x:c r="E17" s="6"/>
-      <x:c r="F17" s="6"/>
-      <x:c r="G17" s="6"/>
-      <x:c r="H17" s="6"/>
-    </x:row>
-    <x:row r="18" ht="28" customHeight="1">
-      <x:c r="A18" s="60" t="str">
-        <x:v>PENDIENTE</x:v>
-      </x:c>
-      <x:c r="B18" s="60" t="str">
-        <x:v>→</x:v>
-      </x:c>
-      <x:c r="C18" s="60" t="str">
-        <x:v>READY</x:v>
-      </x:c>
-      <x:c r="D18" s="60" t="str">
-        <x:v>→</x:v>
-      </x:c>
-      <x:c r="E18" s="48"/>
-      <x:c r="F18" s="48"/>
-      <x:c r="G18" s="48"/>
-      <x:c r="H18" s="48"/>
-    </x:row>
-    <x:row r="19" ht="28" customHeight="1">
-      <x:c r="A19" s="60" t="str">
-        <x:v>EN_PROGRESO</x:v>
-      </x:c>
-      <x:c r="B19" s="60" t="str">
-        <x:v>→</x:v>
-      </x:c>
-      <x:c r="C19" s="60" t="str">
-        <x:v>EN_QA</x:v>
-      </x:c>
-      <x:c r="D19" s="60" t="str">
-        <x:v>→ COMPLETADA</x:v>
-      </x:c>
-      <x:c r="E19" s="48"/>
-      <x:c r="F19" s="48"/>
-      <x:c r="G19" s="48"/>
-      <x:c r="H19" s="48"/>
-    </x:row>
-    <x:row r="20" ht="28" customHeight="1">
-      <x:c r="A20" s="60" t="str">
-        <x:v>Si QA falla</x:v>
-      </x:c>
-      <x:c r="B20" s="60" t="str">
-        <x:v>→</x:v>
-      </x:c>
-      <x:c r="C20" s="60" t="str">
-        <x:v>EN_PROGRESO</x:v>
-      </x:c>
-      <x:c r="D20" s="60" t="str">
-        <x:v>corregir y re-QA</x:v>
-      </x:c>
-      <x:c r="E20" s="48"/>
-      <x:c r="F20" s="48"/>
-      <x:c r="G20" s="48"/>
-      <x:c r="H20" s="48"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="55" t="str">
-        <x:v>Cómo usar este backlog:
-1) Cada integrante filtra Owner y Estado=READY. 2) Verifica dependencias y DoR. 3) Cambia a EN_PROGRESO y registra rama/fecha. 4) Al terminar, abre PR, adjunta evidencia y cambia a EN_QA. 5) El reviewer ejecuta criterios de aceptación + DoD. Si falla, vuelve a EN_PROGRESO. 6) Solo con PASS se marca COMPLETADA. Para tareas shared/cross-domain, el reviewer indicado es obligatorio.</x:v>
-      </x:c>
-      <x:c r="B22" s="55"/>
-      <x:c r="C22" s="55"/>
-      <x:c r="D22" s="55"/>
-      <x:c r="E22" s="55"/>
-      <x:c r="F22" s="55"/>
-      <x:c r="G22" s="55"/>
-      <x:c r="H22" s="55"/>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="55"/>
-      <x:c r="B23" s="55"/>
-      <x:c r="C23" s="55"/>
-      <x:c r="D23" s="55"/>
-      <x:c r="E23" s="55"/>
-      <x:c r="F23" s="55"/>
-      <x:c r="G23" s="55"/>
-      <x:c r="H23" s="55"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="55"/>
-      <x:c r="B24" s="55"/>
-      <x:c r="C24" s="55"/>
-      <x:c r="D24" s="55"/>
-      <x:c r="E24" s="55"/>
-      <x:c r="F24" s="55"/>
-      <x:c r="G24" s="55"/>
-      <x:c r="H24" s="55"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="55"/>
-      <x:c r="B25" s="55"/>
-      <x:c r="C25" s="55"/>
-      <x:c r="D25" s="55"/>
-      <x:c r="E25" s="55"/>
-      <x:c r="F25" s="55"/>
-      <x:c r="G25" s="55"/>
-      <x:c r="H25" s="55"/>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:H2"/>
-    <x:mergeCell ref="A3:H3"/>
-    <x:mergeCell ref="A22:H25"/>
-    <x:mergeCell ref="A17:D17"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43a7b7f5a2c24540"/>
-</x:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="str">
+        <v>Backlog de Implementación — PMS Hotel Boutique</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="26" t="str">
+        <v>Fuente oficial de trabajo para WEB-1..4 y ANDROID-1. Archivo canónico: docs/Backlog_Implementacion_PMS_V1.xlsx. No avanzar una tarea dependiente hasta que sus dependencias estén COMPLETADAS y el DoD haya pasado QA.</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="34" t="str">
+        <v>Total tareas</v>
+      </c>
+      <c r="B5" s="34" t="str">
+        <v>READY</v>
+      </c>
+      <c r="C5" s="34" t="str">
+        <v>En progreso</v>
+      </c>
+      <c r="D5" s="34" t="str">
+        <v>En QA</v>
+      </c>
+      <c r="E5" s="34" t="str">
+        <v>Bloqueadas</v>
+      </c>
+      <c r="F5" s="34" t="str">
+        <v>Completadas</v>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="41" t="n">
+        <f>COUNTA('01_Backlog'!A2:A156)</f>
+        <v>155</v>
+      </c>
+      <c r="B6" s="41" t="n">
+        <f>COUNTIF('01_Backlog'!J2:J156,"READY")</f>
+        <v>0</v>
+      </c>
+      <c r="C6" s="41" t="n">
+        <f>COUNTIF('01_Backlog'!J2:J156,"EN_PROGRESO")</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="41" t="n">
+        <f>COUNTIF('01_Backlog'!J2:J156,"EN_QA")</f>
+        <v>1</v>
+      </c>
+      <c r="E6" s="41" t="n">
+        <f>COUNTIF('01_Backlog'!J2:J156,"BLOQUEADA")</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="41" t="n">
+        <f>COUNTIF('01_Backlog'!J2:J156,"COMPLETADA")</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="str">
+        <v>Owner</v>
+      </c>
+      <c r="B9" s="6" t="str">
+        <v>Total asignadas</v>
+      </c>
+      <c r="C9" s="6" t="str">
+        <v>Estado inicial READY</v>
+      </c>
+      <c r="E9" s="6" t="str">
+        <v>Aplicación</v>
+      </c>
+      <c r="F9" s="6" t="str">
+        <v>Total</v>
+      </c>
+      <c r="G9" s="6" t="str">
+        <v>Completadas</v>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="12" t="str">
+        <v>WEB-1</v>
+      </c>
+      <c r="B10" s="12" t="n">
+        <f>COUNTIF('01_Backlog'!E2:E156,A10)</f>
+        <v>17</v>
+      </c>
+      <c r="C10" s="12" t="n">
+        <f>COUNTIFS('01_Backlog'!E2:E156,A10,'01_Backlog'!J2:J156,"READY")</f>
+        <v>0</v>
+      </c>
+      <c r="E10" t="str">
+        <v>WEB</v>
+      </c>
+      <c r="F10" t="n">
+        <f>COUNTIF('01_Backlog'!C2:C156,E10)</f>
+        <v>114</v>
+      </c>
+      <c r="G10" t="n">
+        <f>COUNTIFS('01_Backlog'!C2:C156,E10,'01_Backlog'!J2:J156,"COMPLETADA")</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="12" t="str">
+        <v>WEB-2</v>
+      </c>
+      <c r="B11" s="12" t="n">
+        <f>COUNTIF('01_Backlog'!E2:E156,A11)</f>
+        <v>26</v>
+      </c>
+      <c r="C11" s="12" t="n">
+        <f>COUNTIFS('01_Backlog'!E2:E156,A11,'01_Backlog'!J2:J156,"READY")</f>
+        <v>0</v>
+      </c>
+      <c r="E11" t="str">
+        <v>ANDROID</v>
+      </c>
+      <c r="F11" t="n">
+        <f>COUNTIF('01_Backlog'!C2:C156,E11)</f>
+        <v>41</v>
+      </c>
+      <c r="G11" t="n">
+        <f>COUNTIFS('01_Backlog'!C2:C156,E11,'01_Backlog'!J2:J156,"COMPLETADA")</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="12" t="str">
+        <v>WEB-3</v>
+      </c>
+      <c r="B12" s="12" t="n">
+        <f>COUNTIF('01_Backlog'!E2:E156,A12)</f>
+        <v>45</v>
+      </c>
+      <c r="C12" s="12" t="n">
+        <f>COUNTIFS('01_Backlog'!E2:E156,A12,'01_Backlog'!J2:J156,"READY")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="12" t="str">
+        <v>WEB-4</v>
+      </c>
+      <c r="B13" s="12" t="n">
+        <f>COUNTIF('01_Backlog'!E2:E156,A13)</f>
+        <v>26</v>
+      </c>
+      <c r="C13" s="12" t="n">
+        <f>COUNTIFS('01_Backlog'!E2:E156,A13,'01_Backlog'!J2:J156,"READY")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="12" t="str">
+        <v>ANDROID-1</v>
+      </c>
+      <c r="B14" s="12" t="n">
+        <f>COUNTIF('01_Backlog'!E2:E156,A14)</f>
+        <v>41</v>
+      </c>
+      <c r="C14" s="12" t="n">
+        <f>COUNTIFS('01_Backlog'!E2:E156,A14,'01_Backlog'!J2:J156,"READY")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="str">
+        <v>Flujo obligatorio</v>
+      </c>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="60" t="str">
+        <v>PENDIENTE</v>
+      </c>
+      <c r="B18" s="60" t="str">
+        <v>→</v>
+      </c>
+      <c r="C18" s="60" t="str">
+        <v>READY</v>
+      </c>
+      <c r="D18" s="60" t="str">
+        <v>→</v>
+      </c>
+      <c r="E18" s="48"/>
+      <c r="F18" s="48"/>
+      <c r="G18" s="48"/>
+      <c r="H18" s="48"/>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="60" t="str">
+        <v>EN_PROGRESO</v>
+      </c>
+      <c r="B19" s="60" t="str">
+        <v>→</v>
+      </c>
+      <c r="C19" s="60" t="str">
+        <v>EN_QA</v>
+      </c>
+      <c r="D19" s="60" t="str">
+        <v>→ COMPLETADA</v>
+      </c>
+      <c r="E19" s="48"/>
+      <c r="F19" s="48"/>
+      <c r="G19" s="48"/>
+      <c r="H19" s="48"/>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="60" t="str">
+        <v>Si QA falla</v>
+      </c>
+      <c r="B20" s="60" t="str">
+        <v>→</v>
+      </c>
+      <c r="C20" s="60" t="str">
+        <v>EN_PROGRESO</v>
+      </c>
+      <c r="D20" s="60" t="str">
+        <v>corregir y re-QA</v>
+      </c>
+      <c r="E20" s="48"/>
+      <c r="F20" s="48"/>
+      <c r="G20" s="48"/>
+      <c r="H20" s="48"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="55" t="str">
+        <v>Cómo usar este backlog:
+1) Cada integrante filtra Owner y Estado=READY. 2) Verifica dependencias y DoR. 3) Cambia a EN_PROGRESO y registra rama/fecha. 4) Al terminar, abre PR, adjunta evidencia y cambia a EN_QA. 5) El reviewer ejecuta criterios de aceptación + DoD. Si falla, vuelve a EN_PROGRESO. 6) Solo con PASS se marca COMPLETADA. Para tareas shared/cross-domain, el reviewer indicado es obligatorio.</v>
+      </c>
+      <c r="B22" s="55"/>
+      <c r="C22" s="55"/>
+      <c r="D22" s="55"/>
+      <c r="E22" s="55"/>
+      <c r="F22" s="55"/>
+      <c r="G22" s="55"/>
+      <c r="H22" s="55"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="55"/>
+      <c r="B23" s="55"/>
+      <c r="C23" s="55"/>
+      <c r="D23" s="55"/>
+      <c r="E23" s="55"/>
+      <c r="F23" s="55"/>
+      <c r="G23" s="55"/>
+      <c r="H23" s="55"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="55"/>
+      <c r="B24" s="55"/>
+      <c r="C24" s="55"/>
+      <c r="D24" s="55"/>
+      <c r="E24" s="55"/>
+      <c r="F24" s="55"/>
+      <c r="G24" s="55"/>
+      <c r="H24" s="55"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="55"/>
+      <c r="B25" s="55"/>
+      <c r="C25" s="55"/>
+      <c r="D25" s="55"/>
+      <c r="E25" s="55"/>
+      <c r="F25" s="55"/>
+      <c r="G25" s="55"/>
+      <c r="H25" s="55"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A1:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A22:H25"/>
+    <mergeCell ref="A17:D17"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing ns1:id="R43a7b7f5a2c24540"/>
+</worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11173,7 +11173,7 @@
       <c r="X141" s="14"/>
       <c r="Y141" s="14"/>
       <c r="Z141" s="14" t="str">
-        <v>No iniciar hasta que exista y se apruebe la capacidad de contexto/sesión real de reserva vinculada.</v>
+        <v>No iniciar hasta que exista y se apruebe la capacidad de contexto/sesión real de reserva vinculada. IMP-AND-0501–0503 forman parte del prerequisito de foundation/contexto; fuente visual, confirmación e invalidación formal siguen pendientes.</v>
       </c>
     </row>
     <row r="142" ht="84" customHeight="1">
@@ -11985,6 +11985,326 @@
       <c r="X152"/>
       <c r="Y152"/>
       <c r="Z152"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>IMP-AND-0501</v>
+      </c>
+      <c r="B153" t="str">
+        <v>S5 Android Guest Auth</v>
+      </c>
+      <c r="C153" t="str">
+        <v>ANDROID</v>
+      </c>
+      <c r="D153" t="str">
+        <v>Auth / Context</v>
+      </c>
+      <c r="E153" t="str">
+        <v>ANDROID-1</v>
+      </c>
+      <c r="F153" t="str">
+        <v>WEB-2</v>
+      </c>
+      <c r="G153" t="str">
+        <v>guest-auth</v>
+      </c>
+      <c r="H153" t="str">
+        <v>FEATURE</v>
+      </c>
+      <c r="I153" t="str">
+        <v>CRÍTICA</v>
+      </c>
+      <c r="J153" t="str">
+        <v>EN_QA</v>
+      </c>
+      <c r="K153" t="str">
+        <v>IMP-AND-0108, IMP-AND-0109, IMP-AND-0201</v>
+      </c>
+      <c r="L153" t="str">
+        <v>Android Guest Auth frontend-first</v>
+      </c>
+      <c r="M153" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N153" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="O153" t="str">
+        <v>Guest Auth + Reservation Context foundation</v>
+      </c>
+      <c r="P153" t="str">
+        <v>Crear contracts domain, DTO/mapper de selección, interfaces, mocks sustituibles, providers session-only y resolver puro; sin UI ni rutas.</v>
+      </c>
+      <c r="Q153" t="str">
+        <v>GuestAuthSession, GuestAccount canónico, LinkedReservations y ActiveReservationContext quedan separados; 0 token/password persistido; 0 rutas nuevas.</v>
+      </c>
+      <c r="R153" t="str">
+        <v>Dependencias completadas; Change Control 32 y contrato 33 aprobados; autoridad frontend-first registrada.</v>
+      </c>
+      <c r="S153" t="str">
+        <v>Tests unitarios, typecheck, lint y diff-check PASS; no DTO en UI ni persistencia.</v>
+      </c>
+      <c r="T153" t="str">
+        <v>unit</v>
+      </c>
+      <c r="U153" t="str">
+        <v>src/modules/guest-auth/*; tests/guest-auth-foundation.test.tsx; docs 01/04/24/25/32/33</v>
+      </c>
+      <c r="V153" t="str">
+        <v>feature/android-guest-auth-foundation</v>
+      </c>
+      <c r="W153" t="str">
+        <v>EN_QA: tests foundation PASS; suite completa PASS; typecheck, lint, diff-check y Expo Doctor 21/21 PASS. Sin export: no requerido por DoD de 0501.</v>
+      </c>
+      <c r="X153" t="str">
+        <v>2026-09-25</v>
+      </c>
+      <c r="Y153" t="str">
+        <v/>
+      </c>
+      <c r="Z153" t="str">
+        <v>No Backend, HTTP real, tokens, AsyncStorage, SecureStore, Login UI, selector ni cambio de rutas.</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>IMP-AND-0502</v>
+      </c>
+      <c r="B154" t="str">
+        <v>S5 Android Guest Auth</v>
+      </c>
+      <c r="C154" t="str">
+        <v>ANDROID</v>
+      </c>
+      <c r="D154" t="str">
+        <v>Auth</v>
+      </c>
+      <c r="E154" t="str">
+        <v>ANDROID-1</v>
+      </c>
+      <c r="F154" t="str">
+        <v>WEB-2</v>
+      </c>
+      <c r="G154" t="str">
+        <v>guest-auth</v>
+      </c>
+      <c r="H154" t="str">
+        <v>FEATURE</v>
+      </c>
+      <c r="I154" t="str">
+        <v>CRÍTICA</v>
+      </c>
+      <c r="J154" t="str">
+        <v>PENDIENTE</v>
+      </c>
+      <c r="K154" t="str">
+        <v>IMP-AND-0501</v>
+      </c>
+      <c r="L154" t="str">
+        <v>Frontend-first approved — Guest Login</v>
+      </c>
+      <c r="M154" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N154" t="str">
+        <v>/login</v>
+      </c>
+      <c r="O154" t="str">
+        <v>Guest Login</v>
+      </c>
+      <c r="P154" t="str">
+        <v>Implementar email+password, validación local, mutation y estados Base/validación/submitting/rejected/error/offline; acción secundaria a Access.</v>
+      </c>
+      <c r="Q154" t="str">
+        <v>Login fuera de shell; copy genérico para credenciales; accesibilidad; no registro, recovery, social ni biometría.</v>
+      </c>
+      <c r="R154" t="str">
+        <v>IMP-AND-0501 COMPLETADA; contrato y autoridad visual frontend-first vigentes.</v>
+      </c>
+      <c r="S154" t="str">
+        <v>UI/tests/a11y PASS; sin persistir password ni tokens; rutas existentes no se rompen.</v>
+      </c>
+      <c r="T154" t="str">
+        <v>unit/ui</v>
+      </c>
+      <c r="U154" t="str">
+        <v>src/modules/guest-auth/*; app/login.tsx; tests/guest-login.test.tsx</v>
+      </c>
+      <c r="V154" t="str">
+        <v>feature/android-guest-login</v>
+      </c>
+      <c r="W154" t="str">
+        <v>PENDIENTE: no iniciar antes de 0501 COMPLETADA.</v>
+      </c>
+      <c r="X154" t="str">
+        <v/>
+      </c>
+      <c r="Y154" t="str">
+        <v/>
+      </c>
+      <c r="Z154" t="str">
+        <v>No Backend/auth real ni selección implícita de reserva.</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>IMP-AND-0503</v>
+      </c>
+      <c r="B155" t="str">
+        <v>S5 Android Guest Auth</v>
+      </c>
+      <c r="C155" t="str">
+        <v>ANDROID</v>
+      </c>
+      <c r="D155" t="str">
+        <v>Reservations / Context</v>
+      </c>
+      <c r="E155" t="str">
+        <v>ANDROID-1</v>
+      </c>
+      <c r="F155" t="str">
+        <v>WEB-2</v>
+      </c>
+      <c r="G155" t="str">
+        <v>guest-auth, stay</v>
+      </c>
+      <c r="H155" t="str">
+        <v>FEATURE</v>
+      </c>
+      <c r="I155" t="str">
+        <v>CRÍTICA</v>
+      </c>
+      <c r="J155" t="str">
+        <v>PENDIENTE</v>
+      </c>
+      <c r="K155" t="str">
+        <v>IMP-AND-0501, IMP-AND-0502</v>
+      </c>
+      <c r="L155" t="str">
+        <v>Frontend-first approved — Linked Reservations + Active Context</v>
+      </c>
+      <c r="M155" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N155" t="str">
+        <v>/reservations</v>
+      </c>
+      <c r="O155" t="str">
+        <v>Linked Reservations + Active Context</v>
+      </c>
+      <c r="P155" t="str">
+        <v>Implementar listado/selector, resolución 0/1/múltiples, guards y migración context-aware de Stay; invalidar solo datos reservation-scoped aprobados.</v>
+      </c>
+      <c r="Q155" t="str">
+        <v>Sin selección implícita; Empty CTA a Access; una reserva auto-contextualiza; múltiples requieren selección; Account/Profile/Rewards no se invalidan; Promotions/Chat sin cambios.</v>
+      </c>
+      <c r="R155" t="str">
+        <v>0501 y 0502 COMPLETADAS; estrategia de cache/guards y tests aprobados.</v>
+      </c>
+      <c r="S155" t="str">
+        <v>UI/tests/navigation/cache isolation PASS; sin tocar Access como Login ni reasignar Promotions/Chat.</v>
+      </c>
+      <c r="T155" t="str">
+        <v>unit/ui/navigation</v>
+      </c>
+      <c r="U155" t="str">
+        <v>src/modules/guest-auth/*; app/reservations.tsx; stay hooks; tests/guest-reservation-context.test.tsx</v>
+      </c>
+      <c r="V155" t="str">
+        <v>feature/android-linked-reservations-context</v>
+      </c>
+      <c r="W155" t="str">
+        <v>PENDIENTE: prerequisito parcial de IMP-AND-0116.</v>
+      </c>
+      <c r="X155" t="str">
+        <v/>
+      </c>
+      <c r="Y155" t="str">
+        <v/>
+      </c>
+      <c r="Z155" t="str">
+        <v>No Backend, HTTP real, persistencia ni contexto de ReservationStay copiado.</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>IMP-AND-0504</v>
+      </c>
+      <c r="B156" t="str">
+        <v>S5 Android Guest Auth</v>
+      </c>
+      <c r="C156" t="str">
+        <v>ANDROID</v>
+      </c>
+      <c r="D156" t="str">
+        <v>QA</v>
+      </c>
+      <c r="E156" t="str">
+        <v>ANDROID-1</v>
+      </c>
+      <c r="F156" t="str">
+        <v>WEB-2</v>
+      </c>
+      <c r="G156" t="str">
+        <v>guest-auth</v>
+      </c>
+      <c r="H156" t="str">
+        <v>QA</v>
+      </c>
+      <c r="I156" t="str">
+        <v>CRÍTICA</v>
+      </c>
+      <c r="J156" t="str">
+        <v>PENDIENTE</v>
+      </c>
+      <c r="K156" t="str">
+        <v>IMP-AND-0502, IMP-AND-0503</v>
+      </c>
+      <c r="L156" t="str">
+        <v>Android Guest Auth / Active Reservation journey</v>
+      </c>
+      <c r="M156" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N156" t="str">
+        <v>/login → /reservations → /account</v>
+      </c>
+      <c r="O156" t="str">
+        <v>QA Guest Auth / Active Reservation journey</v>
+      </c>
+      <c r="P156" t="str">
+        <v>Validar Login, 0/1/múltiples reservas, Access separado, guards, cold start e aislamiento de datos por contexto.</v>
+      </c>
+      <c r="Q156" t="str">
+        <v>Journey completo PASS; Guest/Staff separados; sin password logs/persistencia; no selección implícita.</v>
+      </c>
+      <c r="R156" t="str">
+        <v>0502 y 0503 COMPLETADAS.</v>
+      </c>
+      <c r="S156" t="str">
+        <v>Global DoD Android, regresión y QA manual PASS.</v>
+      </c>
+      <c r="T156" t="str">
+        <v>build/tests/manual</v>
+      </c>
+      <c r="U156" t="str">
+        <v>Android S5; tests guest auth/context</v>
+      </c>
+      <c r="V156" t="str">
+        <v>test/android-guest-auth-context</v>
+      </c>
+      <c r="W156" t="str">
+        <v>PENDIENTE: no iniciar antes de 0502 y 0503 COMPLETADAS.</v>
+      </c>
+      <c r="X156" t="str">
+        <v/>
+      </c>
+      <c r="Y156" t="str">
+        <v/>
+      </c>
+      <c r="Z156" t="str">
+        <v>Después de 0504 continúa IMP-AND-0116 y Android Release.</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="J2:J142">

</xml_diff>

<commit_message>
feat(android): implement guest login and session logout
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -820,7 +820,7 @@
       </c>
       <c r="F6" s="41" t="n">
         <f>COUNTIF('01_Backlog'!J2:J156,"COMPLETADA")</f>
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9">
@@ -888,7 +888,7 @@
       </c>
       <c r="G11" t="n">
         <f>COUNTIFS('01_Backlog'!C2:C156,E11,'01_Backlog'!J2:J156,"COMPLETADA")</f>
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
@@ -12015,7 +12015,7 @@
         <v>CRÍTICA</v>
       </c>
       <c r="J153" t="str">
-        <v>EN_QA</v>
+        <v>COMPLETADA</v>
       </c>
       <c r="K153" t="str">
         <v>IMP-AND-0108, IMP-AND-0109, IMP-AND-0201</v>
@@ -12054,13 +12054,13 @@
         <v>feature/android-guest-auth-foundation</v>
       </c>
       <c r="W153" t="str">
-        <v>EN_QA: tests foundation PASS; suite completa PASS; typecheck, lint, diff-check y Expo Doctor 21/21 PASS. Sin export: no requerido por DoD de 0501.</v>
+        <v>COMPLETADA: foundation mergeada; contracts, mocks, providers session-only y tests aprobados como autoridad para 0502.</v>
       </c>
       <c r="X153" t="str">
         <v>2026-09-25</v>
       </c>
       <c r="Y153" t="str">
-        <v/>
+        <v>2026-09-25</v>
       </c>
       <c r="Z153" t="str">
         <v>No Backend, HTTP real, tokens, AsyncStorage, SecureStore, Login UI, selector ni cambio de rutas.</v>
@@ -12095,7 +12095,7 @@
         <v>CRÍTICA</v>
       </c>
       <c r="J154" t="str">
-        <v>PENDIENTE</v>
+        <v>EN_QA</v>
       </c>
       <c r="K154" t="str">
         <v>IMP-AND-0501</v>
@@ -12134,10 +12134,10 @@
         <v>feature/android-guest-login</v>
       </c>
       <c r="W154" t="str">
-        <v>PENDIENTE: no iniciar antes de 0501 COMPLETADA.</v>
+        <v>EN_QA: guest-login/access/foundation focal PASS; suite completa PASS; typecheck, lint, diff-check, Expo Doctor 21/21 y Android export PASS. QA manual pendiente.</v>
       </c>
       <c r="X154" t="str">
-        <v/>
+        <v>2026-09-25</v>
       </c>
       <c r="Y154" t="str">
         <v/>

</xml_diff>

<commit_message>
test(android): close loyalty profile QA
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -11725,7 +11725,7 @@
         <v>CRÍTICA</v>
       </c>
       <c r="J149" t="str">
-        <v>PENDIENTE</v>
+        <v>EN_QA</v>
       </c>
       <c r="K149" t="str">
         <v>IMP-AND-0301, IMP-AND-0302, IMP-AND-0202</v>
@@ -11764,7 +11764,7 @@
         <v>test/android-loyalty</v>
       </c>
       <c r="W149" s="14" t="str">
-        <v>Change Control 31: dependencia de Profile sustituida por IMP-AND-0202, implementación canónica. Permanece PENDIENTE hasta completar 0202.</v>
+        <v>Change Control 31: dependencia de Profile sustituida por IMP-AND-0202, implementación canónica. QA-AND-0304-01 y QA-AND-0304-02 corregidos y regresiones automáticas PASS; EN_QA pendiente de revalidación manual física.</v>
       </c>
       <c r="X149"/>
       <c r="Y149"/>

</xml_diff>

<commit_message>
feat(android): add universal UI states
</commit_message>
<xml_diff>
--- a/docs/Backlog_Implementacion_PMS_V1.xlsx
+++ b/docs/Backlog_Implementacion_PMS_V1.xlsx
@@ -11799,7 +11799,7 @@
         <v>CRÍTICA</v>
       </c>
       <c r="J150" t="str">
-        <v>PENDIENTE</v>
+        <v>EN_QA</v>
       </c>
       <c r="K150" t="str">
         <v>IMP-AND-0009</v>
@@ -11837,7 +11837,9 @@
       <c r="V150" t="str">
         <v>feature/android-universal-states</v>
       </c>
-      <c r="W150"/>
+      <c r="W150" s="14" t="str">
+        <v>UniversalState shared implementado; QA automática PASS (tests, typecheck, lint, diff-check, Doctor y export). Pendiente revisión manual y WEB-2.</v>
+      </c>
       <c r="X150"/>
       <c r="Y150"/>
       <c r="Z150"/>

</xml_diff>